<commit_message>
feat(catalog): integrate OpenAPI 3.0, Swagger UI, Postman collection and B-tree indexes migration
</commit_message>
<xml_diff>
--- a/plan/backlog-freshflow-mvp-12-tuan-updated.xlsx
+++ b/plan/backlog-freshflow-mvp-12-tuan-updated.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30412"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30501"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\FreshFlow\plan\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F99A07B0-0871-4FC3-93C8-3FD03B1269E9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D5307DE1-9AE7-45D6-A8CA-2DD3B5147EA9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="600" yWindow="-120" windowWidth="28320" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Backlog 12 Tuan" sheetId="1" r:id="rId1"/>
@@ -19,6 +19,7 @@
     <sheet name="Dashboard" sheetId="4" r:id="rId4"/>
     <sheet name="Database Track" sheetId="5" r:id="rId5"/>
     <sheet name="Database Guide" sheetId="6" r:id="rId6"/>
+    <sheet name="Note" sheetId="7" r:id="rId7"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Backlog 12 Tuan'!$A$2:$U$170</definedName>
@@ -46,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2814" uniqueCount="1618">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2815" uniqueCount="1619">
   <si>
     <t>Task ID</t>
   </si>
@@ -4900,6 +4901,9 @@
   </si>
   <si>
     <t>In Progress</t>
+  </si>
+  <si>
+    <t>13/9/2026</t>
   </si>
 </sst>
 </file>
@@ -4925,7 +4929,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="14">
+  <fills count="22">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -5000,6 +5004,54 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF92D050"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF00B0F0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="3" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="2" tint="-0.249977111117893"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="3">
     <border>
@@ -5029,7 +5081,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -5074,6 +5126,30 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="13" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="16" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="17" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="18" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="19" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="20" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="21" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -5156,6 +5232,143 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>460538</xdr:colOff>
+      <xdr:row>32</xdr:row>
+      <xdr:rowOff>95249</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{C36B6887-1390-E139-3D76-3095CA616469}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="7775738" cy="6191249"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>32</xdr:row>
+      <xdr:rowOff>95250</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>14</xdr:col>
+      <xdr:colOff>287209</xdr:colOff>
+      <xdr:row>65</xdr:row>
+      <xdr:rowOff>9524</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Picture 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{7A3C827B-52A1-D0D0-64CA-5DB2EA71865C}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="6191250"/>
+          <a:ext cx="8821609" cy="6200774"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>428625</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>25</xdr:col>
+      <xdr:colOff>134415</xdr:colOff>
+      <xdr:row>32</xdr:row>
+      <xdr:rowOff>96114</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="4" name="Picture 3">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F423D454-3A76-41DA-1365-CBD4D896E695}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="7743825" y="0"/>
+          <a:ext cx="7630590" cy="6192114"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -5628,7 +5841,7 @@
       <c r="P3" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="Q3" s="3"/>
+      <c r="Q3" s="21"/>
       <c r="R3" s="3" t="s">
         <v>34</v>
       </c>
@@ -5683,7 +5896,7 @@
       <c r="P4" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="Q4" s="3"/>
+      <c r="Q4" s="21"/>
       <c r="R4" s="3"/>
       <c r="S4" s="3"/>
       <c r="T4" s="3"/>
@@ -5736,7 +5949,7 @@
       <c r="P5" s="6" t="s">
         <v>33</v>
       </c>
-      <c r="Q5" s="3"/>
+      <c r="Q5" s="21"/>
       <c r="R5" s="3"/>
       <c r="S5" s="3"/>
       <c r="T5" s="3"/>
@@ -5789,7 +6002,7 @@
       <c r="P6" s="6" t="s">
         <v>33</v>
       </c>
-      <c r="Q6" s="3"/>
+      <c r="Q6" s="21"/>
       <c r="R6" s="3"/>
       <c r="S6" s="3"/>
       <c r="T6" s="3"/>
@@ -5842,7 +6055,7 @@
       <c r="P7" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="Q7" s="3"/>
+      <c r="Q7" s="21"/>
       <c r="R7" s="3"/>
       <c r="S7" s="3"/>
       <c r="T7" s="3"/>
@@ -5895,7 +6108,7 @@
       <c r="P8" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="Q8" s="3"/>
+      <c r="Q8" s="21"/>
       <c r="R8" s="3"/>
       <c r="S8" s="3" t="s">
         <v>80</v>
@@ -5954,7 +6167,7 @@
       <c r="P9" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="Q9" s="3"/>
+      <c r="Q9" s="21"/>
       <c r="R9" s="3"/>
       <c r="S9" s="3"/>
       <c r="T9" s="3"/>
@@ -6005,9 +6218,9 @@
       </c>
       <c r="O10" s="3"/>
       <c r="P10" s="3" t="s">
-        <v>1617</v>
-      </c>
-      <c r="Q10" s="3"/>
+        <v>33</v>
+      </c>
+      <c r="Q10" s="21"/>
       <c r="R10" s="3"/>
       <c r="S10" s="3"/>
       <c r="T10" s="3"/>
@@ -6058,9 +6271,9 @@
       </c>
       <c r="O11" s="3"/>
       <c r="P11" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="Q11" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="Q11" s="21" t="s">
         <v>1616</v>
       </c>
       <c r="R11" s="3"/>
@@ -6119,9 +6332,9 @@
       </c>
       <c r="O12" s="3"/>
       <c r="P12" s="3" t="s">
-        <v>71</v>
-      </c>
-      <c r="Q12" s="3"/>
+        <v>33</v>
+      </c>
+      <c r="Q12" s="21"/>
       <c r="R12" s="3"/>
       <c r="S12" s="3"/>
       <c r="T12" s="3"/>
@@ -6172,9 +6385,9 @@
       </c>
       <c r="O13" s="3"/>
       <c r="P13" s="3" t="s">
-        <v>71</v>
-      </c>
-      <c r="Q13" s="3"/>
+        <v>33</v>
+      </c>
+      <c r="Q13" s="21"/>
       <c r="R13" s="3"/>
       <c r="S13" s="3"/>
       <c r="T13" s="3"/>
@@ -6225,9 +6438,9 @@
       </c>
       <c r="O14" s="3"/>
       <c r="P14" s="3" t="s">
-        <v>71</v>
-      </c>
-      <c r="Q14" s="3"/>
+        <v>33</v>
+      </c>
+      <c r="Q14" s="21"/>
       <c r="R14" s="3"/>
       <c r="S14" s="3"/>
       <c r="T14" s="3"/>
@@ -6280,7 +6493,7 @@
       <c r="P15" s="3" t="s">
         <v>71</v>
       </c>
-      <c r="Q15" s="3"/>
+      <c r="Q15" s="21"/>
       <c r="R15" s="3"/>
       <c r="S15" s="3"/>
       <c r="T15" s="3"/>
@@ -6333,14 +6546,14 @@
       <c r="P16" s="3" t="s">
         <v>71</v>
       </c>
-      <c r="Q16" s="3"/>
+      <c r="Q16" s="21"/>
       <c r="R16" s="3"/>
       <c r="S16" s="3"/>
       <c r="T16" s="3"/>
       <c r="U16" s="3"/>
     </row>
     <row r="17" spans="1:21" ht="78" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="3" t="s">
+      <c r="A17" s="25" t="s">
         <v>149</v>
       </c>
       <c r="B17" s="3">
@@ -6349,7 +6562,7 @@
       <c r="C17" s="3" t="s">
         <v>150</v>
       </c>
-      <c r="D17" s="3" t="s">
+      <c r="D17" s="24" t="s">
         <v>23</v>
       </c>
       <c r="E17" s="3" t="s">
@@ -6386,7 +6599,7 @@
         <v>157</v>
       </c>
       <c r="P17" s="3" t="s">
-        <v>71</v>
+        <v>33</v>
       </c>
       <c r="Q17" s="3"/>
       <c r="R17" s="3"/>
@@ -6401,7 +6614,7 @@
       </c>
     </row>
     <row r="18" spans="1:21" ht="78" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="3" t="s">
+      <c r="A18" s="25" t="s">
         <v>161</v>
       </c>
       <c r="B18" s="3">
@@ -6410,7 +6623,7 @@
       <c r="C18" s="3" t="s">
         <v>150</v>
       </c>
-      <c r="D18" s="3" t="s">
+      <c r="D18" s="24" t="s">
         <v>23</v>
       </c>
       <c r="E18" s="3" t="s">
@@ -6447,7 +6660,7 @@
         <v>169</v>
       </c>
       <c r="P18" s="3" t="s">
-        <v>71</v>
+        <v>33</v>
       </c>
       <c r="Q18" s="3"/>
       <c r="R18" s="3"/>
@@ -6462,7 +6675,7 @@
       </c>
     </row>
     <row r="19" spans="1:21" ht="78" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="3" t="s">
+      <c r="A19" s="25" t="s">
         <v>172</v>
       </c>
       <c r="B19" s="3">
@@ -6471,7 +6684,7 @@
       <c r="C19" s="3" t="s">
         <v>150</v>
       </c>
-      <c r="D19" s="3" t="s">
+      <c r="D19" s="16" t="s">
         <v>45</v>
       </c>
       <c r="E19" s="3" t="s">
@@ -6508,7 +6721,7 @@
         <v>179</v>
       </c>
       <c r="P19" s="3" t="s">
-        <v>71</v>
+        <v>33</v>
       </c>
       <c r="Q19" s="3"/>
       <c r="R19" s="3"/>
@@ -6517,7 +6730,7 @@
       <c r="U19" s="3"/>
     </row>
     <row r="20" spans="1:21" ht="78" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="3" t="s">
+      <c r="A20" s="25" t="s">
         <v>180</v>
       </c>
       <c r="B20" s="3">
@@ -6526,7 +6739,7 @@
       <c r="C20" s="3" t="s">
         <v>150</v>
       </c>
-      <c r="D20" s="3" t="s">
+      <c r="D20" s="16" t="s">
         <v>45</v>
       </c>
       <c r="E20" s="3" t="s">
@@ -6563,7 +6776,7 @@
         <v>179</v>
       </c>
       <c r="P20" s="3" t="s">
-        <v>71</v>
+        <v>33</v>
       </c>
       <c r="Q20" s="3"/>
       <c r="R20" s="3"/>
@@ -6572,7 +6785,7 @@
       <c r="U20" s="3"/>
     </row>
     <row r="21" spans="1:21" ht="78" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="3" t="s">
+      <c r="A21" s="25" t="s">
         <v>187</v>
       </c>
       <c r="B21" s="3">
@@ -6581,7 +6794,7 @@
       <c r="C21" s="3" t="s">
         <v>150</v>
       </c>
-      <c r="D21" s="3" t="s">
+      <c r="D21" s="23" t="s">
         <v>63</v>
       </c>
       <c r="E21" s="3" t="s">
@@ -6618,7 +6831,7 @@
         <v>195</v>
       </c>
       <c r="P21" s="3" t="s">
-        <v>71</v>
+        <v>33</v>
       </c>
       <c r="Q21" s="3"/>
       <c r="R21" s="3"/>
@@ -6627,7 +6840,7 @@
       <c r="U21" s="3"/>
     </row>
     <row r="22" spans="1:21" ht="78" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="3" t="s">
+      <c r="A22" s="25" t="s">
         <v>196</v>
       </c>
       <c r="B22" s="3">
@@ -6636,7 +6849,7 @@
       <c r="C22" s="3" t="s">
         <v>150</v>
       </c>
-      <c r="D22" s="3" t="s">
+      <c r="D22" s="23" t="s">
         <v>63</v>
       </c>
       <c r="E22" s="3" t="s">
@@ -6673,7 +6886,7 @@
         <v>203</v>
       </c>
       <c r="P22" s="3" t="s">
-        <v>71</v>
+        <v>33</v>
       </c>
       <c r="Q22" s="3"/>
       <c r="R22" s="3"/>
@@ -6682,7 +6895,7 @@
       <c r="U22" s="3"/>
     </row>
     <row r="23" spans="1:21" ht="78" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="3" t="s">
+      <c r="A23" s="25" t="s">
         <v>204</v>
       </c>
       <c r="B23" s="3">
@@ -6691,7 +6904,7 @@
       <c r="C23" s="3" t="s">
         <v>150</v>
       </c>
-      <c r="D23" s="3" t="s">
+      <c r="D23" s="22" t="s">
         <v>84</v>
       </c>
       <c r="E23" s="3" t="s">
@@ -6728,7 +6941,7 @@
         <v>211</v>
       </c>
       <c r="P23" s="3" t="s">
-        <v>71</v>
+        <v>33</v>
       </c>
       <c r="Q23" s="3"/>
       <c r="R23" s="3"/>
@@ -6743,7 +6956,7 @@
       </c>
     </row>
     <row r="24" spans="1:21" ht="78" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="3" t="s">
+      <c r="A24" s="25" t="s">
         <v>215</v>
       </c>
       <c r="B24" s="3">
@@ -6752,7 +6965,7 @@
       <c r="C24" s="3" t="s">
         <v>150</v>
       </c>
-      <c r="D24" s="3" t="s">
+      <c r="D24" s="22" t="s">
         <v>84</v>
       </c>
       <c r="E24" s="3" t="s">
@@ -6789,7 +7002,7 @@
         <v>211</v>
       </c>
       <c r="P24" s="3" t="s">
-        <v>71</v>
+        <v>1617</v>
       </c>
       <c r="Q24" s="3"/>
       <c r="R24" s="3"/>
@@ -6804,7 +7017,7 @@
       </c>
     </row>
     <row r="25" spans="1:21" ht="78" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="3" t="s">
+      <c r="A25" s="25" t="s">
         <v>226</v>
       </c>
       <c r="B25" s="3">
@@ -6813,7 +7026,7 @@
       <c r="C25" s="3" t="s">
         <v>150</v>
       </c>
-      <c r="D25" s="3" t="s">
+      <c r="D25" s="21" t="s">
         <v>100</v>
       </c>
       <c r="E25" s="3" t="s">
@@ -6850,7 +7063,7 @@
         <v>211</v>
       </c>
       <c r="P25" s="3" t="s">
-        <v>71</v>
+        <v>1617</v>
       </c>
       <c r="Q25" s="3"/>
       <c r="R25" s="3"/>
@@ -6859,7 +7072,7 @@
       <c r="U25" s="3"/>
     </row>
     <row r="26" spans="1:21" ht="78" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="3" t="s">
+      <c r="A26" s="25" t="s">
         <v>233</v>
       </c>
       <c r="B26" s="3">
@@ -6868,7 +7081,7 @@
       <c r="C26" s="3" t="s">
         <v>150</v>
       </c>
-      <c r="D26" s="3" t="s">
+      <c r="D26" s="21" t="s">
         <v>100</v>
       </c>
       <c r="E26" s="3" t="s">
@@ -6905,7 +7118,7 @@
         <v>241</v>
       </c>
       <c r="P26" s="3" t="s">
-        <v>71</v>
+        <v>1617</v>
       </c>
       <c r="Q26" s="3"/>
       <c r="R26" s="3"/>
@@ -6914,7 +7127,7 @@
       <c r="U26" s="3"/>
     </row>
     <row r="27" spans="1:21" ht="78" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="3" t="s">
+      <c r="A27" s="25" t="s">
         <v>242</v>
       </c>
       <c r="B27" s="3">
@@ -6923,7 +7136,7 @@
       <c r="C27" s="3" t="s">
         <v>150</v>
       </c>
-      <c r="D27" s="3" t="s">
+      <c r="D27" s="19" t="s">
         <v>119</v>
       </c>
       <c r="E27" s="3" t="s">
@@ -6960,7 +7173,7 @@
         <v>250</v>
       </c>
       <c r="P27" s="3" t="s">
-        <v>71</v>
+        <v>1617</v>
       </c>
       <c r="Q27" s="3"/>
       <c r="R27" s="3"/>
@@ -6969,7 +7182,7 @@
       <c r="U27" s="3"/>
     </row>
     <row r="28" spans="1:21" ht="78" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="3" t="s">
+      <c r="A28" s="25" t="s">
         <v>251</v>
       </c>
       <c r="B28" s="3">
@@ -6978,7 +7191,7 @@
       <c r="C28" s="3" t="s">
         <v>150</v>
       </c>
-      <c r="D28" s="3" t="s">
+      <c r="D28" s="19" t="s">
         <v>119</v>
       </c>
       <c r="E28" s="3" t="s">
@@ -7015,7 +7228,7 @@
         <v>250</v>
       </c>
       <c r="P28" s="3" t="s">
-        <v>71</v>
+        <v>1617</v>
       </c>
       <c r="Q28" s="3"/>
       <c r="R28" s="3"/>
@@ -7024,7 +7237,7 @@
       <c r="U28" s="3"/>
     </row>
     <row r="29" spans="1:21" ht="78" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="3" t="s">
+      <c r="A29" s="25" t="s">
         <v>259</v>
       </c>
       <c r="B29" s="3">
@@ -7033,7 +7246,7 @@
       <c r="C29" s="3" t="s">
         <v>150</v>
       </c>
-      <c r="D29" s="3" t="s">
+      <c r="D29" s="20" t="s">
         <v>135</v>
       </c>
       <c r="E29" s="3" t="s">
@@ -7070,7 +7283,7 @@
         <v>266</v>
       </c>
       <c r="P29" s="3" t="s">
-        <v>71</v>
+        <v>1617</v>
       </c>
       <c r="Q29" s="3"/>
       <c r="R29" s="3"/>
@@ -7079,7 +7292,7 @@
       <c r="U29" s="3"/>
     </row>
     <row r="30" spans="1:21" ht="78" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="3" t="s">
+      <c r="A30" s="25" t="s">
         <v>267</v>
       </c>
       <c r="B30" s="3">
@@ -7088,7 +7301,7 @@
       <c r="C30" s="3" t="s">
         <v>150</v>
       </c>
-      <c r="D30" s="3" t="s">
+      <c r="D30" s="20" t="s">
         <v>135</v>
       </c>
       <c r="E30" s="3" t="s">
@@ -7125,10 +7338,12 @@
         <v>266</v>
       </c>
       <c r="P30" s="3" t="s">
-        <v>71</v>
+        <v>1617</v>
       </c>
       <c r="Q30" s="3"/>
-      <c r="R30" s="3"/>
+      <c r="R30" s="3" t="s">
+        <v>1618</v>
+      </c>
       <c r="S30" s="3"/>
       <c r="T30" s="3"/>
       <c r="U30" s="3"/>
@@ -8701,7 +8916,7 @@
       <c r="E59" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="F59" s="3" t="s">
+      <c r="F59" s="18" t="s">
         <v>495</v>
       </c>
       <c r="G59" s="3" t="s">
@@ -8762,7 +8977,7 @@
       <c r="E60" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="F60" s="3" t="s">
+      <c r="F60" s="18" t="s">
         <v>495</v>
       </c>
       <c r="G60" s="3" t="s">
@@ -8817,7 +9032,7 @@
       <c r="E61" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="F61" s="3" t="s">
+      <c r="F61" s="18" t="s">
         <v>495</v>
       </c>
       <c r="G61" s="3" t="s">
@@ -8872,7 +9087,7 @@
       <c r="E62" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="F62" s="3" t="s">
+      <c r="F62" s="18" t="s">
         <v>495</v>
       </c>
       <c r="G62" s="3" t="s">
@@ -8927,7 +9142,7 @@
       <c r="E63" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="F63" s="3" t="s">
+      <c r="F63" s="18" t="s">
         <v>495</v>
       </c>
       <c r="G63" s="3" t="s">
@@ -8982,7 +9197,7 @@
       <c r="E64" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="F64" s="3" t="s">
+      <c r="F64" s="18" t="s">
         <v>495</v>
       </c>
       <c r="G64" s="3" t="s">
@@ -9043,7 +9258,7 @@
       <c r="E65" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="F65" s="3" t="s">
+      <c r="F65" s="18" t="s">
         <v>495</v>
       </c>
       <c r="G65" s="3" t="s">
@@ -9098,7 +9313,7 @@
       <c r="E66" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="F66" s="3" t="s">
+      <c r="F66" s="18" t="s">
         <v>495</v>
       </c>
       <c r="G66" s="3" t="s">
@@ -9153,7 +9368,7 @@
       <c r="E67" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="F67" s="3" t="s">
+      <c r="F67" s="18" t="s">
         <v>495</v>
       </c>
       <c r="G67" s="3" t="s">
@@ -9485,7 +9700,7 @@
       <c r="E73" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="F73" s="3" t="s">
+      <c r="F73" s="18" t="s">
         <v>495</v>
       </c>
       <c r="G73" s="3" t="s">
@@ -9540,7 +9755,7 @@
       <c r="E74" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="F74" s="3" t="s">
+      <c r="F74" s="18" t="s">
         <v>495</v>
       </c>
       <c r="G74" s="3" t="s">
@@ -9595,7 +9810,7 @@
       <c r="E75" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="F75" s="3" t="s">
+      <c r="F75" s="18" t="s">
         <v>495</v>
       </c>
       <c r="G75" s="3" t="s">
@@ -9827,7 +10042,7 @@
       <c r="E79" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="F79" s="3" t="s">
+      <c r="F79" s="18" t="s">
         <v>495</v>
       </c>
       <c r="G79" s="3" t="s">
@@ -9882,7 +10097,7 @@
       <c r="E80" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="F80" s="3" t="s">
+      <c r="F80" s="18" t="s">
         <v>495</v>
       </c>
       <c r="G80" s="3" t="s">
@@ -9992,7 +10207,7 @@
       <c r="E82" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="F82" s="3" t="s">
+      <c r="F82" s="18" t="s">
         <v>495</v>
       </c>
       <c r="G82" s="3" t="s">
@@ -10499,7 +10714,7 @@
       <c r="E91" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="F91" s="3" t="s">
+      <c r="F91" s="19" t="s">
         <v>276</v>
       </c>
       <c r="G91" s="3" t="s">
@@ -10554,7 +10769,7 @@
       <c r="E92" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="F92" s="3" t="s">
+      <c r="F92" s="19" t="s">
         <v>276</v>
       </c>
       <c r="G92" s="3" t="s">
@@ -10609,7 +10824,7 @@
       <c r="E93" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="F93" s="3" t="s">
+      <c r="F93" s="18" t="s">
         <v>495</v>
       </c>
       <c r="G93" s="3" t="s">
@@ -10664,7 +10879,7 @@
       <c r="E94" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="F94" s="3" t="s">
+      <c r="F94" s="18" t="s">
         <v>495</v>
       </c>
       <c r="G94" s="3" t="s">
@@ -15332,7 +15547,7 @@
       </c>
       <c r="B11" s="7" t="str">
         <f>COUNTIF('Backlog 12 Tuan'!P:P,"Done")&amp;" / "&amp;COUNTA('Backlog 12 Tuan'!A:A)-1&amp;" task Done"</f>
-        <v>7 / 168 task Done</v>
+        <v>19 / 168 task Done</v>
       </c>
     </row>
     <row r="12" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -15341,7 +15556,7 @@
       </c>
       <c r="B12" s="8">
         <f>COUNTIF('Backlog 12 Tuan'!P:P,"Done")/(COUNTA('Backlog 12 Tuan'!A:A)-1)</f>
-        <v>4.1666666666666664E-2</v>
+        <v>0.1130952380952381</v>
       </c>
     </row>
     <row r="13" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -16619,4 +16834,14 @@
     <oddFooter>&amp;L&amp;C&amp;R</oddFooter>
   </headerFooter>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F5F6CA76-DC76-4953-93F0-709FEA2EE783}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
test(catalog): add unit tests for access service, variant service, and controller
</commit_message>
<xml_diff>
--- a/plan/backlog-freshflow-mvp-12-tuan-updated.xlsx
+++ b/plan/backlog-freshflow-mvp-12-tuan-updated.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\FreshFlow\plan\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D5307DE1-9AE7-45D6-A8CA-2DD3B5147EA9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{24143C62-ECD9-493F-AB50-F20AA407B670}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="600" yWindow="-120" windowWidth="28320" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="14655" yWindow="0" windowWidth="14250" windowHeight="16305" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Backlog 12 Tuan" sheetId="1" r:id="rId1"/>
@@ -7002,7 +7002,7 @@
         <v>211</v>
       </c>
       <c r="P24" s="3" t="s">
-        <v>1617</v>
+        <v>33</v>
       </c>
       <c r="Q24" s="3"/>
       <c r="R24" s="3"/>
@@ -15547,7 +15547,7 @@
       </c>
       <c r="B11" s="7" t="str">
         <f>COUNTIF('Backlog 12 Tuan'!P:P,"Done")&amp;" / "&amp;COUNTA('Backlog 12 Tuan'!A:A)-1&amp;" task Done"</f>
-        <v>19 / 168 task Done</v>
+        <v>20 / 168 task Done</v>
       </c>
     </row>
     <row r="12" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -15556,7 +15556,7 @@
       </c>
       <c r="B12" s="8">
         <f>COUNTIF('Backlog 12 Tuan'!P:P,"Done")/(COUNTA('Backlog 12 Tuan'!A:A)-1)</f>
-        <v>0.1130952380952381</v>
+        <v>0.11904761904761904</v>
       </c>
     </row>
     <row r="13" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
complete design for web front developer
</commit_message>
<xml_diff>
--- a/plan/backlog-freshflow-mvp-12-tuan-updated.xlsx
+++ b/plan/backlog-freshflow-mvp-12-tuan-updated.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30501"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30508"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\FreshFlow\plan\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{007AE543-DEB2-4F30-BE7F-72FD693F22A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F587CE1E-BCC0-4459-B5C1-E80613089EBF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="600" yWindow="-120" windowWidth="28320" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -4929,7 +4929,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="22">
+  <fills count="27">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -5052,6 +5052,36 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="3" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF00B050"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="-0.249977111117893"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF0000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="3">
     <border>
@@ -5081,7 +5111,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -5150,6 +5180,21 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="21" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="22" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="23" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="24" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="25" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="26" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -7173,7 +7218,7 @@
         <v>250</v>
       </c>
       <c r="P27" s="3" t="s">
-        <v>1617</v>
+        <v>33</v>
       </c>
       <c r="Q27" s="3"/>
       <c r="R27" s="3"/>
@@ -7228,7 +7273,7 @@
         <v>250</v>
       </c>
       <c r="P28" s="3" t="s">
-        <v>1617</v>
+        <v>33</v>
       </c>
       <c r="Q28" s="3"/>
       <c r="R28" s="3"/>
@@ -7283,7 +7328,7 @@
         <v>266</v>
       </c>
       <c r="P29" s="3" t="s">
-        <v>1617</v>
+        <v>33</v>
       </c>
       <c r="Q29" s="3"/>
       <c r="R29" s="3"/>
@@ -7349,7 +7394,7 @@
       <c r="U30" s="3"/>
     </row>
     <row r="31" spans="1:21" ht="78" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="3" t="s">
+      <c r="A31" s="26" t="s">
         <v>274</v>
       </c>
       <c r="B31" s="3">
@@ -7358,7 +7403,7 @@
       <c r="C31" s="3" t="s">
         <v>275</v>
       </c>
-      <c r="D31" s="3" t="s">
+      <c r="D31" s="19" t="s">
         <v>23</v>
       </c>
       <c r="E31" s="3" t="s">
@@ -7404,7 +7449,7 @@
       <c r="U31" s="3"/>
     </row>
     <row r="32" spans="1:21" ht="78" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="3" t="s">
+      <c r="A32" s="26" t="s">
         <v>283</v>
       </c>
       <c r="B32" s="3">
@@ -7413,7 +7458,7 @@
       <c r="C32" s="3" t="s">
         <v>275</v>
       </c>
-      <c r="D32" s="3" t="s">
+      <c r="D32" s="19" t="s">
         <v>23</v>
       </c>
       <c r="E32" s="3" t="s">
@@ -7459,7 +7504,7 @@
       <c r="U32" s="3"/>
     </row>
     <row r="33" spans="1:21" ht="78" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="3" t="s">
+      <c r="A33" s="26" t="s">
         <v>291</v>
       </c>
       <c r="B33" s="3">
@@ -7468,7 +7513,7 @@
       <c r="C33" s="3" t="s">
         <v>275</v>
       </c>
-      <c r="D33" s="3" t="s">
+      <c r="D33" s="27" t="s">
         <v>45</v>
       </c>
       <c r="E33" s="3" t="s">
@@ -7514,7 +7559,7 @@
       <c r="U33" s="3"/>
     </row>
     <row r="34" spans="1:21" ht="78" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="3" t="s">
+      <c r="A34" s="26" t="s">
         <v>298</v>
       </c>
       <c r="B34" s="3">
@@ -7523,7 +7568,7 @@
       <c r="C34" s="3" t="s">
         <v>275</v>
       </c>
-      <c r="D34" s="3" t="s">
+      <c r="D34" s="27" t="s">
         <v>45</v>
       </c>
       <c r="E34" s="3" t="s">
@@ -7569,7 +7614,7 @@
       <c r="U34" s="3"/>
     </row>
     <row r="35" spans="1:21" ht="78" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="3" t="s">
+      <c r="A35" s="26" t="s">
         <v>305</v>
       </c>
       <c r="B35" s="3">
@@ -7578,7 +7623,7 @@
       <c r="C35" s="3" t="s">
         <v>275</v>
       </c>
-      <c r="D35" s="3" t="s">
+      <c r="D35" s="22" t="s">
         <v>63</v>
       </c>
       <c r="E35" s="3" t="s">
@@ -7624,7 +7669,7 @@
       <c r="U35" s="3"/>
     </row>
     <row r="36" spans="1:21" ht="78" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="3" t="s">
+      <c r="A36" s="26" t="s">
         <v>313</v>
       </c>
       <c r="B36" s="3">
@@ -7633,7 +7678,7 @@
       <c r="C36" s="3" t="s">
         <v>275</v>
       </c>
-      <c r="D36" s="3" t="s">
+      <c r="D36" s="22" t="s">
         <v>63</v>
       </c>
       <c r="E36" s="3" t="s">
@@ -7679,7 +7724,7 @@
       <c r="U36" s="3"/>
     </row>
     <row r="37" spans="1:21" ht="78" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="3" t="s">
+      <c r="A37" s="26" t="s">
         <v>321</v>
       </c>
       <c r="B37" s="3">
@@ -7688,7 +7733,7 @@
       <c r="C37" s="3" t="s">
         <v>275</v>
       </c>
-      <c r="D37" s="3" t="s">
+      <c r="D37" s="21" t="s">
         <v>84</v>
       </c>
       <c r="E37" s="3" t="s">
@@ -7734,7 +7779,7 @@
       <c r="U37" s="3"/>
     </row>
     <row r="38" spans="1:21" ht="78" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="3" t="s">
+      <c r="A38" s="26" t="s">
         <v>328</v>
       </c>
       <c r="B38" s="3">
@@ -7743,7 +7788,7 @@
       <c r="C38" s="3" t="s">
         <v>275</v>
       </c>
-      <c r="D38" s="3" t="s">
+      <c r="D38" s="21" t="s">
         <v>84</v>
       </c>
       <c r="E38" s="3" t="s">
@@ -7789,7 +7834,7 @@
       <c r="U38" s="3"/>
     </row>
     <row r="39" spans="1:21" ht="78" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="3" t="s">
+      <c r="A39" s="26" t="s">
         <v>336</v>
       </c>
       <c r="B39" s="3">
@@ -7798,7 +7843,7 @@
       <c r="C39" s="3" t="s">
         <v>275</v>
       </c>
-      <c r="D39" s="3" t="s">
+      <c r="D39" s="28" t="s">
         <v>100</v>
       </c>
       <c r="E39" s="3" t="s">
@@ -7844,7 +7889,7 @@
       <c r="U39" s="3"/>
     </row>
     <row r="40" spans="1:21" ht="78" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A40" s="3" t="s">
+      <c r="A40" s="26" t="s">
         <v>343</v>
       </c>
       <c r="B40" s="3">
@@ -7853,7 +7898,7 @@
       <c r="C40" s="3" t="s">
         <v>275</v>
       </c>
-      <c r="D40" s="3" t="s">
+      <c r="D40" s="28" t="s">
         <v>100</v>
       </c>
       <c r="E40" s="3" t="s">
@@ -7899,7 +7944,7 @@
       <c r="U40" s="3"/>
     </row>
     <row r="41" spans="1:21" ht="78" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="3" t="s">
+      <c r="A41" s="26" t="s">
         <v>350</v>
       </c>
       <c r="B41" s="3">
@@ -7908,7 +7953,7 @@
       <c r="C41" s="3" t="s">
         <v>275</v>
       </c>
-      <c r="D41" s="3" t="s">
+      <c r="D41" s="30" t="s">
         <v>119</v>
       </c>
       <c r="E41" s="3" t="s">
@@ -7954,7 +7999,7 @@
       <c r="U41" s="3"/>
     </row>
     <row r="42" spans="1:21" ht="78" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A42" s="3" t="s">
+      <c r="A42" s="26" t="s">
         <v>358</v>
       </c>
       <c r="B42" s="3">
@@ -7963,7 +8008,7 @@
       <c r="C42" s="3" t="s">
         <v>275</v>
       </c>
-      <c r="D42" s="3" t="s">
+      <c r="D42" s="30" t="s">
         <v>119</v>
       </c>
       <c r="E42" s="3" t="s">
@@ -8009,7 +8054,7 @@
       <c r="U42" s="3"/>
     </row>
     <row r="43" spans="1:21" ht="78" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A43" s="3" t="s">
+      <c r="A43" s="26" t="s">
         <v>366</v>
       </c>
       <c r="B43" s="3">
@@ -8018,7 +8063,7 @@
       <c r="C43" s="3" t="s">
         <v>275</v>
       </c>
-      <c r="D43" s="3" t="s">
+      <c r="D43" s="29" t="s">
         <v>135</v>
       </c>
       <c r="E43" s="3" t="s">
@@ -8064,7 +8109,7 @@
       <c r="U43" s="3"/>
     </row>
     <row r="44" spans="1:21" ht="78" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A44" s="3" t="s">
+      <c r="A44" s="26" t="s">
         <v>374</v>
       </c>
       <c r="B44" s="3">
@@ -8073,7 +8118,7 @@
       <c r="C44" s="3" t="s">
         <v>275</v>
       </c>
-      <c r="D44" s="3" t="s">
+      <c r="D44" s="29" t="s">
         <v>135</v>
       </c>
       <c r="E44" s="3" t="s">
@@ -8119,7 +8164,7 @@
       <c r="U44" s="3"/>
     </row>
     <row r="45" spans="1:21" ht="78" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A45" s="3" t="s">
+      <c r="A45" s="26" t="s">
         <v>381</v>
       </c>
       <c r="B45" s="3">
@@ -8174,7 +8219,7 @@
       <c r="U45" s="3"/>
     </row>
     <row r="46" spans="1:21" ht="78" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A46" s="3" t="s">
+      <c r="A46" s="26" t="s">
         <v>389</v>
       </c>
       <c r="B46" s="3">
@@ -8235,7 +8280,7 @@
       </c>
     </row>
     <row r="47" spans="1:21" ht="78" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A47" s="3" t="s">
+      <c r="A47" s="26" t="s">
         <v>399</v>
       </c>
       <c r="B47" s="3">
@@ -8290,7 +8335,7 @@
       <c r="U47" s="3"/>
     </row>
     <row r="48" spans="1:21" ht="78" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A48" s="3" t="s">
+      <c r="A48" s="26" t="s">
         <v>407</v>
       </c>
       <c r="B48" s="3">
@@ -8345,7 +8390,7 @@
       <c r="U48" s="3"/>
     </row>
     <row r="49" spans="1:21" ht="78" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A49" s="3" t="s">
+      <c r="A49" s="26" t="s">
         <v>414</v>
       </c>
       <c r="B49" s="3">
@@ -8400,7 +8445,7 @@
       <c r="U49" s="3"/>
     </row>
     <row r="50" spans="1:21" ht="78" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A50" s="3" t="s">
+      <c r="A50" s="26" t="s">
         <v>422</v>
       </c>
       <c r="B50" s="3">
@@ -8461,7 +8506,7 @@
       </c>
     </row>
     <row r="51" spans="1:21" ht="78" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A51" s="3" t="s">
+      <c r="A51" s="26" t="s">
         <v>433</v>
       </c>
       <c r="B51" s="3">
@@ -8516,7 +8561,7 @@
       <c r="U51" s="3"/>
     </row>
     <row r="52" spans="1:21" ht="78" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A52" s="3" t="s">
+      <c r="A52" s="26" t="s">
         <v>440</v>
       </c>
       <c r="B52" s="3">
@@ -8571,7 +8616,7 @@
       <c r="U52" s="3"/>
     </row>
     <row r="53" spans="1:21" ht="78" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A53" s="3" t="s">
+      <c r="A53" s="26" t="s">
         <v>448</v>
       </c>
       <c r="B53" s="3">
@@ -8626,7 +8671,7 @@
       <c r="U53" s="3"/>
     </row>
     <row r="54" spans="1:21" ht="78" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A54" s="3" t="s">
+      <c r="A54" s="26" t="s">
         <v>456</v>
       </c>
       <c r="B54" s="3">
@@ -8681,7 +8726,7 @@
       <c r="U54" s="3"/>
     </row>
     <row r="55" spans="1:21" ht="78" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A55" s="3" t="s">
+      <c r="A55" s="26" t="s">
         <v>463</v>
       </c>
       <c r="B55" s="3">
@@ -8736,7 +8781,7 @@
       <c r="U55" s="3"/>
     </row>
     <row r="56" spans="1:21" ht="78" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A56" s="3" t="s">
+      <c r="A56" s="26" t="s">
         <v>471</v>
       </c>
       <c r="B56" s="3">
@@ -8791,7 +8836,7 @@
       <c r="U56" s="3"/>
     </row>
     <row r="57" spans="1:21" ht="78" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A57" s="3" t="s">
+      <c r="A57" s="26" t="s">
         <v>478</v>
       </c>
       <c r="B57" s="3">
@@ -8846,7 +8891,7 @@
       <c r="U57" s="3"/>
     </row>
     <row r="58" spans="1:21" ht="78" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A58" s="3" t="s">
+      <c r="A58" s="26" t="s">
         <v>486</v>
       </c>
       <c r="B58" s="3">
@@ -15547,7 +15592,7 @@
       </c>
       <c r="B11" s="7" t="str">
         <f>COUNTIF('Backlog 12 Tuan'!P:P,"Done")&amp;" / "&amp;COUNTA('Backlog 12 Tuan'!A:A)-1&amp;" task Done"</f>
-        <v>22 / 168 task Done</v>
+        <v>25 / 168 task Done</v>
       </c>
     </row>
     <row r="12" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -15556,7 +15601,7 @@
       </c>
       <c r="B12" s="8">
         <f>COUNTIF('Backlog 12 Tuan'!P:P,"Done")/(COUNTA('Backlog 12 Tuan'!A:A)-1)</f>
-        <v>0.13095238095238096</v>
+        <v>0.14880952380952381</v>
       </c>
     </row>
     <row r="13" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Conplete from FF-03-01-1 to FF-03-03-2 : React app web
</commit_message>
<xml_diff>
--- a/plan/backlog-freshflow-mvp-12-tuan-updated.xlsx
+++ b/plan/backlog-freshflow-mvp-12-tuan-updated.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\FreshFlow\plan\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0A60F87F-EC6D-4FE2-95F5-CB8667EF5585}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DD2E82C9-392A-437D-8EC4-475B8202D835}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="600" yWindow="-120" windowWidth="28320" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -47,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2815" uniqueCount="1618">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2816" uniqueCount="1620">
   <si>
     <t>Task ID</t>
   </si>
@@ -4900,7 +4900,13 @@
     <t xml:space="preserve">LÀM NHẦM --- CẦN XXEM LẠI XEM ĐÃ ĐỦ CHƯA </t>
   </si>
   <si>
+    <t>In Progress</t>
+  </si>
+  <si>
     <t>13/9/2026</t>
+  </si>
+  <si>
+    <t>25/9/2026</t>
   </si>
 </sst>
 </file>
@@ -7384,7 +7390,7 @@
       </c>
       <c r="Q30" s="3"/>
       <c r="R30" s="3" t="s">
-        <v>1617</v>
+        <v>1618</v>
       </c>
       <c r="S30" s="3"/>
       <c r="T30" s="3"/>
@@ -7437,7 +7443,7 @@
         <v>266</v>
       </c>
       <c r="P31" s="3" t="s">
-        <v>71</v>
+        <v>1617</v>
       </c>
       <c r="Q31" s="3"/>
       <c r="R31" s="3"/>
@@ -7492,7 +7498,7 @@
         <v>290</v>
       </c>
       <c r="P32" s="3" t="s">
-        <v>71</v>
+        <v>1617</v>
       </c>
       <c r="Q32" s="3"/>
       <c r="R32" s="3"/>
@@ -7547,7 +7553,7 @@
         <v>290</v>
       </c>
       <c r="P33" s="3" t="s">
-        <v>71</v>
+        <v>1617</v>
       </c>
       <c r="Q33" s="3"/>
       <c r="R33" s="3"/>
@@ -7602,7 +7608,7 @@
         <v>241</v>
       </c>
       <c r="P34" s="3" t="s">
-        <v>71</v>
+        <v>1617</v>
       </c>
       <c r="Q34" s="3"/>
       <c r="R34" s="3"/>
@@ -7657,7 +7663,7 @@
         <v>312</v>
       </c>
       <c r="P35" s="3" t="s">
-        <v>71</v>
+        <v>1617</v>
       </c>
       <c r="Q35" s="3"/>
       <c r="R35" s="3"/>
@@ -7712,7 +7718,7 @@
         <v>320</v>
       </c>
       <c r="P36" s="3" t="s">
-        <v>71</v>
+        <v>1617</v>
       </c>
       <c r="Q36" s="3"/>
       <c r="R36" s="3"/>
@@ -8154,7 +8160,9 @@
       <c r="P44" s="3" t="s">
         <v>71</v>
       </c>
-      <c r="Q44" s="3"/>
+      <c r="Q44" s="3" t="s">
+        <v>1619</v>
+      </c>
       <c r="R44" s="3"/>
       <c r="S44" s="3"/>
       <c r="T44" s="3"/>

</xml_diff>

<commit_message>
git commit -m "feat(web/catalog): complete Sprint 3 merchant catalog features, tests and a11y polish
- [FF-03-04-1] ProductCreateForm with nested variants, inventory modes, and presets
- [FF-03-04-2] ProductEditModal, PATCH semantics, soft hide, and dependent category availability
- [FF-03-05-1] Toast notification system, ErrorBoundary, and EmptyState with dual CTA
- [FF-03-05-2] Comprehensive component tests (12 RTL tests + 67 smoke assertions)
- [FF-03-06-2] Accessibility & responsive pass: WCAG AA contrast, 100% label coverage, keyboard navigation
- [FF-03-07-1] Weekly review W03, component boundary review, refactor backlog, and 0 TODO audit
- Quality Gates: 100% pass on npm run lint (0 errors/warnings), npm test (104 assertions), npm run build"
</commit_message>
<xml_diff>
--- a/plan/backlog-freshflow-mvp-12-tuan-updated.xlsx
+++ b/plan/backlog-freshflow-mvp-12-tuan-updated.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30508"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30514"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\FreshFlow\plan\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DD2E82C9-392A-437D-8EC4-475B8202D835}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{895D1615-B2F6-488E-8B80-61585DB67812}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="600" yWindow="-120" windowWidth="28320" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -47,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2816" uniqueCount="1620">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2816" uniqueCount="1619">
   <si>
     <t>Task ID</t>
   </si>
@@ -4898,9 +4898,6 @@
   </si>
   <si>
     <t xml:space="preserve">LÀM NHẦM --- CẦN XXEM LẠI XEM ĐÃ ĐỦ CHƯA </t>
-  </si>
-  <si>
-    <t>In Progress</t>
   </si>
   <si>
     <t>13/9/2026</t>
@@ -7390,7 +7387,7 @@
       </c>
       <c r="Q30" s="3"/>
       <c r="R30" s="3" t="s">
-        <v>1618</v>
+        <v>1617</v>
       </c>
       <c r="S30" s="3"/>
       <c r="T30" s="3"/>
@@ -7443,7 +7440,7 @@
         <v>266</v>
       </c>
       <c r="P31" s="3" t="s">
-        <v>1617</v>
+        <v>53</v>
       </c>
       <c r="Q31" s="3"/>
       <c r="R31" s="3"/>
@@ -7498,7 +7495,7 @@
         <v>290</v>
       </c>
       <c r="P32" s="3" t="s">
-        <v>1617</v>
+        <v>53</v>
       </c>
       <c r="Q32" s="3"/>
       <c r="R32" s="3"/>
@@ -7553,7 +7550,7 @@
         <v>290</v>
       </c>
       <c r="P33" s="3" t="s">
-        <v>1617</v>
+        <v>53</v>
       </c>
       <c r="Q33" s="3"/>
       <c r="R33" s="3"/>
@@ -7608,7 +7605,7 @@
         <v>241</v>
       </c>
       <c r="P34" s="3" t="s">
-        <v>1617</v>
+        <v>53</v>
       </c>
       <c r="Q34" s="3"/>
       <c r="R34" s="3"/>
@@ -7663,7 +7660,7 @@
         <v>312</v>
       </c>
       <c r="P35" s="3" t="s">
-        <v>1617</v>
+        <v>53</v>
       </c>
       <c r="Q35" s="3"/>
       <c r="R35" s="3"/>
@@ -7718,7 +7715,7 @@
         <v>320</v>
       </c>
       <c r="P36" s="3" t="s">
-        <v>1617</v>
+        <v>53</v>
       </c>
       <c r="Q36" s="3"/>
       <c r="R36" s="3"/>
@@ -7773,7 +7770,7 @@
         <v>320</v>
       </c>
       <c r="P37" s="3" t="s">
-        <v>71</v>
+        <v>53</v>
       </c>
       <c r="Q37" s="3"/>
       <c r="R37" s="3"/>
@@ -7828,7 +7825,7 @@
         <v>335</v>
       </c>
       <c r="P38" s="3" t="s">
-        <v>71</v>
+        <v>53</v>
       </c>
       <c r="Q38" s="3"/>
       <c r="R38" s="3"/>
@@ -8161,7 +8158,7 @@
         <v>71</v>
       </c>
       <c r="Q44" s="3" t="s">
-        <v>1619</v>
+        <v>1618</v>
       </c>
       <c r="R44" s="3"/>
       <c r="S44" s="3"/>

</xml_diff>

<commit_message>
complete task backend FF-05-05-2
</commit_message>
<xml_diff>
--- a/plan/backlog-freshflow-mvp-12-tuan-updated.xlsx
+++ b/plan/backlog-freshflow-mvp-12-tuan-updated.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\FreshFlow\plan\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C90D02F1-871C-44F3-9E04-00B3C2F218EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DD486B3E-26D7-4B1E-B9BA-1808B9C95506}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="600" yWindow="-120" windowWidth="28320" windowHeight="16440" tabRatio="845" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -49,7 +49,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5590" uniqueCount="1854">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5575" uniqueCount="1838">
   <si>
     <t>FRESHFLOW MVP — TỔNG QUAN DỰ ÁN &amp; TIẾN ĐỘ THEO CỤC (BACKEND-FIRST DASHBOARD)</t>
   </si>
@@ -5550,67 +5550,19 @@
     <t>Docs khớp schema; restore smoke pass</t>
   </si>
   <si>
-    <t>28/09/2026</t>
-  </si>
-  <si>
-    <t>29/09/2026</t>
-  </si>
-  <si>
-    <t>30/09/2026</t>
-  </si>
-  <si>
-    <t>13/10/2026</t>
-  </si>
-  <si>
-    <t>14/10/2026</t>
-  </si>
-  <si>
-    <t>15/10/2026</t>
-  </si>
-  <si>
-    <t>16/10/2026</t>
-  </si>
-  <si>
-    <t>17/10/2026</t>
-  </si>
-  <si>
-    <t>18/10/2026</t>
-  </si>
-  <si>
-    <t>19/10/2026</t>
-  </si>
-  <si>
-    <t>20/10/2026</t>
-  </si>
-  <si>
-    <t>21/10/2026</t>
-  </si>
-  <si>
-    <t>22/10/2026</t>
-  </si>
-  <si>
-    <t>23/10/2026</t>
-  </si>
-  <si>
-    <t>24/10/2026</t>
-  </si>
-  <si>
-    <t>25/10/2026</t>
-  </si>
-  <si>
-    <t>26/10/2026</t>
-  </si>
-  <si>
-    <t>27/10/2026</t>
-  </si>
-  <si>
-    <t>28/10/2026</t>
-  </si>
-  <si>
-    <t>29/10/2026</t>
-  </si>
-  <si>
-    <t>30/10/2026</t>
+    <t>28/9/2026</t>
+  </si>
+  <si>
+    <t>28/9/1026</t>
+  </si>
+  <si>
+    <t>29/9/2026</t>
+  </si>
+  <si>
+    <t>30/9/2026</t>
+  </si>
+  <si>
+    <t>1/10/1016</t>
   </si>
 </sst>
 </file>
@@ -5713,7 +5665,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="43">
+  <fills count="45">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -5962,6 +5914,18 @@
         <bgColor rgb="FFD9E1F2"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="7">
     <border>
@@ -6051,7 +6015,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1"/>
   </cellStyleXfs>
-  <cellXfs count="75">
+  <cellXfs count="82">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -6215,32 +6179,9 @@
     <xf numFmtId="164" fontId="3" fillId="38" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="33" borderId="1" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="35" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="34" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="42" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="32" borderId="1" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="6" fillId="31" borderId="1" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -6256,13 +6197,59 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="34" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="35" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="42" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="33" borderId="1" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="17" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="43" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="44" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="13" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="15" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="14" fontId="15" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="15" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="14" fontId="3" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -6892,59 +6879,59 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:17" ht="36" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="59" t="s">
+      <c r="A1" s="70" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="57"/>
-      <c r="C1" s="57"/>
-      <c r="D1" s="57"/>
-      <c r="E1" s="57"/>
-      <c r="F1" s="57"/>
-      <c r="G1" s="57"/>
-      <c r="H1" s="57"/>
-      <c r="I1" s="57"/>
-      <c r="J1" s="57"/>
-      <c r="K1" s="57"/>
-      <c r="L1" s="57"/>
-      <c r="M1" s="57"/>
+      <c r="B1" s="64"/>
+      <c r="C1" s="64"/>
+      <c r="D1" s="64"/>
+      <c r="E1" s="64"/>
+      <c r="F1" s="64"/>
+      <c r="G1" s="64"/>
+      <c r="H1" s="64"/>
+      <c r="I1" s="64"/>
+      <c r="J1" s="64"/>
+      <c r="K1" s="64"/>
+      <c r="L1" s="64"/>
+      <c r="M1" s="64"/>
       <c r="N1" s="37"/>
       <c r="O1" s="37"/>
       <c r="P1" s="37"/>
       <c r="Q1" s="37"/>
     </row>
     <row r="2" spans="1:17" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="58" t="s">
+      <c r="A2" s="69" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="57"/>
-      <c r="C2" s="57"/>
-      <c r="D2" s="57"/>
-      <c r="E2" s="57"/>
-      <c r="F2" s="57"/>
-      <c r="G2" s="57"/>
-      <c r="H2" s="57"/>
-      <c r="I2" s="57"/>
-      <c r="J2" s="57"/>
-      <c r="K2" s="57"/>
-      <c r="L2" s="57"/>
-      <c r="M2" s="57"/>
+      <c r="B2" s="64"/>
+      <c r="C2" s="64"/>
+      <c r="D2" s="64"/>
+      <c r="E2" s="64"/>
+      <c r="F2" s="64"/>
+      <c r="G2" s="64"/>
+      <c r="H2" s="64"/>
+      <c r="I2" s="64"/>
+      <c r="J2" s="64"/>
+      <c r="K2" s="64"/>
+      <c r="L2" s="64"/>
+      <c r="M2" s="64"/>
     </row>
     <row r="4" spans="1:17" ht="26.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="63" t="s">
+      <c r="A4" s="66" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="57"/>
-      <c r="C4" s="57"/>
-      <c r="D4" s="57"/>
-      <c r="E4" s="57"/>
-      <c r="F4" s="57"/>
-      <c r="G4" s="57"/>
-      <c r="H4" s="57"/>
-      <c r="I4" s="57"/>
-      <c r="J4" s="57"/>
-      <c r="K4" s="57"/>
-      <c r="L4" s="57"/>
-      <c r="M4" s="57"/>
+      <c r="B4" s="64"/>
+      <c r="C4" s="64"/>
+      <c r="D4" s="64"/>
+      <c r="E4" s="64"/>
+      <c r="F4" s="64"/>
+      <c r="G4" s="64"/>
+      <c r="H4" s="64"/>
+      <c r="I4" s="64"/>
+      <c r="J4" s="64"/>
+      <c r="K4" s="64"/>
+      <c r="L4" s="64"/>
+      <c r="M4" s="64"/>
     </row>
     <row r="5" spans="1:17" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="38" t="s">
@@ -6956,18 +6943,18 @@
       <c r="C5" s="38" t="s">
         <v>5</v>
       </c>
-      <c r="D5" s="62" t="s">
+      <c r="D5" s="67" t="s">
         <v>6</v>
       </c>
-      <c r="E5" s="57"/>
-      <c r="F5" s="57"/>
-      <c r="G5" s="57"/>
-      <c r="H5" s="57"/>
-      <c r="I5" s="57"/>
-      <c r="J5" s="57"/>
-      <c r="K5" s="57"/>
-      <c r="L5" s="57"/>
-      <c r="M5" s="57"/>
+      <c r="E5" s="64"/>
+      <c r="F5" s="64"/>
+      <c r="G5" s="64"/>
+      <c r="H5" s="64"/>
+      <c r="I5" s="64"/>
+      <c r="J5" s="64"/>
+      <c r="K5" s="64"/>
+      <c r="L5" s="64"/>
+      <c r="M5" s="64"/>
     </row>
     <row r="6" spans="1:17" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="39" t="s">
@@ -6981,18 +6968,18 @@
         <f t="shared" ref="C6:C11" si="0">B6/$B$12</f>
         <v>0.15476190476190477</v>
       </c>
-      <c r="D6" s="61" t="s">
+      <c r="D6" s="63" t="s">
         <v>8</v>
       </c>
-      <c r="E6" s="57"/>
-      <c r="F6" s="57"/>
-      <c r="G6" s="57"/>
-      <c r="H6" s="57"/>
-      <c r="I6" s="57"/>
-      <c r="J6" s="57"/>
-      <c r="K6" s="57"/>
-      <c r="L6" s="57"/>
-      <c r="M6" s="57"/>
+      <c r="E6" s="64"/>
+      <c r="F6" s="64"/>
+      <c r="G6" s="64"/>
+      <c r="H6" s="64"/>
+      <c r="I6" s="64"/>
+      <c r="J6" s="64"/>
+      <c r="K6" s="64"/>
+      <c r="L6" s="64"/>
+      <c r="M6" s="64"/>
     </row>
     <row r="7" spans="1:17" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="43" t="s">
@@ -7006,18 +6993,18 @@
         <f t="shared" si="0"/>
         <v>0.16071428571428573</v>
       </c>
-      <c r="D7" s="61" t="s">
+      <c r="D7" s="63" t="s">
         <v>10</v>
       </c>
-      <c r="E7" s="57"/>
-      <c r="F7" s="57"/>
-      <c r="G7" s="57"/>
-      <c r="H7" s="57"/>
-      <c r="I7" s="57"/>
-      <c r="J7" s="57"/>
-      <c r="K7" s="57"/>
-      <c r="L7" s="57"/>
-      <c r="M7" s="57"/>
+      <c r="E7" s="64"/>
+      <c r="F7" s="64"/>
+      <c r="G7" s="64"/>
+      <c r="H7" s="64"/>
+      <c r="I7" s="64"/>
+      <c r="J7" s="64"/>
+      <c r="K7" s="64"/>
+      <c r="L7" s="64"/>
+      <c r="M7" s="64"/>
     </row>
     <row r="8" spans="1:17" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="44" t="s">
@@ -7025,24 +7012,24 @@
       </c>
       <c r="B8" s="40">
         <f>COUNTIF('Kế hoạch theo cục'!$P$3:$P$250, "In Progress")</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C8" s="41">
         <f t="shared" si="0"/>
-        <v>1.1904761904761904E-2</v>
-      </c>
-      <c r="D8" s="61" t="s">
+        <v>1.7857142857142856E-2</v>
+      </c>
+      <c r="D8" s="63" t="s">
         <v>12</v>
       </c>
-      <c r="E8" s="57"/>
-      <c r="F8" s="57"/>
-      <c r="G8" s="57"/>
-      <c r="H8" s="57"/>
-      <c r="I8" s="57"/>
-      <c r="J8" s="57"/>
-      <c r="K8" s="57"/>
-      <c r="L8" s="57"/>
-      <c r="M8" s="57"/>
+      <c r="E8" s="64"/>
+      <c r="F8" s="64"/>
+      <c r="G8" s="64"/>
+      <c r="H8" s="64"/>
+      <c r="I8" s="64"/>
+      <c r="J8" s="64"/>
+      <c r="K8" s="64"/>
+      <c r="L8" s="64"/>
+      <c r="M8" s="64"/>
     </row>
     <row r="9" spans="1:17" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="45" t="s">
@@ -7056,18 +7043,18 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="D9" s="61" t="s">
+      <c r="D9" s="63" t="s">
         <v>14</v>
       </c>
-      <c r="E9" s="57"/>
-      <c r="F9" s="57"/>
-      <c r="G9" s="57"/>
-      <c r="H9" s="57"/>
-      <c r="I9" s="57"/>
-      <c r="J9" s="57"/>
-      <c r="K9" s="57"/>
-      <c r="L9" s="57"/>
-      <c r="M9" s="57"/>
+      <c r="E9" s="64"/>
+      <c r="F9" s="64"/>
+      <c r="G9" s="64"/>
+      <c r="H9" s="64"/>
+      <c r="I9" s="64"/>
+      <c r="J9" s="64"/>
+      <c r="K9" s="64"/>
+      <c r="L9" s="64"/>
+      <c r="M9" s="64"/>
     </row>
     <row r="10" spans="1:17" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="46" t="s">
@@ -7081,18 +7068,18 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="D10" s="61" t="s">
+      <c r="D10" s="63" t="s">
         <v>16</v>
       </c>
-      <c r="E10" s="57"/>
-      <c r="F10" s="57"/>
-      <c r="G10" s="57"/>
-      <c r="H10" s="57"/>
-      <c r="I10" s="57"/>
-      <c r="J10" s="57"/>
-      <c r="K10" s="57"/>
-      <c r="L10" s="57"/>
-      <c r="M10" s="57"/>
+      <c r="E10" s="64"/>
+      <c r="F10" s="64"/>
+      <c r="G10" s="64"/>
+      <c r="H10" s="64"/>
+      <c r="I10" s="64"/>
+      <c r="J10" s="64"/>
+      <c r="K10" s="64"/>
+      <c r="L10" s="64"/>
+      <c r="M10" s="64"/>
     </row>
     <row r="11" spans="1:17" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="47" t="s">
@@ -7100,24 +7087,24 @@
       </c>
       <c r="B11" s="40">
         <f>COUNTIF('Kế hoạch theo cục'!$P$3:$P$250, "Todo")</f>
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C11" s="41">
         <f t="shared" si="0"/>
-        <v>0.67261904761904767</v>
-      </c>
-      <c r="D11" s="61" t="s">
+        <v>0.66666666666666663</v>
+      </c>
+      <c r="D11" s="63" t="s">
         <v>18</v>
       </c>
-      <c r="E11" s="57"/>
-      <c r="F11" s="57"/>
-      <c r="G11" s="57"/>
-      <c r="H11" s="57"/>
-      <c r="I11" s="57"/>
-      <c r="J11" s="57"/>
-      <c r="K11" s="57"/>
-      <c r="L11" s="57"/>
-      <c r="M11" s="57"/>
+      <c r="E11" s="64"/>
+      <c r="F11" s="64"/>
+      <c r="G11" s="64"/>
+      <c r="H11" s="64"/>
+      <c r="I11" s="64"/>
+      <c r="J11" s="64"/>
+      <c r="K11" s="64"/>
+      <c r="L11" s="64"/>
+      <c r="M11" s="64"/>
     </row>
     <row r="12" spans="1:17" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="48" t="s">
@@ -7131,35 +7118,35 @@
         <f>SUM(C6:C11)</f>
         <v>1</v>
       </c>
-      <c r="D12" s="64" t="s">
+      <c r="D12" s="68" t="s">
         <v>20</v>
       </c>
-      <c r="E12" s="57"/>
-      <c r="F12" s="57"/>
-      <c r="G12" s="57"/>
-      <c r="H12" s="57"/>
-      <c r="I12" s="57"/>
-      <c r="J12" s="57"/>
-      <c r="K12" s="57"/>
-      <c r="L12" s="57"/>
-      <c r="M12" s="57"/>
+      <c r="E12" s="64"/>
+      <c r="F12" s="64"/>
+      <c r="G12" s="64"/>
+      <c r="H12" s="64"/>
+      <c r="I12" s="64"/>
+      <c r="J12" s="64"/>
+      <c r="K12" s="64"/>
+      <c r="L12" s="64"/>
+      <c r="M12" s="64"/>
     </row>
     <row r="14" spans="1:17" ht="26.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="63" t="s">
+      <c r="A14" s="66" t="s">
         <v>21</v>
       </c>
-      <c r="B14" s="57"/>
-      <c r="C14" s="57"/>
-      <c r="D14" s="57"/>
-      <c r="E14" s="57"/>
-      <c r="F14" s="57"/>
-      <c r="G14" s="57"/>
-      <c r="H14" s="57"/>
-      <c r="I14" s="57"/>
-      <c r="J14" s="57"/>
-      <c r="K14" s="57"/>
-      <c r="L14" s="57"/>
-      <c r="M14" s="57"/>
+      <c r="B14" s="64"/>
+      <c r="C14" s="64"/>
+      <c r="D14" s="64"/>
+      <c r="E14" s="64"/>
+      <c r="F14" s="64"/>
+      <c r="G14" s="64"/>
+      <c r="H14" s="64"/>
+      <c r="I14" s="64"/>
+      <c r="J14" s="64"/>
+      <c r="K14" s="64"/>
+      <c r="L14" s="64"/>
+      <c r="M14" s="64"/>
     </row>
     <row r="15" spans="1:17" ht="26.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="51" t="s">
@@ -7274,7 +7261,7 @@
       </c>
       <c r="F17" s="44">
         <f>COUNTIFS('Kế hoạch theo cục'!$C$3:$C$250, "CỤC 2", 'Kế hoạch theo cục'!$P$3:$P$250, "In Progress")</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G17" s="53">
         <f>COUNTIFS('Kế hoạch theo cục'!$C$3:$C$250, "CỤC 2", 'Kế hoạch theo cục'!$P$3:$P$250, "Blocked") + COUNTIFS('Kế hoạch theo cục'!$C$3:$C$250, "CỤC 2", 'Kế hoạch theo cục'!$P$3:$P$250, "Deferred")</f>
@@ -7282,7 +7269,7 @@
       </c>
       <c r="H17" s="53">
         <f>COUNTIFS('Kế hoạch theo cục'!$C$3:$C$250, "CỤC 2", 'Kế hoạch theo cục'!$P$3:$P$250, "Todo")</f>
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="I17" s="54">
         <f t="shared" si="1"/>
@@ -7294,11 +7281,11 @@
       </c>
       <c r="K17" s="56">
         <f t="shared" si="3"/>
-        <v>1.6949152542372881E-2</v>
+        <v>3.3898305084745763E-2</v>
       </c>
       <c r="L17" s="41">
         <f t="shared" si="4"/>
-        <v>0.66101694915254239</v>
+        <v>0.64406779661016944</v>
       </c>
       <c r="M17" s="42" t="s">
         <v>36</v>
@@ -7529,7 +7516,7 @@
       </c>
       <c r="F22" s="48">
         <f t="shared" si="5"/>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G22" s="48">
         <f t="shared" si="5"/>
@@ -7537,7 +7524,7 @@
       </c>
       <c r="H22" s="48">
         <f t="shared" si="5"/>
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="I22" s="49">
         <f t="shared" si="1"/>
@@ -7549,32 +7536,32 @@
       </c>
       <c r="K22" s="49">
         <f t="shared" si="3"/>
-        <v>1.1904761904761904E-2</v>
+        <v>1.7857142857142856E-2</v>
       </c>
       <c r="L22" s="49">
         <f t="shared" si="4"/>
-        <v>0.67261904761904767</v>
+        <v>0.66666666666666663</v>
       </c>
       <c r="M22" s="50" t="s">
         <v>51</v>
       </c>
     </row>
     <row r="24" spans="1:13" ht="26.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="63" t="s">
+      <c r="A24" s="66" t="s">
         <v>52</v>
       </c>
-      <c r="B24" s="57"/>
-      <c r="C24" s="57"/>
-      <c r="D24" s="57"/>
-      <c r="E24" s="57"/>
-      <c r="F24" s="57"/>
-      <c r="G24" s="57"/>
-      <c r="H24" s="57"/>
-      <c r="I24" s="57"/>
-      <c r="J24" s="57"/>
-      <c r="K24" s="57"/>
-      <c r="L24" s="57"/>
-      <c r="M24" s="57"/>
+      <c r="B24" s="64"/>
+      <c r="C24" s="64"/>
+      <c r="D24" s="64"/>
+      <c r="E24" s="64"/>
+      <c r="F24" s="64"/>
+      <c r="G24" s="64"/>
+      <c r="H24" s="64"/>
+      <c r="I24" s="64"/>
+      <c r="J24" s="64"/>
+      <c r="K24" s="64"/>
+      <c r="L24" s="64"/>
+      <c r="M24" s="64"/>
     </row>
     <row r="25" spans="1:13" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="26" spans="1:13" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -7608,21 +7595,21 @@
     <row r="54" spans="1:13" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="55" spans="1:13" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="56" spans="1:13" ht="26.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A56" s="63" t="s">
+      <c r="A56" s="66" t="s">
         <v>53</v>
       </c>
-      <c r="B56" s="57"/>
-      <c r="C56" s="57"/>
-      <c r="D56" s="57"/>
-      <c r="E56" s="57"/>
-      <c r="F56" s="57"/>
-      <c r="G56" s="57"/>
-      <c r="H56" s="57"/>
-      <c r="I56" s="57"/>
-      <c r="J56" s="57"/>
-      <c r="K56" s="57"/>
-      <c r="L56" s="57"/>
-      <c r="M56" s="57"/>
+      <c r="B56" s="64"/>
+      <c r="C56" s="64"/>
+      <c r="D56" s="64"/>
+      <c r="E56" s="64"/>
+      <c r="F56" s="64"/>
+      <c r="G56" s="64"/>
+      <c r="H56" s="64"/>
+      <c r="I56" s="64"/>
+      <c r="J56" s="64"/>
+      <c r="K56" s="64"/>
+      <c r="L56" s="64"/>
+      <c r="M56" s="64"/>
     </row>
     <row r="57" spans="1:13" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A57" s="38" t="s">
@@ -7634,18 +7621,18 @@
       <c r="C57" s="38" t="s">
         <v>55</v>
       </c>
-      <c r="D57" s="62" t="s">
+      <c r="D57" s="67" t="s">
         <v>56</v>
       </c>
-      <c r="E57" s="57"/>
-      <c r="F57" s="57"/>
-      <c r="G57" s="57"/>
-      <c r="H57" s="57"/>
-      <c r="I57" s="57"/>
-      <c r="J57" s="57"/>
-      <c r="K57" s="57"/>
-      <c r="L57" s="57"/>
-      <c r="M57" s="57"/>
+      <c r="E57" s="64"/>
+      <c r="F57" s="64"/>
+      <c r="G57" s="64"/>
+      <c r="H57" s="64"/>
+      <c r="I57" s="64"/>
+      <c r="J57" s="64"/>
+      <c r="K57" s="64"/>
+      <c r="L57" s="64"/>
+      <c r="M57" s="64"/>
     </row>
     <row r="58" spans="1:13" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A58" s="40" t="s">
@@ -7657,18 +7644,18 @@
       <c r="C58" s="53">
         <v>4</v>
       </c>
-      <c r="D58" s="60" t="s">
+      <c r="D58" s="65" t="s">
         <v>58</v>
       </c>
-      <c r="E58" s="57"/>
-      <c r="F58" s="57"/>
-      <c r="G58" s="57"/>
-      <c r="H58" s="57"/>
-      <c r="I58" s="57"/>
-      <c r="J58" s="57"/>
-      <c r="K58" s="57"/>
-      <c r="L58" s="57"/>
-      <c r="M58" s="57"/>
+      <c r="E58" s="64"/>
+      <c r="F58" s="64"/>
+      <c r="G58" s="64"/>
+      <c r="H58" s="64"/>
+      <c r="I58" s="64"/>
+      <c r="J58" s="64"/>
+      <c r="K58" s="64"/>
+      <c r="L58" s="64"/>
+      <c r="M58" s="64"/>
     </row>
     <row r="59" spans="1:13" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A59" s="40" t="s">
@@ -7680,18 +7667,18 @@
       <c r="C59" s="53">
         <v>4</v>
       </c>
-      <c r="D59" s="60" t="s">
+      <c r="D59" s="65" t="s">
         <v>60</v>
       </c>
-      <c r="E59" s="57"/>
-      <c r="F59" s="57"/>
-      <c r="G59" s="57"/>
-      <c r="H59" s="57"/>
-      <c r="I59" s="57"/>
-      <c r="J59" s="57"/>
-      <c r="K59" s="57"/>
-      <c r="L59" s="57"/>
-      <c r="M59" s="57"/>
+      <c r="E59" s="64"/>
+      <c r="F59" s="64"/>
+      <c r="G59" s="64"/>
+      <c r="H59" s="64"/>
+      <c r="I59" s="64"/>
+      <c r="J59" s="64"/>
+      <c r="K59" s="64"/>
+      <c r="L59" s="64"/>
+      <c r="M59" s="64"/>
     </row>
     <row r="60" spans="1:13" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A60" s="40" t="s">
@@ -7703,18 +7690,18 @@
       <c r="C60" s="53">
         <v>6</v>
       </c>
-      <c r="D60" s="60" t="s">
+      <c r="D60" s="65" t="s">
         <v>62</v>
       </c>
-      <c r="E60" s="57"/>
-      <c r="F60" s="57"/>
-      <c r="G60" s="57"/>
-      <c r="H60" s="57"/>
-      <c r="I60" s="57"/>
-      <c r="J60" s="57"/>
-      <c r="K60" s="57"/>
-      <c r="L60" s="57"/>
-      <c r="M60" s="57"/>
+      <c r="E60" s="64"/>
+      <c r="F60" s="64"/>
+      <c r="G60" s="64"/>
+      <c r="H60" s="64"/>
+      <c r="I60" s="64"/>
+      <c r="J60" s="64"/>
+      <c r="K60" s="64"/>
+      <c r="L60" s="64"/>
+      <c r="M60" s="64"/>
     </row>
     <row r="61" spans="1:13" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A61" s="40" t="s">
@@ -7726,18 +7713,18 @@
       <c r="C61" s="53">
         <v>14</v>
       </c>
-      <c r="D61" s="60" t="s">
+      <c r="D61" s="65" t="s">
         <v>64</v>
       </c>
-      <c r="E61" s="57"/>
-      <c r="F61" s="57"/>
-      <c r="G61" s="57"/>
-      <c r="H61" s="57"/>
-      <c r="I61" s="57"/>
-      <c r="J61" s="57"/>
-      <c r="K61" s="57"/>
-      <c r="L61" s="57"/>
-      <c r="M61" s="57"/>
+      <c r="E61" s="64"/>
+      <c r="F61" s="64"/>
+      <c r="G61" s="64"/>
+      <c r="H61" s="64"/>
+      <c r="I61" s="64"/>
+      <c r="J61" s="64"/>
+      <c r="K61" s="64"/>
+      <c r="L61" s="64"/>
+      <c r="M61" s="64"/>
     </row>
     <row r="62" spans="1:13" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A62" s="40" t="s">
@@ -7749,18 +7736,18 @@
       <c r="C62" s="53">
         <v>10</v>
       </c>
-      <c r="D62" s="60" t="s">
+      <c r="D62" s="65" t="s">
         <v>66</v>
       </c>
-      <c r="E62" s="57"/>
-      <c r="F62" s="57"/>
-      <c r="G62" s="57"/>
-      <c r="H62" s="57"/>
-      <c r="I62" s="57"/>
-      <c r="J62" s="57"/>
-      <c r="K62" s="57"/>
-      <c r="L62" s="57"/>
-      <c r="M62" s="57"/>
+      <c r="E62" s="64"/>
+      <c r="F62" s="64"/>
+      <c r="G62" s="64"/>
+      <c r="H62" s="64"/>
+      <c r="I62" s="64"/>
+      <c r="J62" s="64"/>
+      <c r="K62" s="64"/>
+      <c r="L62" s="64"/>
+      <c r="M62" s="64"/>
     </row>
     <row r="63" spans="1:13" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A63" s="40" t="s">
@@ -7772,18 +7759,18 @@
       <c r="C63" s="53">
         <v>1</v>
       </c>
-      <c r="D63" s="60" t="s">
+      <c r="D63" s="65" t="s">
         <v>68</v>
       </c>
-      <c r="E63" s="57"/>
-      <c r="F63" s="57"/>
-      <c r="G63" s="57"/>
-      <c r="H63" s="57"/>
-      <c r="I63" s="57"/>
-      <c r="J63" s="57"/>
-      <c r="K63" s="57"/>
-      <c r="L63" s="57"/>
-      <c r="M63" s="57"/>
+      <c r="E63" s="64"/>
+      <c r="F63" s="64"/>
+      <c r="G63" s="64"/>
+      <c r="H63" s="64"/>
+      <c r="I63" s="64"/>
+      <c r="J63" s="64"/>
+      <c r="K63" s="64"/>
+      <c r="L63" s="64"/>
+      <c r="M63" s="64"/>
     </row>
     <row r="64" spans="1:13" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A64" s="40" t="s">
@@ -7795,18 +7782,18 @@
       <c r="C64" s="53">
         <v>7</v>
       </c>
-      <c r="D64" s="60" t="s">
+      <c r="D64" s="65" t="s">
         <v>70</v>
       </c>
-      <c r="E64" s="57"/>
-      <c r="F64" s="57"/>
-      <c r="G64" s="57"/>
-      <c r="H64" s="57"/>
-      <c r="I64" s="57"/>
-      <c r="J64" s="57"/>
-      <c r="K64" s="57"/>
-      <c r="L64" s="57"/>
-      <c r="M64" s="57"/>
+      <c r="E64" s="64"/>
+      <c r="F64" s="64"/>
+      <c r="G64" s="64"/>
+      <c r="H64" s="64"/>
+      <c r="I64" s="64"/>
+      <c r="J64" s="64"/>
+      <c r="K64" s="64"/>
+      <c r="L64" s="64"/>
+      <c r="M64" s="64"/>
     </row>
     <row r="65" spans="1:13" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A65" s="40" t="s">
@@ -7818,18 +7805,18 @@
       <c r="C65" s="53">
         <v>12</v>
       </c>
-      <c r="D65" s="60" t="s">
+      <c r="D65" s="65" t="s">
         <v>72</v>
       </c>
-      <c r="E65" s="57"/>
-      <c r="F65" s="57"/>
-      <c r="G65" s="57"/>
-      <c r="H65" s="57"/>
-      <c r="I65" s="57"/>
-      <c r="J65" s="57"/>
-      <c r="K65" s="57"/>
-      <c r="L65" s="57"/>
-      <c r="M65" s="57"/>
+      <c r="E65" s="64"/>
+      <c r="F65" s="64"/>
+      <c r="G65" s="64"/>
+      <c r="H65" s="64"/>
+      <c r="I65" s="64"/>
+      <c r="J65" s="64"/>
+      <c r="K65" s="64"/>
+      <c r="L65" s="64"/>
+      <c r="M65" s="64"/>
     </row>
     <row r="66" spans="1:13" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A66" s="40" t="s">
@@ -7841,18 +7828,18 @@
       <c r="C66" s="53">
         <v>7</v>
       </c>
-      <c r="D66" s="60" t="s">
+      <c r="D66" s="65" t="s">
         <v>74</v>
       </c>
-      <c r="E66" s="57"/>
-      <c r="F66" s="57"/>
-      <c r="G66" s="57"/>
-      <c r="H66" s="57"/>
-      <c r="I66" s="57"/>
-      <c r="J66" s="57"/>
-      <c r="K66" s="57"/>
-      <c r="L66" s="57"/>
-      <c r="M66" s="57"/>
+      <c r="E66" s="64"/>
+      <c r="F66" s="64"/>
+      <c r="G66" s="64"/>
+      <c r="H66" s="64"/>
+      <c r="I66" s="64"/>
+      <c r="J66" s="64"/>
+      <c r="K66" s="64"/>
+      <c r="L66" s="64"/>
+      <c r="M66" s="64"/>
     </row>
     <row r="67" spans="1:13" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A67" s="40" t="s">
@@ -7864,18 +7851,18 @@
       <c r="C67" s="53">
         <v>7</v>
       </c>
-      <c r="D67" s="60" t="s">
+      <c r="D67" s="65" t="s">
         <v>76</v>
       </c>
-      <c r="E67" s="57"/>
-      <c r="F67" s="57"/>
-      <c r="G67" s="57"/>
-      <c r="H67" s="57"/>
-      <c r="I67" s="57"/>
-      <c r="J67" s="57"/>
-      <c r="K67" s="57"/>
-      <c r="L67" s="57"/>
-      <c r="M67" s="57"/>
+      <c r="E67" s="64"/>
+      <c r="F67" s="64"/>
+      <c r="G67" s="64"/>
+      <c r="H67" s="64"/>
+      <c r="I67" s="64"/>
+      <c r="J67" s="64"/>
+      <c r="K67" s="64"/>
+      <c r="L67" s="64"/>
+      <c r="M67" s="64"/>
     </row>
     <row r="68" spans="1:13" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A68" s="40" t="s">
@@ -7887,18 +7874,18 @@
       <c r="C68" s="53">
         <v>4</v>
       </c>
-      <c r="D68" s="60" t="s">
+      <c r="D68" s="65" t="s">
         <v>78</v>
       </c>
-      <c r="E68" s="57"/>
-      <c r="F68" s="57"/>
-      <c r="G68" s="57"/>
-      <c r="H68" s="57"/>
-      <c r="I68" s="57"/>
-      <c r="J68" s="57"/>
-      <c r="K68" s="57"/>
-      <c r="L68" s="57"/>
-      <c r="M68" s="57"/>
+      <c r="E68" s="64"/>
+      <c r="F68" s="64"/>
+      <c r="G68" s="64"/>
+      <c r="H68" s="64"/>
+      <c r="I68" s="64"/>
+      <c r="J68" s="64"/>
+      <c r="K68" s="64"/>
+      <c r="L68" s="64"/>
+      <c r="M68" s="64"/>
     </row>
     <row r="69" spans="1:13" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A69" s="40" t="s">
@@ -7910,18 +7897,18 @@
       <c r="C69" s="53">
         <v>10</v>
       </c>
-      <c r="D69" s="60" t="s">
+      <c r="D69" s="65" t="s">
         <v>80</v>
       </c>
-      <c r="E69" s="57"/>
-      <c r="F69" s="57"/>
-      <c r="G69" s="57"/>
-      <c r="H69" s="57"/>
-      <c r="I69" s="57"/>
-      <c r="J69" s="57"/>
-      <c r="K69" s="57"/>
-      <c r="L69" s="57"/>
-      <c r="M69" s="57"/>
+      <c r="E69" s="64"/>
+      <c r="F69" s="64"/>
+      <c r="G69" s="64"/>
+      <c r="H69" s="64"/>
+      <c r="I69" s="64"/>
+      <c r="J69" s="64"/>
+      <c r="K69" s="64"/>
+      <c r="L69" s="64"/>
+      <c r="M69" s="64"/>
     </row>
     <row r="70" spans="1:13" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A70" s="40" t="s">
@@ -7933,18 +7920,18 @@
       <c r="C70" s="53">
         <v>3</v>
       </c>
-      <c r="D70" s="60" t="s">
+      <c r="D70" s="65" t="s">
         <v>82</v>
       </c>
-      <c r="E70" s="57"/>
-      <c r="F70" s="57"/>
-      <c r="G70" s="57"/>
-      <c r="H70" s="57"/>
-      <c r="I70" s="57"/>
-      <c r="J70" s="57"/>
-      <c r="K70" s="57"/>
-      <c r="L70" s="57"/>
-      <c r="M70" s="57"/>
+      <c r="E70" s="64"/>
+      <c r="F70" s="64"/>
+      <c r="G70" s="64"/>
+      <c r="H70" s="64"/>
+      <c r="I70" s="64"/>
+      <c r="J70" s="64"/>
+      <c r="K70" s="64"/>
+      <c r="L70" s="64"/>
+      <c r="M70" s="64"/>
     </row>
     <row r="71" spans="1:13" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A71" s="40" t="s">
@@ -7956,18 +7943,18 @@
       <c r="C71" s="53">
         <v>3</v>
       </c>
-      <c r="D71" s="60" t="s">
+      <c r="D71" s="65" t="s">
         <v>84</v>
       </c>
-      <c r="E71" s="57"/>
-      <c r="F71" s="57"/>
-      <c r="G71" s="57"/>
-      <c r="H71" s="57"/>
-      <c r="I71" s="57"/>
-      <c r="J71" s="57"/>
-      <c r="K71" s="57"/>
-      <c r="L71" s="57"/>
-      <c r="M71" s="57"/>
+      <c r="E71" s="64"/>
+      <c r="F71" s="64"/>
+      <c r="G71" s="64"/>
+      <c r="H71" s="64"/>
+      <c r="I71" s="64"/>
+      <c r="J71" s="64"/>
+      <c r="K71" s="64"/>
+      <c r="L71" s="64"/>
+      <c r="M71" s="64"/>
     </row>
     <row r="72" spans="1:13" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A72" s="40" t="s">
@@ -7979,18 +7966,18 @@
       <c r="C72" s="53">
         <v>6</v>
       </c>
-      <c r="D72" s="60" t="s">
+      <c r="D72" s="65" t="s">
         <v>86</v>
       </c>
-      <c r="E72" s="57"/>
-      <c r="F72" s="57"/>
-      <c r="G72" s="57"/>
-      <c r="H72" s="57"/>
-      <c r="I72" s="57"/>
-      <c r="J72" s="57"/>
-      <c r="K72" s="57"/>
-      <c r="L72" s="57"/>
-      <c r="M72" s="57"/>
+      <c r="E72" s="64"/>
+      <c r="F72" s="64"/>
+      <c r="G72" s="64"/>
+      <c r="H72" s="64"/>
+      <c r="I72" s="64"/>
+      <c r="J72" s="64"/>
+      <c r="K72" s="64"/>
+      <c r="L72" s="64"/>
+      <c r="M72" s="64"/>
     </row>
     <row r="73" spans="1:13" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A73" s="40" t="s">
@@ -8002,18 +7989,18 @@
       <c r="C73" s="53">
         <v>3</v>
       </c>
-      <c r="D73" s="60" t="s">
+      <c r="D73" s="65" t="s">
         <v>88</v>
       </c>
-      <c r="E73" s="57"/>
-      <c r="F73" s="57"/>
-      <c r="G73" s="57"/>
-      <c r="H73" s="57"/>
-      <c r="I73" s="57"/>
-      <c r="J73" s="57"/>
-      <c r="K73" s="57"/>
-      <c r="L73" s="57"/>
-      <c r="M73" s="57"/>
+      <c r="E73" s="64"/>
+      <c r="F73" s="64"/>
+      <c r="G73" s="64"/>
+      <c r="H73" s="64"/>
+      <c r="I73" s="64"/>
+      <c r="J73" s="64"/>
+      <c r="K73" s="64"/>
+      <c r="L73" s="64"/>
+      <c r="M73" s="64"/>
     </row>
     <row r="74" spans="1:13" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A74" s="40" t="s">
@@ -8025,18 +8012,18 @@
       <c r="C74" s="53">
         <v>3</v>
       </c>
-      <c r="D74" s="60" t="s">
+      <c r="D74" s="65" t="s">
         <v>90</v>
       </c>
-      <c r="E74" s="57"/>
-      <c r="F74" s="57"/>
-      <c r="G74" s="57"/>
-      <c r="H74" s="57"/>
-      <c r="I74" s="57"/>
-      <c r="J74" s="57"/>
-      <c r="K74" s="57"/>
-      <c r="L74" s="57"/>
-      <c r="M74" s="57"/>
+      <c r="E74" s="64"/>
+      <c r="F74" s="64"/>
+      <c r="G74" s="64"/>
+      <c r="H74" s="64"/>
+      <c r="I74" s="64"/>
+      <c r="J74" s="64"/>
+      <c r="K74" s="64"/>
+      <c r="L74" s="64"/>
+      <c r="M74" s="64"/>
     </row>
     <row r="75" spans="1:13" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A75" s="40" t="s">
@@ -8048,18 +8035,18 @@
       <c r="C75" s="53">
         <v>4</v>
       </c>
-      <c r="D75" s="60" t="s">
+      <c r="D75" s="65" t="s">
         <v>92</v>
       </c>
-      <c r="E75" s="57"/>
-      <c r="F75" s="57"/>
-      <c r="G75" s="57"/>
-      <c r="H75" s="57"/>
-      <c r="I75" s="57"/>
-      <c r="J75" s="57"/>
-      <c r="K75" s="57"/>
-      <c r="L75" s="57"/>
-      <c r="M75" s="57"/>
+      <c r="E75" s="64"/>
+      <c r="F75" s="64"/>
+      <c r="G75" s="64"/>
+      <c r="H75" s="64"/>
+      <c r="I75" s="64"/>
+      <c r="J75" s="64"/>
+      <c r="K75" s="64"/>
+      <c r="L75" s="64"/>
+      <c r="M75" s="64"/>
     </row>
     <row r="76" spans="1:13" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A76" s="40" t="s">
@@ -8071,18 +8058,18 @@
       <c r="C76" s="53">
         <v>10</v>
       </c>
-      <c r="D76" s="60" t="s">
+      <c r="D76" s="65" t="s">
         <v>94</v>
       </c>
-      <c r="E76" s="57"/>
-      <c r="F76" s="57"/>
-      <c r="G76" s="57"/>
-      <c r="H76" s="57"/>
-      <c r="I76" s="57"/>
-      <c r="J76" s="57"/>
-      <c r="K76" s="57"/>
-      <c r="L76" s="57"/>
-      <c r="M76" s="57"/>
+      <c r="E76" s="64"/>
+      <c r="F76" s="64"/>
+      <c r="G76" s="64"/>
+      <c r="H76" s="64"/>
+      <c r="I76" s="64"/>
+      <c r="J76" s="64"/>
+      <c r="K76" s="64"/>
+      <c r="L76" s="64"/>
+      <c r="M76" s="64"/>
     </row>
     <row r="77" spans="1:13" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A77" s="40" t="s">
@@ -8094,18 +8081,18 @@
       <c r="C77" s="53">
         <v>8</v>
       </c>
-      <c r="D77" s="60" t="s">
+      <c r="D77" s="65" t="s">
         <v>96</v>
       </c>
-      <c r="E77" s="57"/>
-      <c r="F77" s="57"/>
-      <c r="G77" s="57"/>
-      <c r="H77" s="57"/>
-      <c r="I77" s="57"/>
-      <c r="J77" s="57"/>
-      <c r="K77" s="57"/>
-      <c r="L77" s="57"/>
-      <c r="M77" s="57"/>
+      <c r="E77" s="64"/>
+      <c r="F77" s="64"/>
+      <c r="G77" s="64"/>
+      <c r="H77" s="64"/>
+      <c r="I77" s="64"/>
+      <c r="J77" s="64"/>
+      <c r="K77" s="64"/>
+      <c r="L77" s="64"/>
+      <c r="M77" s="64"/>
     </row>
     <row r="78" spans="1:13" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A78" s="40" t="s">
@@ -8117,18 +8104,18 @@
       <c r="C78" s="53">
         <v>3</v>
       </c>
-      <c r="D78" s="60" t="s">
+      <c r="D78" s="65" t="s">
         <v>98</v>
       </c>
-      <c r="E78" s="57"/>
-      <c r="F78" s="57"/>
-      <c r="G78" s="57"/>
-      <c r="H78" s="57"/>
-      <c r="I78" s="57"/>
-      <c r="J78" s="57"/>
-      <c r="K78" s="57"/>
-      <c r="L78" s="57"/>
-      <c r="M78" s="57"/>
+      <c r="E78" s="64"/>
+      <c r="F78" s="64"/>
+      <c r="G78" s="64"/>
+      <c r="H78" s="64"/>
+      <c r="I78" s="64"/>
+      <c r="J78" s="64"/>
+      <c r="K78" s="64"/>
+      <c r="L78" s="64"/>
+      <c r="M78" s="64"/>
     </row>
     <row r="79" spans="1:13" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A79" s="40" t="s">
@@ -8140,18 +8127,18 @@
       <c r="C79" s="53">
         <v>2</v>
       </c>
-      <c r="D79" s="60" t="s">
+      <c r="D79" s="65" t="s">
         <v>100</v>
       </c>
-      <c r="E79" s="57"/>
-      <c r="F79" s="57"/>
-      <c r="G79" s="57"/>
-      <c r="H79" s="57"/>
-      <c r="I79" s="57"/>
-      <c r="J79" s="57"/>
-      <c r="K79" s="57"/>
-      <c r="L79" s="57"/>
-      <c r="M79" s="57"/>
+      <c r="E79" s="64"/>
+      <c r="F79" s="64"/>
+      <c r="G79" s="64"/>
+      <c r="H79" s="64"/>
+      <c r="I79" s="64"/>
+      <c r="J79" s="64"/>
+      <c r="K79" s="64"/>
+      <c r="L79" s="64"/>
+      <c r="M79" s="64"/>
     </row>
     <row r="80" spans="1:13" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A80" s="40" t="s">
@@ -8163,18 +8150,18 @@
       <c r="C80" s="53">
         <v>3</v>
       </c>
-      <c r="D80" s="60" t="s">
+      <c r="D80" s="65" t="s">
         <v>102</v>
       </c>
-      <c r="E80" s="57"/>
-      <c r="F80" s="57"/>
-      <c r="G80" s="57"/>
-      <c r="H80" s="57"/>
-      <c r="I80" s="57"/>
-      <c r="J80" s="57"/>
-      <c r="K80" s="57"/>
-      <c r="L80" s="57"/>
-      <c r="M80" s="57"/>
+      <c r="E80" s="64"/>
+      <c r="F80" s="64"/>
+      <c r="G80" s="64"/>
+      <c r="H80" s="64"/>
+      <c r="I80" s="64"/>
+      <c r="J80" s="64"/>
+      <c r="K80" s="64"/>
+      <c r="L80" s="64"/>
+      <c r="M80" s="64"/>
     </row>
     <row r="81" spans="1:13" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A81" s="40" t="s">
@@ -8186,18 +8173,18 @@
       <c r="C81" s="53">
         <v>3</v>
       </c>
-      <c r="D81" s="60" t="s">
+      <c r="D81" s="65" t="s">
         <v>104</v>
       </c>
-      <c r="E81" s="57"/>
-      <c r="F81" s="57"/>
-      <c r="G81" s="57"/>
-      <c r="H81" s="57"/>
-      <c r="I81" s="57"/>
-      <c r="J81" s="57"/>
-      <c r="K81" s="57"/>
-      <c r="L81" s="57"/>
-      <c r="M81" s="57"/>
+      <c r="E81" s="64"/>
+      <c r="F81" s="64"/>
+      <c r="G81" s="64"/>
+      <c r="H81" s="64"/>
+      <c r="I81" s="64"/>
+      <c r="J81" s="64"/>
+      <c r="K81" s="64"/>
+      <c r="L81" s="64"/>
+      <c r="M81" s="64"/>
     </row>
     <row r="82" spans="1:13" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A82" s="40" t="s">
@@ -8209,18 +8196,18 @@
       <c r="C82" s="53">
         <v>3</v>
       </c>
-      <c r="D82" s="60" t="s">
+      <c r="D82" s="65" t="s">
         <v>106</v>
       </c>
-      <c r="E82" s="57"/>
-      <c r="F82" s="57"/>
-      <c r="G82" s="57"/>
-      <c r="H82" s="57"/>
-      <c r="I82" s="57"/>
-      <c r="J82" s="57"/>
-      <c r="K82" s="57"/>
-      <c r="L82" s="57"/>
-      <c r="M82" s="57"/>
+      <c r="E82" s="64"/>
+      <c r="F82" s="64"/>
+      <c r="G82" s="64"/>
+      <c r="H82" s="64"/>
+      <c r="I82" s="64"/>
+      <c r="J82" s="64"/>
+      <c r="K82" s="64"/>
+      <c r="L82" s="64"/>
+      <c r="M82" s="64"/>
     </row>
     <row r="83" spans="1:13" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A83" s="40" t="s">
@@ -8232,18 +8219,18 @@
       <c r="C83" s="53">
         <v>6</v>
       </c>
-      <c r="D83" s="60" t="s">
+      <c r="D83" s="65" t="s">
         <v>108</v>
       </c>
-      <c r="E83" s="57"/>
-      <c r="F83" s="57"/>
-      <c r="G83" s="57"/>
-      <c r="H83" s="57"/>
-      <c r="I83" s="57"/>
-      <c r="J83" s="57"/>
-      <c r="K83" s="57"/>
-      <c r="L83" s="57"/>
-      <c r="M83" s="57"/>
+      <c r="E83" s="64"/>
+      <c r="F83" s="64"/>
+      <c r="G83" s="64"/>
+      <c r="H83" s="64"/>
+      <c r="I83" s="64"/>
+      <c r="J83" s="64"/>
+      <c r="K83" s="64"/>
+      <c r="L83" s="64"/>
+      <c r="M83" s="64"/>
     </row>
     <row r="84" spans="1:13" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A84" s="40" t="s">
@@ -8255,18 +8242,18 @@
       <c r="C84" s="53">
         <v>2</v>
       </c>
-      <c r="D84" s="60" t="s">
+      <c r="D84" s="65" t="s">
         <v>110</v>
       </c>
-      <c r="E84" s="57"/>
-      <c r="F84" s="57"/>
-      <c r="G84" s="57"/>
-      <c r="H84" s="57"/>
-      <c r="I84" s="57"/>
-      <c r="J84" s="57"/>
-      <c r="K84" s="57"/>
-      <c r="L84" s="57"/>
-      <c r="M84" s="57"/>
+      <c r="E84" s="64"/>
+      <c r="F84" s="64"/>
+      <c r="G84" s="64"/>
+      <c r="H84" s="64"/>
+      <c r="I84" s="64"/>
+      <c r="J84" s="64"/>
+      <c r="K84" s="64"/>
+      <c r="L84" s="64"/>
+      <c r="M84" s="64"/>
     </row>
     <row r="85" spans="1:13" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A85" s="40" t="s">
@@ -8278,18 +8265,18 @@
       <c r="C85" s="53">
         <v>4</v>
       </c>
-      <c r="D85" s="60" t="s">
+      <c r="D85" s="65" t="s">
         <v>112</v>
       </c>
-      <c r="E85" s="57"/>
-      <c r="F85" s="57"/>
-      <c r="G85" s="57"/>
-      <c r="H85" s="57"/>
-      <c r="I85" s="57"/>
-      <c r="J85" s="57"/>
-      <c r="K85" s="57"/>
-      <c r="L85" s="57"/>
-      <c r="M85" s="57"/>
+      <c r="E85" s="64"/>
+      <c r="F85" s="64"/>
+      <c r="G85" s="64"/>
+      <c r="H85" s="64"/>
+      <c r="I85" s="64"/>
+      <c r="J85" s="64"/>
+      <c r="K85" s="64"/>
+      <c r="L85" s="64"/>
+      <c r="M85" s="64"/>
     </row>
     <row r="86" spans="1:13" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A86" s="40" t="s">
@@ -8301,18 +8288,18 @@
       <c r="C86" s="53">
         <v>4</v>
       </c>
-      <c r="D86" s="60" t="s">
+      <c r="D86" s="65" t="s">
         <v>114</v>
       </c>
-      <c r="E86" s="57"/>
-      <c r="F86" s="57"/>
-      <c r="G86" s="57"/>
-      <c r="H86" s="57"/>
-      <c r="I86" s="57"/>
-      <c r="J86" s="57"/>
-      <c r="K86" s="57"/>
-      <c r="L86" s="57"/>
-      <c r="M86" s="57"/>
+      <c r="E86" s="64"/>
+      <c r="F86" s="64"/>
+      <c r="G86" s="64"/>
+      <c r="H86" s="64"/>
+      <c r="I86" s="64"/>
+      <c r="J86" s="64"/>
+      <c r="K86" s="64"/>
+      <c r="L86" s="64"/>
+      <c r="M86" s="64"/>
     </row>
     <row r="87" spans="1:13" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A87" s="40" t="s">
@@ -8324,18 +8311,18 @@
       <c r="C87" s="53">
         <v>2</v>
       </c>
-      <c r="D87" s="60" t="s">
+      <c r="D87" s="65" t="s">
         <v>116</v>
       </c>
-      <c r="E87" s="57"/>
-      <c r="F87" s="57"/>
-      <c r="G87" s="57"/>
-      <c r="H87" s="57"/>
-      <c r="I87" s="57"/>
-      <c r="J87" s="57"/>
-      <c r="K87" s="57"/>
-      <c r="L87" s="57"/>
-      <c r="M87" s="57"/>
+      <c r="E87" s="64"/>
+      <c r="F87" s="64"/>
+      <c r="G87" s="64"/>
+      <c r="H87" s="64"/>
+      <c r="I87" s="64"/>
+      <c r="J87" s="64"/>
+      <c r="K87" s="64"/>
+      <c r="L87" s="64"/>
+      <c r="M87" s="64"/>
     </row>
     <row r="88" spans="1:13" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A88" s="40" t="s">
@@ -8347,18 +8334,18 @@
       <c r="C88" s="53">
         <v>4</v>
       </c>
-      <c r="D88" s="60" t="s">
+      <c r="D88" s="65" t="s">
         <v>118</v>
       </c>
-      <c r="E88" s="57"/>
-      <c r="F88" s="57"/>
-      <c r="G88" s="57"/>
-      <c r="H88" s="57"/>
-      <c r="I88" s="57"/>
-      <c r="J88" s="57"/>
-      <c r="K88" s="57"/>
-      <c r="L88" s="57"/>
-      <c r="M88" s="57"/>
+      <c r="E88" s="64"/>
+      <c r="F88" s="64"/>
+      <c r="G88" s="64"/>
+      <c r="H88" s="64"/>
+      <c r="I88" s="64"/>
+      <c r="J88" s="64"/>
+      <c r="K88" s="64"/>
+      <c r="L88" s="64"/>
+      <c r="M88" s="64"/>
     </row>
     <row r="89" spans="1:13" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A89" s="40" t="s">
@@ -8370,21 +8357,52 @@
       <c r="C89" s="53">
         <v>4</v>
       </c>
-      <c r="D89" s="60" t="s">
+      <c r="D89" s="65" t="s">
         <v>120</v>
       </c>
-      <c r="E89" s="57"/>
-      <c r="F89" s="57"/>
-      <c r="G89" s="57"/>
-      <c r="H89" s="57"/>
-      <c r="I89" s="57"/>
-      <c r="J89" s="57"/>
-      <c r="K89" s="57"/>
-      <c r="L89" s="57"/>
-      <c r="M89" s="57"/>
+      <c r="E89" s="64"/>
+      <c r="F89" s="64"/>
+      <c r="G89" s="64"/>
+      <c r="H89" s="64"/>
+      <c r="I89" s="64"/>
+      <c r="J89" s="64"/>
+      <c r="K89" s="64"/>
+      <c r="L89" s="64"/>
+      <c r="M89" s="64"/>
     </row>
   </sheetData>
   <mergeCells count="47">
+    <mergeCell ref="D64:M64"/>
+    <mergeCell ref="D82:M82"/>
+    <mergeCell ref="A2:M2"/>
+    <mergeCell ref="A1:M1"/>
+    <mergeCell ref="D65:M65"/>
+    <mergeCell ref="D6:M6"/>
+    <mergeCell ref="D77:M77"/>
+    <mergeCell ref="D57:M57"/>
+    <mergeCell ref="D11:M11"/>
+    <mergeCell ref="D76:M76"/>
+    <mergeCell ref="D61:M61"/>
+    <mergeCell ref="D70:M70"/>
+    <mergeCell ref="D66:M66"/>
+    <mergeCell ref="A56:M56"/>
+    <mergeCell ref="D75:M75"/>
+    <mergeCell ref="D7:M7"/>
+    <mergeCell ref="D89:M89"/>
+    <mergeCell ref="D67:M67"/>
+    <mergeCell ref="D79:M79"/>
+    <mergeCell ref="D85:M85"/>
+    <mergeCell ref="D88:M88"/>
+    <mergeCell ref="D69:M69"/>
+    <mergeCell ref="D81:M81"/>
+    <mergeCell ref="D80:M80"/>
+    <mergeCell ref="D86:M86"/>
+    <mergeCell ref="D87:M87"/>
+    <mergeCell ref="D72:M72"/>
+    <mergeCell ref="D83:M83"/>
+    <mergeCell ref="D73:M73"/>
+    <mergeCell ref="D84:M84"/>
+    <mergeCell ref="D78:M78"/>
     <mergeCell ref="D9:M9"/>
     <mergeCell ref="D74:M74"/>
     <mergeCell ref="A4:M4"/>
@@ -8401,37 +8419,6 @@
     <mergeCell ref="D62:M62"/>
     <mergeCell ref="D12:M12"/>
     <mergeCell ref="D58:M58"/>
-    <mergeCell ref="D89:M89"/>
-    <mergeCell ref="D67:M67"/>
-    <mergeCell ref="D79:M79"/>
-    <mergeCell ref="D85:M85"/>
-    <mergeCell ref="D88:M88"/>
-    <mergeCell ref="D69:M69"/>
-    <mergeCell ref="D81:M81"/>
-    <mergeCell ref="D80:M80"/>
-    <mergeCell ref="D86:M86"/>
-    <mergeCell ref="D87:M87"/>
-    <mergeCell ref="D72:M72"/>
-    <mergeCell ref="D83:M83"/>
-    <mergeCell ref="D73:M73"/>
-    <mergeCell ref="D64:M64"/>
-    <mergeCell ref="D82:M82"/>
-    <mergeCell ref="A2:M2"/>
-    <mergeCell ref="A1:M1"/>
-    <mergeCell ref="D65:M65"/>
-    <mergeCell ref="D84:M84"/>
-    <mergeCell ref="D6:M6"/>
-    <mergeCell ref="D77:M77"/>
-    <mergeCell ref="D57:M57"/>
-    <mergeCell ref="D11:M11"/>
-    <mergeCell ref="D76:M76"/>
-    <mergeCell ref="D61:M61"/>
-    <mergeCell ref="D70:M70"/>
-    <mergeCell ref="D66:M66"/>
-    <mergeCell ref="A56:M56"/>
-    <mergeCell ref="D75:M75"/>
-    <mergeCell ref="D7:M7"/>
-    <mergeCell ref="D78:M78"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -8459,35 +8446,16 @@
     <col min="14" max="14" width="10" style="9" customWidth="1"/>
     <col min="15" max="15" width="14" style="9" customWidth="1"/>
     <col min="16" max="16" width="16" style="9" customWidth="1"/>
-    <col min="17" max="17" width="20" style="70" customWidth="1"/>
+    <col min="17" max="17" width="20" style="61" customWidth="1"/>
     <col min="18" max="18" width="35" style="9" customWidth="1"/>
     <col min="19" max="19" width="16" style="9" customWidth="1"/>
     <col min="20" max="21" width="35" style="9" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:21" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="68" t="s">
+      <c r="A1" s="59" t="s">
         <v>121</v>
       </c>
-      <c r="B1" s="66"/>
-      <c r="C1" s="66"/>
-      <c r="D1" s="66"/>
-      <c r="E1" s="66"/>
-      <c r="F1" s="66"/>
-      <c r="G1" s="66"/>
-      <c r="H1" s="66"/>
-      <c r="I1" s="66"/>
-      <c r="J1" s="66"/>
-      <c r="K1" s="66"/>
-      <c r="L1" s="66"/>
-      <c r="M1" s="66"/>
-      <c r="N1" s="66"/>
-      <c r="O1" s="66"/>
-      <c r="P1" s="66"/>
-      <c r="R1" s="66"/>
-      <c r="S1" s="66"/>
-      <c r="T1" s="66"/>
-      <c r="U1" s="66"/>
     </row>
     <row r="2" spans="1:21" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="33" t="s">
@@ -8538,7 +8506,7 @@
       <c r="P2" s="33" t="s">
         <v>136</v>
       </c>
-      <c r="Q2" s="69" t="s">
+      <c r="Q2" s="60" t="s">
         <v>137</v>
       </c>
       <c r="R2" s="33" t="s">
@@ -8555,52 +8523,14 @@
       </c>
     </row>
     <row r="3" spans="1:21" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="67" t="s">
+      <c r="A3" s="58" t="s">
         <v>142</v>
       </c>
-      <c r="B3" s="66"/>
-      <c r="C3" s="66"/>
-      <c r="D3" s="66"/>
-      <c r="E3" s="66"/>
-      <c r="F3" s="66"/>
-      <c r="G3" s="66"/>
-      <c r="H3" s="66"/>
-      <c r="I3" s="66"/>
-      <c r="J3" s="66"/>
-      <c r="K3" s="66"/>
-      <c r="L3" s="66"/>
-      <c r="M3" s="66"/>
-      <c r="N3" s="66"/>
-      <c r="O3" s="66"/>
-      <c r="P3" s="66"/>
-      <c r="R3" s="66"/>
-      <c r="S3" s="66"/>
-      <c r="T3" s="66"/>
-      <c r="U3" s="66"/>
     </row>
     <row r="4" spans="1:21" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="65" t="s">
+      <c r="A4" s="57" t="s">
         <v>143</v>
       </c>
-      <c r="B4" s="66"/>
-      <c r="C4" s="66"/>
-      <c r="D4" s="66"/>
-      <c r="E4" s="66"/>
-      <c r="F4" s="66"/>
-      <c r="G4" s="66"/>
-      <c r="H4" s="66"/>
-      <c r="I4" s="66"/>
-      <c r="J4" s="66"/>
-      <c r="K4" s="66"/>
-      <c r="L4" s="66"/>
-      <c r="M4" s="66"/>
-      <c r="N4" s="66"/>
-      <c r="O4" s="66"/>
-      <c r="P4" s="66"/>
-      <c r="R4" s="66"/>
-      <c r="S4" s="66"/>
-      <c r="T4" s="66"/>
-      <c r="U4" s="66"/>
     </row>
     <row r="5" spans="1:21" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="34">
@@ -8649,7 +8579,7 @@
       <c r="P5" s="36" t="s">
         <v>7</v>
       </c>
-      <c r="Q5" s="71"/>
+      <c r="Q5" s="62"/>
       <c r="R5" s="35" t="s">
         <v>155</v>
       </c>
@@ -8704,7 +8634,7 @@
       <c r="P6" s="36" t="s">
         <v>7</v>
       </c>
-      <c r="Q6" s="71"/>
+      <c r="Q6" s="62"/>
       <c r="R6" s="35"/>
       <c r="S6" s="34"/>
       <c r="T6" s="35"/>
@@ -8757,7 +8687,7 @@
       <c r="P7" s="36" t="s">
         <v>7</v>
       </c>
-      <c r="Q7" s="71"/>
+      <c r="Q7" s="62"/>
       <c r="R7" s="35"/>
       <c r="S7" s="34"/>
       <c r="T7" s="35"/>
@@ -8810,35 +8740,16 @@
       <c r="P8" s="36" t="s">
         <v>7</v>
       </c>
-      <c r="Q8" s="71"/>
+      <c r="Q8" s="62"/>
       <c r="R8" s="35"/>
       <c r="S8" s="34"/>
       <c r="T8" s="35"/>
       <c r="U8" s="35"/>
     </row>
     <row r="9" spans="1:21" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="65" t="s">
+      <c r="A9" s="57" t="s">
         <v>180</v>
       </c>
-      <c r="B9" s="66"/>
-      <c r="C9" s="66"/>
-      <c r="D9" s="66"/>
-      <c r="E9" s="66"/>
-      <c r="F9" s="66"/>
-      <c r="G9" s="66"/>
-      <c r="H9" s="66"/>
-      <c r="I9" s="66"/>
-      <c r="J9" s="66"/>
-      <c r="K9" s="66"/>
-      <c r="L9" s="66"/>
-      <c r="M9" s="66"/>
-      <c r="N9" s="66"/>
-      <c r="O9" s="66"/>
-      <c r="P9" s="66"/>
-      <c r="R9" s="66"/>
-      <c r="S9" s="66"/>
-      <c r="T9" s="66"/>
-      <c r="U9" s="66"/>
     </row>
     <row r="10" spans="1:21" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="34">
@@ -8887,7 +8798,7 @@
       <c r="P10" s="36" t="s">
         <v>7</v>
       </c>
-      <c r="Q10" s="71"/>
+      <c r="Q10" s="62"/>
       <c r="R10" s="35"/>
       <c r="S10" s="34"/>
       <c r="T10" s="35"/>
@@ -8940,7 +8851,7 @@
       <c r="P11" s="36" t="s">
         <v>7</v>
       </c>
-      <c r="Q11" s="71"/>
+      <c r="Q11" s="62"/>
       <c r="R11" s="35"/>
       <c r="S11" s="34" t="s">
         <v>198</v>
@@ -8999,7 +8910,7 @@
       <c r="P12" s="36" t="s">
         <v>7</v>
       </c>
-      <c r="Q12" s="71"/>
+      <c r="Q12" s="62"/>
       <c r="R12" s="35"/>
       <c r="S12" s="34"/>
       <c r="T12" s="35"/>
@@ -9052,35 +8963,16 @@
       <c r="P13" s="36" t="s">
         <v>7</v>
       </c>
-      <c r="Q13" s="71"/>
+      <c r="Q13" s="62"/>
       <c r="R13" s="35"/>
       <c r="S13" s="34"/>
       <c r="T13" s="35"/>
       <c r="U13" s="35"/>
     </row>
     <row r="14" spans="1:21" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="65" t="s">
+      <c r="A14" s="57" t="s">
         <v>216</v>
       </c>
-      <c r="B14" s="66"/>
-      <c r="C14" s="66"/>
-      <c r="D14" s="66"/>
-      <c r="E14" s="66"/>
-      <c r="F14" s="66"/>
-      <c r="G14" s="66"/>
-      <c r="H14" s="66"/>
-      <c r="I14" s="66"/>
-      <c r="J14" s="66"/>
-      <c r="K14" s="66"/>
-      <c r="L14" s="66"/>
-      <c r="M14" s="66"/>
-      <c r="N14" s="66"/>
-      <c r="O14" s="66"/>
-      <c r="P14" s="66"/>
-      <c r="R14" s="66"/>
-      <c r="S14" s="66"/>
-      <c r="T14" s="66"/>
-      <c r="U14" s="66"/>
     </row>
     <row r="15" spans="1:21" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="34">
@@ -9129,7 +9021,7 @@
       <c r="P15" s="36" t="s">
         <v>7</v>
       </c>
-      <c r="Q15" s="71" t="s">
+      <c r="Q15" s="62" t="s">
         <v>225</v>
       </c>
       <c r="R15" s="35"/>
@@ -9190,7 +9082,7 @@
       <c r="P16" s="36" t="s">
         <v>7</v>
       </c>
-      <c r="Q16" s="71"/>
+      <c r="Q16" s="62"/>
       <c r="R16" s="35"/>
       <c r="S16" s="34"/>
       <c r="T16" s="35"/>
@@ -9243,7 +9135,7 @@
       <c r="P17" s="36" t="s">
         <v>7</v>
       </c>
-      <c r="Q17" s="71"/>
+      <c r="Q17" s="62"/>
       <c r="R17" s="35"/>
       <c r="S17" s="34"/>
       <c r="T17" s="35"/>
@@ -9296,7 +9188,7 @@
       <c r="P18" s="36" t="s">
         <v>7</v>
       </c>
-      <c r="Q18" s="71"/>
+      <c r="Q18" s="62"/>
       <c r="R18" s="35"/>
       <c r="S18" s="34"/>
       <c r="T18" s="35"/>
@@ -9349,7 +9241,7 @@
       <c r="P19" s="36" t="s">
         <v>17</v>
       </c>
-      <c r="Q19" s="71"/>
+      <c r="Q19" s="62"/>
       <c r="R19" s="35"/>
       <c r="S19" s="34"/>
       <c r="T19" s="35"/>
@@ -9402,59 +9294,21 @@
       <c r="P20" s="36" t="s">
         <v>17</v>
       </c>
-      <c r="Q20" s="71"/>
+      <c r="Q20" s="62"/>
       <c r="R20" s="35"/>
       <c r="S20" s="34"/>
       <c r="T20" s="35"/>
       <c r="U20" s="35"/>
     </row>
     <row r="21" spans="1:21" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="67" t="s">
+      <c r="A21" s="58" t="s">
         <v>266</v>
       </c>
-      <c r="B21" s="66"/>
-      <c r="C21" s="66"/>
-      <c r="D21" s="66"/>
-      <c r="E21" s="66"/>
-      <c r="F21" s="66"/>
-      <c r="G21" s="66"/>
-      <c r="H21" s="66"/>
-      <c r="I21" s="66"/>
-      <c r="J21" s="66"/>
-      <c r="K21" s="66"/>
-      <c r="L21" s="66"/>
-      <c r="M21" s="66"/>
-      <c r="N21" s="66"/>
-      <c r="O21" s="66"/>
-      <c r="P21" s="66"/>
-      <c r="R21" s="66"/>
-      <c r="S21" s="66"/>
-      <c r="T21" s="66"/>
-      <c r="U21" s="66"/>
     </row>
     <row r="22" spans="1:21" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="65" t="s">
+      <c r="A22" s="57" t="s">
         <v>267</v>
       </c>
-      <c r="B22" s="66"/>
-      <c r="C22" s="66"/>
-      <c r="D22" s="66"/>
-      <c r="E22" s="66"/>
-      <c r="F22" s="66"/>
-      <c r="G22" s="66"/>
-      <c r="H22" s="66"/>
-      <c r="I22" s="66"/>
-      <c r="J22" s="66"/>
-      <c r="K22" s="66"/>
-      <c r="L22" s="66"/>
-      <c r="M22" s="66"/>
-      <c r="N22" s="66"/>
-      <c r="O22" s="66"/>
-      <c r="P22" s="66"/>
-      <c r="R22" s="66"/>
-      <c r="S22" s="66"/>
-      <c r="T22" s="66"/>
-      <c r="U22" s="66"/>
     </row>
     <row r="23" spans="1:21" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="34">
@@ -9469,7 +9323,7 @@
       <c r="D23" s="35" t="s">
         <v>269</v>
       </c>
-      <c r="E23" s="34" t="s">
+      <c r="E23" s="72" t="s">
         <v>270</v>
       </c>
       <c r="F23" s="34" t="s">
@@ -9505,7 +9359,7 @@
       <c r="P23" s="36" t="s">
         <v>7</v>
       </c>
-      <c r="Q23" s="71"/>
+      <c r="Q23" s="62"/>
       <c r="R23" s="35" t="s">
         <v>278</v>
       </c>
@@ -9532,7 +9386,7 @@
       <c r="D24" s="35" t="s">
         <v>269</v>
       </c>
-      <c r="E24" s="34" t="s">
+      <c r="E24" s="72" t="s">
         <v>270</v>
       </c>
       <c r="F24" s="34" t="s">
@@ -9568,7 +9422,7 @@
       <c r="P24" s="36" t="s">
         <v>7</v>
       </c>
-      <c r="Q24" s="71"/>
+      <c r="Q24" s="62"/>
       <c r="R24" s="35" t="s">
         <v>278</v>
       </c>
@@ -9595,7 +9449,7 @@
       <c r="D25" s="35" t="s">
         <v>269</v>
       </c>
-      <c r="E25" s="34" t="s">
+      <c r="E25" s="72" t="s">
         <v>270</v>
       </c>
       <c r="F25" s="34" t="s">
@@ -9631,7 +9485,7 @@
       <c r="P25" s="36" t="s">
         <v>7</v>
       </c>
-      <c r="Q25" s="71"/>
+      <c r="Q25" s="62"/>
       <c r="R25" s="35" t="s">
         <v>278</v>
       </c>
@@ -9652,7 +9506,7 @@
       <c r="D26" s="35" t="s">
         <v>269</v>
       </c>
-      <c r="E26" s="34" t="s">
+      <c r="E26" s="72" t="s">
         <v>270</v>
       </c>
       <c r="F26" s="34" t="s">
@@ -9688,7 +9542,7 @@
       <c r="P26" s="36" t="s">
         <v>7</v>
       </c>
-      <c r="Q26" s="71"/>
+      <c r="Q26" s="62"/>
       <c r="R26" s="35" t="s">
         <v>278</v>
       </c>
@@ -9709,7 +9563,7 @@
       <c r="D27" s="35" t="s">
         <v>269</v>
       </c>
-      <c r="E27" s="34" t="s">
+      <c r="E27" s="72" t="s">
         <v>270</v>
       </c>
       <c r="F27" s="34" t="s">
@@ -9745,7 +9599,7 @@
       <c r="P27" s="36" t="s">
         <v>7</v>
       </c>
-      <c r="Q27" s="71"/>
+      <c r="Q27" s="62"/>
       <c r="R27" s="35" t="s">
         <v>278</v>
       </c>
@@ -9766,7 +9620,7 @@
       <c r="D28" s="35" t="s">
         <v>269</v>
       </c>
-      <c r="E28" s="34" t="s">
+      <c r="E28" s="72" t="s">
         <v>270</v>
       </c>
       <c r="F28" s="34" t="s">
@@ -9802,7 +9656,7 @@
       <c r="P28" s="36" t="s">
         <v>7</v>
       </c>
-      <c r="Q28" s="71"/>
+      <c r="Q28" s="62"/>
       <c r="R28" s="35" t="s">
         <v>278</v>
       </c>
@@ -9823,7 +9677,7 @@
       <c r="D29" s="35" t="s">
         <v>269</v>
       </c>
-      <c r="E29" s="34" t="s">
+      <c r="E29" s="72" t="s">
         <v>270</v>
       </c>
       <c r="F29" s="34" t="s">
@@ -9859,7 +9713,7 @@
       <c r="P29" s="36" t="s">
         <v>7</v>
       </c>
-      <c r="Q29" s="71"/>
+      <c r="Q29" s="62"/>
       <c r="R29" s="35" t="s">
         <v>278</v>
       </c>
@@ -9886,7 +9740,7 @@
       <c r="D30" s="35" t="s">
         <v>269</v>
       </c>
-      <c r="E30" s="34" t="s">
+      <c r="E30" s="72" t="s">
         <v>270</v>
       </c>
       <c r="F30" s="34" t="s">
@@ -9922,7 +9776,7 @@
       <c r="P30" s="36" t="s">
         <v>7</v>
       </c>
-      <c r="Q30" s="71"/>
+      <c r="Q30" s="62"/>
       <c r="R30" s="35" t="s">
         <v>278</v>
       </c>
@@ -9949,7 +9803,7 @@
       <c r="D31" s="35" t="s">
         <v>269</v>
       </c>
-      <c r="E31" s="34" t="s">
+      <c r="E31" s="72" t="s">
         <v>270</v>
       </c>
       <c r="F31" s="34" t="s">
@@ -9985,7 +9839,7 @@
       <c r="P31" s="36" t="s">
         <v>7</v>
       </c>
-      <c r="Q31" s="71"/>
+      <c r="Q31" s="62"/>
       <c r="R31" s="35" t="s">
         <v>278</v>
       </c>
@@ -10006,7 +9860,7 @@
       <c r="D32" s="35" t="s">
         <v>269</v>
       </c>
-      <c r="E32" s="34" t="s">
+      <c r="E32" s="72" t="s">
         <v>270</v>
       </c>
       <c r="F32" s="34" t="s">
@@ -10042,7 +9896,7 @@
       <c r="P32" s="36" t="s">
         <v>7</v>
       </c>
-      <c r="Q32" s="71"/>
+      <c r="Q32" s="62"/>
       <c r="R32" s="35" t="s">
         <v>278</v>
       </c>
@@ -10063,7 +9917,7 @@
       <c r="D33" s="35" t="s">
         <v>269</v>
       </c>
-      <c r="E33" s="34" t="s">
+      <c r="E33" s="72" t="s">
         <v>270</v>
       </c>
       <c r="F33" s="34" t="s">
@@ -10099,7 +9953,7 @@
       <c r="P33" s="36" t="s">
         <v>7</v>
       </c>
-      <c r="Q33" s="71"/>
+      <c r="Q33" s="62"/>
       <c r="R33" s="35" t="s">
         <v>278</v>
       </c>
@@ -10120,7 +9974,7 @@
       <c r="D34" s="35" t="s">
         <v>269</v>
       </c>
-      <c r="E34" s="34" t="s">
+      <c r="E34" s="72" t="s">
         <v>270</v>
       </c>
       <c r="F34" s="34" t="s">
@@ -10156,7 +10010,7 @@
       <c r="P34" s="36" t="s">
         <v>7</v>
       </c>
-      <c r="Q34" s="71"/>
+      <c r="Q34" s="62"/>
       <c r="R34" s="35" t="s">
         <v>278</v>
       </c>
@@ -10177,7 +10031,7 @@
       <c r="D35" s="35" t="s">
         <v>269</v>
       </c>
-      <c r="E35" s="34" t="s">
+      <c r="E35" s="72" t="s">
         <v>270</v>
       </c>
       <c r="F35" s="34" t="s">
@@ -10213,7 +10067,7 @@
       <c r="P35" s="36" t="s">
         <v>7</v>
       </c>
-      <c r="Q35" s="71"/>
+      <c r="Q35" s="62"/>
       <c r="R35" s="35" t="s">
         <v>278</v>
       </c>
@@ -10234,7 +10088,7 @@
       <c r="D36" s="35" t="s">
         <v>269</v>
       </c>
-      <c r="E36" s="34" t="s">
+      <c r="E36" s="72" t="s">
         <v>270</v>
       </c>
       <c r="F36" s="34" t="s">
@@ -10270,7 +10124,7 @@
       <c r="P36" s="36" t="s">
         <v>7</v>
       </c>
-      <c r="Q36" s="71"/>
+      <c r="Q36" s="62"/>
       <c r="R36" s="35" t="s">
         <v>395</v>
       </c>
@@ -10279,28 +10133,9 @@
       <c r="U36" s="35"/>
     </row>
     <row r="37" spans="1:21" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="65" t="s">
+      <c r="A37" s="57" t="s">
         <v>396</v>
       </c>
-      <c r="B37" s="66"/>
-      <c r="C37" s="66"/>
-      <c r="D37" s="66"/>
-      <c r="E37" s="66"/>
-      <c r="F37" s="66"/>
-      <c r="G37" s="66"/>
-      <c r="H37" s="66"/>
-      <c r="I37" s="66"/>
-      <c r="J37" s="66"/>
-      <c r="K37" s="66"/>
-      <c r="L37" s="66"/>
-      <c r="M37" s="66"/>
-      <c r="N37" s="66"/>
-      <c r="O37" s="66"/>
-      <c r="P37" s="66"/>
-      <c r="R37" s="66"/>
-      <c r="S37" s="66"/>
-      <c r="T37" s="66"/>
-      <c r="U37" s="66"/>
     </row>
     <row r="38" spans="1:21" ht="24" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A38" s="34">
@@ -10315,7 +10150,7 @@
       <c r="D38" s="35" t="s">
         <v>398</v>
       </c>
-      <c r="E38" s="34" t="s">
+      <c r="E38" s="71" t="s">
         <v>399</v>
       </c>
       <c r="F38" s="34" t="s">
@@ -10351,7 +10186,7 @@
       <c r="P38" s="36" t="s">
         <v>9</v>
       </c>
-      <c r="Q38" s="71"/>
+      <c r="Q38" s="62"/>
       <c r="R38" s="35" t="s">
         <v>278</v>
       </c>
@@ -10378,7 +10213,7 @@
       <c r="D39" s="35" t="s">
         <v>398</v>
       </c>
-      <c r="E39" s="34" t="s">
+      <c r="E39" s="73" t="s">
         <v>410</v>
       </c>
       <c r="F39" s="34" t="s">
@@ -10412,10 +10247,10 @@
         <v>417</v>
       </c>
       <c r="P39" s="36" t="s">
-        <v>11</v>
-      </c>
-      <c r="Q39" s="72" t="s">
-        <v>1833</v>
+        <v>17</v>
+      </c>
+      <c r="Q39" s="78" t="s">
+        <v>1837</v>
       </c>
       <c r="R39" s="35" t="s">
         <v>278</v>
@@ -10443,7 +10278,7 @@
       <c r="D40" s="35" t="s">
         <v>398</v>
       </c>
-      <c r="E40" s="34" t="s">
+      <c r="E40" s="73" t="s">
         <v>410</v>
       </c>
       <c r="F40" s="34" t="s">
@@ -10479,8 +10314,8 @@
       <c r="P40" s="36" t="s">
         <v>17</v>
       </c>
-      <c r="Q40" s="72" t="s">
-        <v>1834</v>
+      <c r="Q40" s="79">
+        <v>46032</v>
       </c>
       <c r="R40" s="35" t="s">
         <v>278</v>
@@ -10502,7 +10337,7 @@
       <c r="D41" s="35" t="s">
         <v>398</v>
       </c>
-      <c r="E41" s="34" t="s">
+      <c r="E41" s="73" t="s">
         <v>410</v>
       </c>
       <c r="F41" s="34" t="s">
@@ -10538,8 +10373,8 @@
       <c r="P41" s="36" t="s">
         <v>17</v>
       </c>
-      <c r="Q41" s="72" t="s">
-        <v>1835</v>
+      <c r="Q41" s="79">
+        <v>46063</v>
       </c>
       <c r="R41" s="35" t="s">
         <v>278</v>
@@ -10561,7 +10396,7 @@
       <c r="D42" s="35" t="s">
         <v>398</v>
       </c>
-      <c r="E42" s="34" t="s">
+      <c r="E42" s="73" t="s">
         <v>410</v>
       </c>
       <c r="F42" s="34" t="s">
@@ -10597,8 +10432,8 @@
       <c r="P42" s="36" t="s">
         <v>17</v>
       </c>
-      <c r="Q42" s="73">
-        <v>46032</v>
+      <c r="Q42" s="79">
+        <v>46063</v>
       </c>
       <c r="R42" s="35" t="s">
         <v>278</v>
@@ -10626,7 +10461,7 @@
       <c r="D43" s="35" t="s">
         <v>398</v>
       </c>
-      <c r="E43" s="34" t="s">
+      <c r="E43" s="73" t="s">
         <v>410</v>
       </c>
       <c r="F43" s="34" t="s">
@@ -10662,8 +10497,8 @@
       <c r="P43" s="36" t="s">
         <v>17</v>
       </c>
-      <c r="Q43" s="73">
-        <v>46063</v>
+      <c r="Q43" s="79">
+        <v>46091</v>
       </c>
       <c r="R43" s="35" t="s">
         <v>278</v>
@@ -10685,7 +10520,7 @@
       <c r="D44" s="35" t="s">
         <v>398</v>
       </c>
-      <c r="E44" s="34" t="s">
+      <c r="E44" s="73" t="s">
         <v>410</v>
       </c>
       <c r="F44" s="34" t="s">
@@ -10721,7 +10556,7 @@
       <c r="P44" s="36" t="s">
         <v>17</v>
       </c>
-      <c r="Q44" s="73">
+      <c r="Q44" s="79">
         <v>46091</v>
       </c>
       <c r="R44" s="35" t="s">
@@ -10744,7 +10579,7 @@
       <c r="D45" s="35" t="s">
         <v>398</v>
       </c>
-      <c r="E45" s="34" t="s">
+      <c r="E45" s="73" t="s">
         <v>410</v>
       </c>
       <c r="F45" s="34" t="s">
@@ -10780,7 +10615,7 @@
       <c r="P45" s="36" t="s">
         <v>17</v>
       </c>
-      <c r="Q45" s="73">
+      <c r="Q45" s="79">
         <v>46122</v>
       </c>
       <c r="R45" s="35" t="s">
@@ -10803,7 +10638,7 @@
       <c r="D46" s="35" t="s">
         <v>398</v>
       </c>
-      <c r="E46" s="34" t="s">
+      <c r="E46" s="73" t="s">
         <v>410</v>
       </c>
       <c r="F46" s="34" t="s">
@@ -10839,8 +10674,8 @@
       <c r="P46" s="36" t="s">
         <v>17</v>
       </c>
-      <c r="Q46" s="73">
-        <v>46152</v>
+      <c r="Q46" s="79">
+        <v>46122</v>
       </c>
       <c r="R46" s="35" t="s">
         <v>278</v>
@@ -10862,7 +10697,7 @@
       <c r="D47" s="35" t="s">
         <v>398</v>
       </c>
-      <c r="E47" s="34" t="s">
+      <c r="E47" s="73" t="s">
         <v>410</v>
       </c>
       <c r="F47" s="34" t="s">
@@ -10898,8 +10733,8 @@
       <c r="P47" s="36" t="s">
         <v>17</v>
       </c>
-      <c r="Q47" s="73">
-        <v>46183</v>
+      <c r="Q47" s="79">
+        <v>46152</v>
       </c>
       <c r="R47" s="35" t="s">
         <v>278</v>
@@ -10909,28 +10744,10 @@
       <c r="U47" s="35"/>
     </row>
     <row r="48" spans="1:21" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A48" s="65" t="s">
+      <c r="A48" s="57" t="s">
         <v>485</v>
       </c>
-      <c r="B48" s="66"/>
-      <c r="C48" s="66"/>
-      <c r="D48" s="66"/>
-      <c r="E48" s="66"/>
-      <c r="F48" s="66"/>
-      <c r="G48" s="66"/>
-      <c r="H48" s="66"/>
-      <c r="I48" s="66"/>
-      <c r="J48" s="66"/>
-      <c r="K48" s="66"/>
-      <c r="L48" s="66"/>
-      <c r="M48" s="66"/>
-      <c r="N48" s="66"/>
-      <c r="O48" s="66"/>
-      <c r="P48" s="66"/>
-      <c r="R48" s="66"/>
-      <c r="S48" s="66"/>
-      <c r="T48" s="66"/>
-      <c r="U48" s="66"/>
+      <c r="Q48" s="80"/>
     </row>
     <row r="49" spans="1:21" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A49" s="34">
@@ -10945,7 +10762,7 @@
       <c r="D49" s="35" t="s">
         <v>487</v>
       </c>
-      <c r="E49" s="34" t="s">
+      <c r="E49" s="74" t="s">
         <v>488</v>
       </c>
       <c r="F49" s="34" t="s">
@@ -10979,10 +10796,10 @@
         <v>495</v>
       </c>
       <c r="P49" s="36" t="s">
-        <v>17</v>
-      </c>
-      <c r="Q49" s="74">
-        <v>46213</v>
+        <v>11</v>
+      </c>
+      <c r="Q49" s="80" t="s">
+        <v>1834</v>
       </c>
       <c r="R49" s="35" t="s">
         <v>278</v>
@@ -10992,28 +10809,9 @@
       <c r="U49" s="35"/>
     </row>
     <row r="50" spans="1:21" ht="24" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A50" s="65" t="s">
+      <c r="A50" s="57" t="s">
         <v>496</v>
       </c>
-      <c r="B50" s="66"/>
-      <c r="C50" s="66"/>
-      <c r="D50" s="66"/>
-      <c r="E50" s="66"/>
-      <c r="F50" s="66"/>
-      <c r="G50" s="66"/>
-      <c r="H50" s="66"/>
-      <c r="I50" s="66"/>
-      <c r="J50" s="66"/>
-      <c r="K50" s="66"/>
-      <c r="L50" s="66"/>
-      <c r="M50" s="66"/>
-      <c r="N50" s="66"/>
-      <c r="O50" s="66"/>
-      <c r="P50" s="66"/>
-      <c r="R50" s="66"/>
-      <c r="S50" s="66"/>
-      <c r="T50" s="66"/>
-      <c r="U50" s="66"/>
     </row>
     <row r="51" spans="1:21" ht="24" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A51" s="34">
@@ -11028,7 +10826,7 @@
       <c r="D51" s="35" t="s">
         <v>498</v>
       </c>
-      <c r="E51" s="34" t="s">
+      <c r="E51" s="75" t="s">
         <v>499</v>
       </c>
       <c r="F51" s="34" t="s">
@@ -11062,10 +10860,10 @@
         <v>371</v>
       </c>
       <c r="P51" s="36" t="s">
-        <v>17</v>
-      </c>
-      <c r="Q51" s="73">
-        <v>46244</v>
+        <v>11</v>
+      </c>
+      <c r="Q51" s="79" t="s">
+        <v>1833</v>
       </c>
       <c r="R51" s="35" t="s">
         <v>278</v>
@@ -11093,7 +10891,7 @@
       <c r="D52" s="35" t="s">
         <v>498</v>
       </c>
-      <c r="E52" s="34" t="s">
+      <c r="E52" s="75" t="s">
         <v>499</v>
       </c>
       <c r="F52" s="34" t="s">
@@ -11129,8 +10927,8 @@
       <c r="P52" s="36" t="s">
         <v>17</v>
       </c>
-      <c r="Q52" s="73">
-        <v>46275</v>
+      <c r="Q52" s="79" t="s">
+        <v>1835</v>
       </c>
       <c r="R52" s="35" t="s">
         <v>278</v>
@@ -11158,7 +10956,7 @@
       <c r="D53" s="35" t="s">
         <v>498</v>
       </c>
-      <c r="E53" s="34" t="s">
+      <c r="E53" s="75" t="s">
         <v>499</v>
       </c>
       <c r="F53" s="34" t="s">
@@ -11194,8 +10992,8 @@
       <c r="P53" s="36" t="s">
         <v>17</v>
       </c>
-      <c r="Q53" s="73">
-        <v>46305</v>
+      <c r="Q53" s="79" t="s">
+        <v>1835</v>
       </c>
       <c r="R53" s="35" t="s">
         <v>278</v>
@@ -11217,7 +11015,7 @@
       <c r="D54" s="35" t="s">
         <v>498</v>
       </c>
-      <c r="E54" s="34" t="s">
+      <c r="E54" s="71" t="s">
         <v>399</v>
       </c>
       <c r="F54" s="34" t="s">
@@ -11253,7 +11051,7 @@
       <c r="P54" s="36" t="s">
         <v>9</v>
       </c>
-      <c r="Q54" s="71"/>
+      <c r="Q54" s="81"/>
       <c r="R54" s="35" t="s">
         <v>278</v>
       </c>
@@ -11274,7 +11072,7 @@
       <c r="D55" s="35" t="s">
         <v>498</v>
       </c>
-      <c r="E55" s="34" t="s">
+      <c r="E55" s="71" t="s">
         <v>399</v>
       </c>
       <c r="F55" s="34" t="s">
@@ -11310,7 +11108,7 @@
       <c r="P55" s="36" t="s">
         <v>9</v>
       </c>
-      <c r="Q55" s="71"/>
+      <c r="Q55" s="81"/>
       <c r="R55" s="35" t="s">
         <v>278</v>
       </c>
@@ -11337,7 +11135,7 @@
       <c r="D56" s="35" t="s">
         <v>498</v>
       </c>
-      <c r="E56" s="34" t="s">
+      <c r="E56" s="71" t="s">
         <v>399</v>
       </c>
       <c r="F56" s="34" t="s">
@@ -11373,7 +11171,7 @@
       <c r="P56" s="36" t="s">
         <v>9</v>
       </c>
-      <c r="Q56" s="71"/>
+      <c r="Q56" s="81"/>
       <c r="R56" s="35" t="s">
         <v>278</v>
       </c>
@@ -11394,7 +11192,7 @@
       <c r="D57" s="35" t="s">
         <v>498</v>
       </c>
-      <c r="E57" s="34" t="s">
+      <c r="E57" s="71" t="s">
         <v>399</v>
       </c>
       <c r="F57" s="34" t="s">
@@ -11430,7 +11228,7 @@
       <c r="P57" s="36" t="s">
         <v>9</v>
       </c>
-      <c r="Q57" s="71"/>
+      <c r="Q57" s="81"/>
       <c r="R57" s="35" t="s">
         <v>278</v>
       </c>
@@ -11439,28 +11237,10 @@
       <c r="U57" s="35"/>
     </row>
     <row r="58" spans="1:21" ht="24" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A58" s="65" t="s">
+      <c r="A58" s="57" t="s">
         <v>560</v>
       </c>
-      <c r="B58" s="66"/>
-      <c r="C58" s="66"/>
-      <c r="D58" s="66"/>
-      <c r="E58" s="66"/>
-      <c r="F58" s="66"/>
-      <c r="G58" s="66"/>
-      <c r="H58" s="66"/>
-      <c r="I58" s="66"/>
-      <c r="J58" s="66"/>
-      <c r="K58" s="66"/>
-      <c r="L58" s="66"/>
-      <c r="M58" s="66"/>
-      <c r="N58" s="66"/>
-      <c r="O58" s="66"/>
-      <c r="P58" s="66"/>
-      <c r="R58" s="66"/>
-      <c r="S58" s="66"/>
-      <c r="T58" s="66"/>
-      <c r="U58" s="66"/>
+      <c r="Q58" s="80"/>
     </row>
     <row r="59" spans="1:21" ht="24" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A59" s="34">
@@ -11475,7 +11255,7 @@
       <c r="D59" s="35" t="s">
         <v>562</v>
       </c>
-      <c r="E59" s="34" t="s">
+      <c r="E59" s="75" t="s">
         <v>499</v>
       </c>
       <c r="F59" s="34" t="s">
@@ -11511,8 +11291,8 @@
       <c r="P59" s="36" t="s">
         <v>17</v>
       </c>
-      <c r="Q59" s="73">
-        <v>46336</v>
+      <c r="Q59" s="79" t="s">
+        <v>1836</v>
       </c>
       <c r="R59" s="35" t="s">
         <v>278</v>
@@ -11534,7 +11314,7 @@
       <c r="D60" s="35" t="s">
         <v>562</v>
       </c>
-      <c r="E60" s="34" t="s">
+      <c r="E60" s="76" t="s">
         <v>570</v>
       </c>
       <c r="F60" s="34" t="s">
@@ -11570,9 +11350,7 @@
       <c r="P60" s="36" t="s">
         <v>17</v>
       </c>
-      <c r="Q60" s="73">
-        <v>46366</v>
-      </c>
+      <c r="Q60" s="79"/>
       <c r="R60" s="35" t="s">
         <v>278</v>
       </c>
@@ -11599,7 +11377,7 @@
       <c r="D61" s="35" t="s">
         <v>562</v>
       </c>
-      <c r="E61" s="34" t="s">
+      <c r="E61" s="76" t="s">
         <v>570</v>
       </c>
       <c r="F61" s="34" t="s">
@@ -11635,9 +11413,7 @@
       <c r="P61" s="36" t="s">
         <v>17</v>
       </c>
-      <c r="Q61" s="72" t="s">
-        <v>1836</v>
-      </c>
+      <c r="Q61" s="78"/>
       <c r="R61" s="35" t="s">
         <v>278</v>
       </c>
@@ -11658,7 +11434,7 @@
       <c r="D62" s="35" t="s">
         <v>562</v>
       </c>
-      <c r="E62" s="34" t="s">
+      <c r="E62" s="76" t="s">
         <v>570</v>
       </c>
       <c r="F62" s="34" t="s">
@@ -11694,9 +11470,7 @@
       <c r="P62" s="36" t="s">
         <v>17</v>
       </c>
-      <c r="Q62" s="72" t="s">
-        <v>1837</v>
-      </c>
+      <c r="Q62" s="78"/>
       <c r="R62" s="35" t="s">
         <v>278</v>
       </c>
@@ -11717,7 +11491,7 @@
       <c r="D63" s="35" t="s">
         <v>562</v>
       </c>
-      <c r="E63" s="34" t="s">
+      <c r="E63" s="76" t="s">
         <v>570</v>
       </c>
       <c r="F63" s="34" t="s">
@@ -11753,9 +11527,7 @@
       <c r="P63" s="36" t="s">
         <v>17</v>
       </c>
-      <c r="Q63" s="72" t="s">
-        <v>1838</v>
-      </c>
+      <c r="Q63" s="78"/>
       <c r="R63" s="35" t="s">
         <v>278</v>
       </c>
@@ -11776,7 +11548,7 @@
       <c r="D64" s="35" t="s">
         <v>562</v>
       </c>
-      <c r="E64" s="34" t="s">
+      <c r="E64" s="76" t="s">
         <v>570</v>
       </c>
       <c r="F64" s="34" t="s">
@@ -11812,9 +11584,7 @@
       <c r="P64" s="36" t="s">
         <v>17</v>
       </c>
-      <c r="Q64" s="72" t="s">
-        <v>1839</v>
-      </c>
+      <c r="Q64" s="78"/>
       <c r="R64" s="35" t="s">
         <v>278</v>
       </c>
@@ -11841,7 +11611,7 @@
       <c r="D65" s="35" t="s">
         <v>562</v>
       </c>
-      <c r="E65" s="34" t="s">
+      <c r="E65" s="76" t="s">
         <v>570</v>
       </c>
       <c r="F65" s="34" t="s">
@@ -11877,9 +11647,7 @@
       <c r="P65" s="36" t="s">
         <v>17</v>
       </c>
-      <c r="Q65" s="72" t="s">
-        <v>1840</v>
-      </c>
+      <c r="Q65" s="78"/>
       <c r="R65" s="35" t="s">
         <v>278</v>
       </c>
@@ -11900,7 +11668,7 @@
       <c r="D66" s="35" t="s">
         <v>562</v>
       </c>
-      <c r="E66" s="34" t="s">
+      <c r="E66" s="76" t="s">
         <v>570</v>
       </c>
       <c r="F66" s="34" t="s">
@@ -11936,9 +11704,7 @@
       <c r="P66" s="36" t="s">
         <v>17</v>
       </c>
-      <c r="Q66" s="72" t="s">
-        <v>1841</v>
-      </c>
+      <c r="Q66" s="78"/>
       <c r="R66" s="35" t="s">
         <v>278</v>
       </c>
@@ -11959,7 +11725,7 @@
       <c r="D67" s="35" t="s">
         <v>562</v>
       </c>
-      <c r="E67" s="34" t="s">
+      <c r="E67" s="76" t="s">
         <v>570</v>
       </c>
       <c r="F67" s="34" t="s">
@@ -11995,9 +11761,7 @@
       <c r="P67" s="36" t="s">
         <v>17</v>
       </c>
-      <c r="Q67" s="72" t="s">
-        <v>1842</v>
-      </c>
+      <c r="Q67" s="78"/>
       <c r="R67" s="35" t="s">
         <v>278</v>
       </c>
@@ -12018,7 +11782,7 @@
       <c r="D68" s="35" t="s">
         <v>562</v>
       </c>
-      <c r="E68" s="34" t="s">
+      <c r="E68" s="76" t="s">
         <v>570</v>
       </c>
       <c r="F68" s="34" t="s">
@@ -12054,9 +11818,7 @@
       <c r="P68" s="36" t="s">
         <v>17</v>
       </c>
-      <c r="Q68" s="72" t="s">
-        <v>1843</v>
-      </c>
+      <c r="Q68" s="78"/>
       <c r="R68" s="35" t="s">
         <v>278</v>
       </c>
@@ -12077,7 +11839,7 @@
       <c r="D69" s="35" t="s">
         <v>562</v>
       </c>
-      <c r="E69" s="34" t="s">
+      <c r="E69" s="76" t="s">
         <v>570</v>
       </c>
       <c r="F69" s="34" t="s">
@@ -12113,9 +11875,7 @@
       <c r="P69" s="36" t="s">
         <v>17</v>
       </c>
-      <c r="Q69" s="72" t="s">
-        <v>1844</v>
-      </c>
+      <c r="Q69" s="78"/>
       <c r="R69" s="35" t="s">
         <v>278</v>
       </c>
@@ -12136,7 +11896,7 @@
       <c r="D70" s="35" t="s">
         <v>562</v>
       </c>
-      <c r="E70" s="34" t="s">
+      <c r="E70" s="76" t="s">
         <v>570</v>
       </c>
       <c r="F70" s="34" t="s">
@@ -12172,9 +11932,7 @@
       <c r="P70" s="36" t="s">
         <v>17</v>
       </c>
-      <c r="Q70" s="72" t="s">
-        <v>1845</v>
-      </c>
+      <c r="Q70" s="78"/>
       <c r="R70" s="35" t="s">
         <v>278</v>
       </c>
@@ -12195,7 +11953,7 @@
       <c r="D71" s="35" t="s">
         <v>562</v>
       </c>
-      <c r="E71" s="34" t="s">
+      <c r="E71" s="76" t="s">
         <v>570</v>
       </c>
       <c r="F71" s="34" t="s">
@@ -12231,9 +11989,7 @@
       <c r="P71" s="36" t="s">
         <v>17</v>
       </c>
-      <c r="Q71" s="72" t="s">
-        <v>1846</v>
-      </c>
+      <c r="Q71" s="78"/>
       <c r="R71" s="35" t="s">
         <v>278</v>
       </c>
@@ -12242,28 +11998,10 @@
       <c r="U71" s="35"/>
     </row>
     <row r="72" spans="1:21" ht="24" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A72" s="65" t="s">
+      <c r="A72" s="57" t="s">
         <v>667</v>
       </c>
-      <c r="B72" s="66"/>
-      <c r="C72" s="66"/>
-      <c r="D72" s="66"/>
-      <c r="E72" s="66"/>
-      <c r="F72" s="66"/>
-      <c r="G72" s="66"/>
-      <c r="H72" s="66"/>
-      <c r="I72" s="66"/>
-      <c r="J72" s="66"/>
-      <c r="K72" s="66"/>
-      <c r="L72" s="66"/>
-      <c r="M72" s="66"/>
-      <c r="N72" s="66"/>
-      <c r="O72" s="66"/>
-      <c r="P72" s="66"/>
-      <c r="R72" s="66"/>
-      <c r="S72" s="66"/>
-      <c r="T72" s="66"/>
-      <c r="U72" s="66"/>
+      <c r="Q72" s="80"/>
     </row>
     <row r="73" spans="1:21" ht="24" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A73" s="34">
@@ -12278,7 +12016,7 @@
       <c r="D73" s="35" t="s">
         <v>669</v>
       </c>
-      <c r="E73" s="34" t="s">
+      <c r="E73" s="77" t="s">
         <v>670</v>
       </c>
       <c r="F73" s="34" t="s">
@@ -12314,9 +12052,7 @@
       <c r="P73" s="36" t="s">
         <v>17</v>
       </c>
-      <c r="Q73" s="72" t="s">
-        <v>1847</v>
-      </c>
+      <c r="Q73" s="78"/>
       <c r="R73" s="35" t="s">
         <v>278</v>
       </c>
@@ -12343,7 +12079,7 @@
       <c r="D74" s="35" t="s">
         <v>669</v>
       </c>
-      <c r="E74" s="34" t="s">
+      <c r="E74" s="77" t="s">
         <v>670</v>
       </c>
       <c r="F74" s="34" t="s">
@@ -12379,9 +12115,7 @@
       <c r="P74" s="36" t="s">
         <v>17</v>
       </c>
-      <c r="Q74" s="72" t="s">
-        <v>1848</v>
-      </c>
+      <c r="Q74" s="78"/>
       <c r="R74" s="35" t="s">
         <v>278</v>
       </c>
@@ -12402,7 +12136,7 @@
       <c r="D75" s="35" t="s">
         <v>669</v>
       </c>
-      <c r="E75" s="34" t="s">
+      <c r="E75" s="77" t="s">
         <v>670</v>
       </c>
       <c r="F75" s="34" t="s">
@@ -12438,9 +12172,7 @@
       <c r="P75" s="36" t="s">
         <v>17</v>
       </c>
-      <c r="Q75" s="72" t="s">
-        <v>1849</v>
-      </c>
+      <c r="Q75" s="78"/>
       <c r="R75" s="35" t="s">
         <v>695</v>
       </c>
@@ -12467,7 +12199,7 @@
       <c r="D76" s="35" t="s">
         <v>669</v>
       </c>
-      <c r="E76" s="34" t="s">
+      <c r="E76" s="77" t="s">
         <v>670</v>
       </c>
       <c r="F76" s="34" t="s">
@@ -12503,9 +12235,7 @@
       <c r="P76" s="36" t="s">
         <v>17</v>
       </c>
-      <c r="Q76" s="72" t="s">
-        <v>1850</v>
-      </c>
+      <c r="Q76" s="78"/>
       <c r="R76" s="35" t="s">
         <v>706</v>
       </c>
@@ -12526,7 +12256,7 @@
       <c r="D77" s="35" t="s">
         <v>669</v>
       </c>
-      <c r="E77" s="34" t="s">
+      <c r="E77" s="77" t="s">
         <v>670</v>
       </c>
       <c r="F77" s="34" t="s">
@@ -12562,9 +12292,7 @@
       <c r="P77" s="36" t="s">
         <v>17</v>
       </c>
-      <c r="Q77" s="72" t="s">
-        <v>1851</v>
-      </c>
+      <c r="Q77" s="78"/>
       <c r="R77" s="35" t="s">
         <v>278</v>
       </c>
@@ -12585,7 +12313,7 @@
       <c r="D78" s="35" t="s">
         <v>669</v>
       </c>
-      <c r="E78" s="34" t="s">
+      <c r="E78" s="77" t="s">
         <v>670</v>
       </c>
       <c r="F78" s="34" t="s">
@@ -12621,9 +12349,7 @@
       <c r="P78" s="36" t="s">
         <v>17</v>
       </c>
-      <c r="Q78" s="72" t="s">
-        <v>1852</v>
-      </c>
+      <c r="Q78" s="78"/>
       <c r="R78" s="35" t="s">
         <v>278</v>
       </c>
@@ -12644,7 +12370,7 @@
       <c r="D79" s="35" t="s">
         <v>669</v>
       </c>
-      <c r="E79" s="34" t="s">
+      <c r="E79" s="77" t="s">
         <v>670</v>
       </c>
       <c r="F79" s="34" t="s">
@@ -12680,9 +12406,7 @@
       <c r="P79" s="36" t="s">
         <v>17</v>
       </c>
-      <c r="Q79" s="72" t="s">
-        <v>1853</v>
-      </c>
+      <c r="Q79" s="78"/>
       <c r="R79" s="35" t="s">
         <v>278</v>
       </c>
@@ -12691,28 +12415,10 @@
       <c r="U79" s="35"/>
     </row>
     <row r="80" spans="1:21" ht="24" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A80" s="65" t="s">
+      <c r="A80" s="57" t="s">
         <v>730</v>
       </c>
-      <c r="B80" s="66"/>
-      <c r="C80" s="66"/>
-      <c r="D80" s="66"/>
-      <c r="E80" s="66"/>
-      <c r="F80" s="66"/>
-      <c r="G80" s="66"/>
-      <c r="H80" s="66"/>
-      <c r="I80" s="66"/>
-      <c r="J80" s="66"/>
-      <c r="K80" s="66"/>
-      <c r="L80" s="66"/>
-      <c r="M80" s="66"/>
-      <c r="N80" s="66"/>
-      <c r="O80" s="66"/>
-      <c r="P80" s="66"/>
-      <c r="R80" s="66"/>
-      <c r="S80" s="66"/>
-      <c r="T80" s="66"/>
-      <c r="U80" s="66"/>
+      <c r="Q80" s="80"/>
     </row>
     <row r="81" spans="1:21" ht="24" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A81" s="34">
@@ -12763,9 +12469,7 @@
       <c r="P81" s="36" t="s">
         <v>17</v>
       </c>
-      <c r="Q81" s="73">
-        <v>46033</v>
-      </c>
+      <c r="Q81" s="79"/>
       <c r="R81" s="35" t="s">
         <v>278</v>
       </c>
@@ -12822,9 +12526,7 @@
       <c r="P82" s="36" t="s">
         <v>17</v>
       </c>
-      <c r="Q82" s="73">
-        <v>46064</v>
-      </c>
+      <c r="Q82" s="79"/>
       <c r="R82" s="35" t="s">
         <v>278</v>
       </c>
@@ -12887,9 +12589,7 @@
       <c r="P83" s="36" t="s">
         <v>17</v>
       </c>
-      <c r="Q83" s="73">
-        <v>46092</v>
-      </c>
+      <c r="Q83" s="79"/>
       <c r="R83" s="35" t="s">
         <v>278</v>
       </c>
@@ -12946,9 +12646,7 @@
       <c r="P84" s="36" t="s">
         <v>17</v>
       </c>
-      <c r="Q84" s="73">
-        <v>46123</v>
-      </c>
+      <c r="Q84" s="79"/>
       <c r="R84" s="35" t="s">
         <v>278</v>
       </c>
@@ -13011,9 +12709,7 @@
       <c r="P85" s="36" t="s">
         <v>17</v>
       </c>
-      <c r="Q85" s="73">
-        <v>46153</v>
-      </c>
+      <c r="Q85" s="79"/>
       <c r="R85" s="35" t="s">
         <v>278</v>
       </c>
@@ -13076,9 +12772,7 @@
       <c r="P86" s="36" t="s">
         <v>17</v>
       </c>
-      <c r="Q86" s="73">
-        <v>46184</v>
-      </c>
+      <c r="Q86" s="79"/>
       <c r="R86" s="35" t="s">
         <v>278</v>
       </c>
@@ -13135,9 +12829,7 @@
       <c r="P87" s="36" t="s">
         <v>17</v>
       </c>
-      <c r="Q87" s="73">
-        <v>46214</v>
-      </c>
+      <c r="Q87" s="79"/>
       <c r="R87" s="35" t="s">
         <v>278</v>
       </c>
@@ -13146,52 +12838,14 @@
       <c r="U87" s="35"/>
     </row>
     <row r="88" spans="1:21" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A88" s="67" t="s">
+      <c r="A88" s="58" t="s">
         <v>798</v>
       </c>
-      <c r="B88" s="66"/>
-      <c r="C88" s="66"/>
-      <c r="D88" s="66"/>
-      <c r="E88" s="66"/>
-      <c r="F88" s="66"/>
-      <c r="G88" s="66"/>
-      <c r="H88" s="66"/>
-      <c r="I88" s="66"/>
-      <c r="J88" s="66"/>
-      <c r="K88" s="66"/>
-      <c r="L88" s="66"/>
-      <c r="M88" s="66"/>
-      <c r="N88" s="66"/>
-      <c r="O88" s="66"/>
-      <c r="P88" s="66"/>
-      <c r="R88" s="66"/>
-      <c r="S88" s="66"/>
-      <c r="T88" s="66"/>
-      <c r="U88" s="66"/>
     </row>
     <row r="89" spans="1:21" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A89" s="65" t="s">
+      <c r="A89" s="57" t="s">
         <v>799</v>
       </c>
-      <c r="B89" s="66"/>
-      <c r="C89" s="66"/>
-      <c r="D89" s="66"/>
-      <c r="E89" s="66"/>
-      <c r="F89" s="66"/>
-      <c r="G89" s="66"/>
-      <c r="H89" s="66"/>
-      <c r="I89" s="66"/>
-      <c r="J89" s="66"/>
-      <c r="K89" s="66"/>
-      <c r="L89" s="66"/>
-      <c r="M89" s="66"/>
-      <c r="N89" s="66"/>
-      <c r="O89" s="66"/>
-      <c r="P89" s="66"/>
-      <c r="R89" s="66"/>
-      <c r="S89" s="66"/>
-      <c r="T89" s="66"/>
-      <c r="U89" s="66"/>
     </row>
     <row r="90" spans="1:21" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A90" s="34">
@@ -13242,7 +12896,7 @@
       <c r="P90" s="36" t="s">
         <v>11</v>
       </c>
-      <c r="Q90" s="71"/>
+      <c r="Q90" s="62"/>
       <c r="R90" s="35" t="s">
         <v>809</v>
       </c>
@@ -13299,7 +12953,7 @@
       <c r="P91" s="36" t="s">
         <v>17</v>
       </c>
-      <c r="Q91" s="71"/>
+      <c r="Q91" s="62"/>
       <c r="R91" s="35" t="s">
         <v>809</v>
       </c>
@@ -13362,7 +13016,7 @@
       <c r="P92" s="36" t="s">
         <v>17</v>
       </c>
-      <c r="Q92" s="71"/>
+      <c r="Q92" s="62"/>
       <c r="R92" s="35" t="s">
         <v>809</v>
       </c>
@@ -13419,7 +13073,7 @@
       <c r="P93" s="36" t="s">
         <v>17</v>
       </c>
-      <c r="Q93" s="71"/>
+      <c r="Q93" s="62"/>
       <c r="R93" s="35" t="s">
         <v>809</v>
       </c>
@@ -13428,28 +13082,9 @@
       <c r="U93" s="35"/>
     </row>
     <row r="94" spans="1:21" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A94" s="65" t="s">
+      <c r="A94" s="57" t="s">
         <v>836</v>
       </c>
-      <c r="B94" s="66"/>
-      <c r="C94" s="66"/>
-      <c r="D94" s="66"/>
-      <c r="E94" s="66"/>
-      <c r="F94" s="66"/>
-      <c r="G94" s="66"/>
-      <c r="H94" s="66"/>
-      <c r="I94" s="66"/>
-      <c r="J94" s="66"/>
-      <c r="K94" s="66"/>
-      <c r="L94" s="66"/>
-      <c r="M94" s="66"/>
-      <c r="N94" s="66"/>
-      <c r="O94" s="66"/>
-      <c r="P94" s="66"/>
-      <c r="R94" s="66"/>
-      <c r="S94" s="66"/>
-      <c r="T94" s="66"/>
-      <c r="U94" s="66"/>
     </row>
     <row r="95" spans="1:21" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A95" s="34">
@@ -13500,7 +13135,7 @@
       <c r="P95" s="36" t="s">
         <v>17</v>
       </c>
-      <c r="Q95" s="71"/>
+      <c r="Q95" s="62"/>
       <c r="R95" s="35" t="s">
         <v>809</v>
       </c>
@@ -13557,7 +13192,7 @@
       <c r="P96" s="36" t="s">
         <v>17</v>
       </c>
-      <c r="Q96" s="71"/>
+      <c r="Q96" s="62"/>
       <c r="R96" s="35" t="s">
         <v>809</v>
       </c>
@@ -13614,7 +13249,7 @@
       <c r="P97" s="36" t="s">
         <v>17</v>
       </c>
-      <c r="Q97" s="71"/>
+      <c r="Q97" s="62"/>
       <c r="R97" s="35" t="s">
         <v>809</v>
       </c>
@@ -13677,7 +13312,7 @@
       <c r="P98" s="36" t="s">
         <v>17</v>
       </c>
-      <c r="Q98" s="71"/>
+      <c r="Q98" s="62"/>
       <c r="R98" s="35" t="s">
         <v>809</v>
       </c>
@@ -13734,7 +13369,7 @@
       <c r="P99" s="36" t="s">
         <v>17</v>
       </c>
-      <c r="Q99" s="71"/>
+      <c r="Q99" s="62"/>
       <c r="R99" s="35" t="s">
         <v>809</v>
       </c>
@@ -13791,7 +13426,7 @@
       <c r="P100" s="36" t="s">
         <v>17</v>
       </c>
-      <c r="Q100" s="71"/>
+      <c r="Q100" s="62"/>
       <c r="R100" s="35" t="s">
         <v>809</v>
       </c>
@@ -13848,7 +13483,7 @@
       <c r="P101" s="36" t="s">
         <v>17</v>
       </c>
-      <c r="Q101" s="71"/>
+      <c r="Q101" s="62"/>
       <c r="R101" s="35" t="s">
         <v>809</v>
       </c>
@@ -13905,7 +13540,7 @@
       <c r="P102" s="36" t="s">
         <v>17</v>
       </c>
-      <c r="Q102" s="71"/>
+      <c r="Q102" s="62"/>
       <c r="R102" s="35" t="s">
         <v>809</v>
       </c>
@@ -13962,7 +13597,7 @@
       <c r="P103" s="36" t="s">
         <v>17</v>
       </c>
-      <c r="Q103" s="71"/>
+      <c r="Q103" s="62"/>
       <c r="R103" s="35" t="s">
         <v>809</v>
       </c>
@@ -14019,7 +13654,7 @@
       <c r="P104" s="36" t="s">
         <v>17</v>
       </c>
-      <c r="Q104" s="71"/>
+      <c r="Q104" s="62"/>
       <c r="R104" s="35" t="s">
         <v>915</v>
       </c>
@@ -14028,28 +13663,9 @@
       <c r="U104" s="35"/>
     </row>
     <row r="105" spans="1:21" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A105" s="65" t="s">
+      <c r="A105" s="57" t="s">
         <v>916</v>
       </c>
-      <c r="B105" s="66"/>
-      <c r="C105" s="66"/>
-      <c r="D105" s="66"/>
-      <c r="E105" s="66"/>
-      <c r="F105" s="66"/>
-      <c r="G105" s="66"/>
-      <c r="H105" s="66"/>
-      <c r="I105" s="66"/>
-      <c r="J105" s="66"/>
-      <c r="K105" s="66"/>
-      <c r="L105" s="66"/>
-      <c r="M105" s="66"/>
-      <c r="N105" s="66"/>
-      <c r="O105" s="66"/>
-      <c r="P105" s="66"/>
-      <c r="R105" s="66"/>
-      <c r="S105" s="66"/>
-      <c r="T105" s="66"/>
-      <c r="U105" s="66"/>
     </row>
     <row r="106" spans="1:21" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A106" s="34">
@@ -14100,7 +13716,7 @@
       <c r="P106" s="36" t="s">
         <v>17</v>
       </c>
-      <c r="Q106" s="71"/>
+      <c r="Q106" s="62"/>
       <c r="R106" s="35" t="s">
         <v>809</v>
       </c>
@@ -14157,7 +13773,7 @@
       <c r="P107" s="36" t="s">
         <v>17</v>
       </c>
-      <c r="Q107" s="71"/>
+      <c r="Q107" s="62"/>
       <c r="R107" s="35" t="s">
         <v>809</v>
       </c>
@@ -14214,7 +13830,7 @@
       <c r="P108" s="36" t="s">
         <v>17</v>
       </c>
-      <c r="Q108" s="71"/>
+      <c r="Q108" s="62"/>
       <c r="R108" s="35" t="s">
         <v>809</v>
       </c>
@@ -14223,28 +13839,9 @@
       <c r="U108" s="35"/>
     </row>
     <row r="109" spans="1:21" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A109" s="65" t="s">
+      <c r="A109" s="57" t="s">
         <v>941</v>
       </c>
-      <c r="B109" s="66"/>
-      <c r="C109" s="66"/>
-      <c r="D109" s="66"/>
-      <c r="E109" s="66"/>
-      <c r="F109" s="66"/>
-      <c r="G109" s="66"/>
-      <c r="H109" s="66"/>
-      <c r="I109" s="66"/>
-      <c r="J109" s="66"/>
-      <c r="K109" s="66"/>
-      <c r="L109" s="66"/>
-      <c r="M109" s="66"/>
-      <c r="N109" s="66"/>
-      <c r="O109" s="66"/>
-      <c r="P109" s="66"/>
-      <c r="R109" s="66"/>
-      <c r="S109" s="66"/>
-      <c r="T109" s="66"/>
-      <c r="U109" s="66"/>
     </row>
     <row r="110" spans="1:21" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A110" s="34">
@@ -14295,7 +13892,7 @@
       <c r="P110" s="36" t="s">
         <v>17</v>
       </c>
-      <c r="Q110" s="71"/>
+      <c r="Q110" s="62"/>
       <c r="R110" s="35" t="s">
         <v>809</v>
       </c>
@@ -14352,7 +13949,7 @@
       <c r="P111" s="36" t="s">
         <v>17</v>
       </c>
-      <c r="Q111" s="71"/>
+      <c r="Q111" s="62"/>
       <c r="R111" s="35" t="s">
         <v>809</v>
       </c>
@@ -14409,7 +14006,7 @@
       <c r="P112" s="36" t="s">
         <v>17</v>
       </c>
-      <c r="Q112" s="71"/>
+      <c r="Q112" s="62"/>
       <c r="R112" s="35" t="s">
         <v>809</v>
       </c>
@@ -14418,28 +14015,9 @@
       <c r="U112" s="35"/>
     </row>
     <row r="113" spans="1:21" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A113" s="65" t="s">
+      <c r="A113" s="57" t="s">
         <v>966</v>
       </c>
-      <c r="B113" s="66"/>
-      <c r="C113" s="66"/>
-      <c r="D113" s="66"/>
-      <c r="E113" s="66"/>
-      <c r="F113" s="66"/>
-      <c r="G113" s="66"/>
-      <c r="H113" s="66"/>
-      <c r="I113" s="66"/>
-      <c r="J113" s="66"/>
-      <c r="K113" s="66"/>
-      <c r="L113" s="66"/>
-      <c r="M113" s="66"/>
-      <c r="N113" s="66"/>
-      <c r="O113" s="66"/>
-      <c r="P113" s="66"/>
-      <c r="R113" s="66"/>
-      <c r="S113" s="66"/>
-      <c r="T113" s="66"/>
-      <c r="U113" s="66"/>
     </row>
     <row r="114" spans="1:21" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A114" s="34">
@@ -14490,7 +14068,7 @@
       <c r="P114" s="36" t="s">
         <v>17</v>
       </c>
-      <c r="Q114" s="71"/>
+      <c r="Q114" s="62"/>
       <c r="R114" s="35" t="s">
         <v>809</v>
       </c>
@@ -14547,7 +14125,7 @@
       <c r="P115" s="36" t="s">
         <v>17</v>
       </c>
-      <c r="Q115" s="71"/>
+      <c r="Q115" s="62"/>
       <c r="R115" s="35" t="s">
         <v>809</v>
       </c>
@@ -14604,7 +14182,7 @@
       <c r="P116" s="36" t="s">
         <v>17</v>
       </c>
-      <c r="Q116" s="71"/>
+      <c r="Q116" s="62"/>
       <c r="R116" s="35" t="s">
         <v>809</v>
       </c>
@@ -14661,7 +14239,7 @@
       <c r="P117" s="36" t="s">
         <v>17</v>
       </c>
-      <c r="Q117" s="71"/>
+      <c r="Q117" s="62"/>
       <c r="R117" s="35" t="s">
         <v>809</v>
       </c>
@@ -14718,7 +14296,7 @@
       <c r="P118" s="36" t="s">
         <v>17</v>
       </c>
-      <c r="Q118" s="71"/>
+      <c r="Q118" s="62"/>
       <c r="R118" s="35" t="s">
         <v>809</v>
       </c>
@@ -14775,7 +14353,7 @@
       <c r="P119" s="36" t="s">
         <v>17</v>
       </c>
-      <c r="Q119" s="71"/>
+      <c r="Q119" s="62"/>
       <c r="R119" s="35" t="s">
         <v>809</v>
       </c>
@@ -14832,7 +14410,7 @@
       <c r="P120" s="36" t="s">
         <v>17</v>
       </c>
-      <c r="Q120" s="71"/>
+      <c r="Q120" s="62"/>
       <c r="R120" s="35" t="s">
         <v>809</v>
       </c>
@@ -14841,28 +14419,9 @@
       <c r="U120" s="35"/>
     </row>
     <row r="121" spans="1:21" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A121" s="65" t="s">
+      <c r="A121" s="57" t="s">
         <v>1020</v>
       </c>
-      <c r="B121" s="66"/>
-      <c r="C121" s="66"/>
-      <c r="D121" s="66"/>
-      <c r="E121" s="66"/>
-      <c r="F121" s="66"/>
-      <c r="G121" s="66"/>
-      <c r="H121" s="66"/>
-      <c r="I121" s="66"/>
-      <c r="J121" s="66"/>
-      <c r="K121" s="66"/>
-      <c r="L121" s="66"/>
-      <c r="M121" s="66"/>
-      <c r="N121" s="66"/>
-      <c r="O121" s="66"/>
-      <c r="P121" s="66"/>
-      <c r="R121" s="66"/>
-      <c r="S121" s="66"/>
-      <c r="T121" s="66"/>
-      <c r="U121" s="66"/>
     </row>
     <row r="122" spans="1:21" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A122" s="34">
@@ -14913,7 +14472,7 @@
       <c r="P122" s="36" t="s">
         <v>17</v>
       </c>
-      <c r="Q122" s="71"/>
+      <c r="Q122" s="62"/>
       <c r="R122" s="35" t="s">
         <v>1030</v>
       </c>
@@ -14970,7 +14529,7 @@
       <c r="P123" s="36" t="s">
         <v>17</v>
       </c>
-      <c r="Q123" s="71"/>
+      <c r="Q123" s="62"/>
       <c r="R123" s="35" t="s">
         <v>809</v>
       </c>
@@ -15027,7 +14586,7 @@
       <c r="P124" s="36" t="s">
         <v>17</v>
       </c>
-      <c r="Q124" s="71"/>
+      <c r="Q124" s="62"/>
       <c r="R124" s="35" t="s">
         <v>809</v>
       </c>
@@ -15036,28 +14595,9 @@
       <c r="U124" s="35"/>
     </row>
     <row r="125" spans="1:21" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A125" s="65" t="s">
+      <c r="A125" s="57" t="s">
         <v>1044</v>
       </c>
-      <c r="B125" s="66"/>
-      <c r="C125" s="66"/>
-      <c r="D125" s="66"/>
-      <c r="E125" s="66"/>
-      <c r="F125" s="66"/>
-      <c r="G125" s="66"/>
-      <c r="H125" s="66"/>
-      <c r="I125" s="66"/>
-      <c r="J125" s="66"/>
-      <c r="K125" s="66"/>
-      <c r="L125" s="66"/>
-      <c r="M125" s="66"/>
-      <c r="N125" s="66"/>
-      <c r="O125" s="66"/>
-      <c r="P125" s="66"/>
-      <c r="R125" s="66"/>
-      <c r="S125" s="66"/>
-      <c r="T125" s="66"/>
-      <c r="U125" s="66"/>
     </row>
     <row r="126" spans="1:21" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A126" s="34">
@@ -15108,7 +14648,7 @@
       <c r="P126" s="36" t="s">
         <v>17</v>
       </c>
-      <c r="Q126" s="71"/>
+      <c r="Q126" s="62"/>
       <c r="R126" s="35" t="s">
         <v>809</v>
       </c>
@@ -15165,7 +14705,7 @@
       <c r="P127" s="36" t="s">
         <v>17</v>
       </c>
-      <c r="Q127" s="71"/>
+      <c r="Q127" s="62"/>
       <c r="R127" s="35" t="s">
         <v>809</v>
       </c>
@@ -15222,7 +14762,7 @@
       <c r="P128" s="36" t="s">
         <v>17</v>
       </c>
-      <c r="Q128" s="71"/>
+      <c r="Q128" s="62"/>
       <c r="R128" s="35" t="s">
         <v>809</v>
       </c>
@@ -15231,52 +14771,14 @@
       <c r="U128" s="35"/>
     </row>
     <row r="129" spans="1:21" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A129" s="67" t="s">
+      <c r="A129" s="58" t="s">
         <v>1068</v>
       </c>
-      <c r="B129" s="66"/>
-      <c r="C129" s="66"/>
-      <c r="D129" s="66"/>
-      <c r="E129" s="66"/>
-      <c r="F129" s="66"/>
-      <c r="G129" s="66"/>
-      <c r="H129" s="66"/>
-      <c r="I129" s="66"/>
-      <c r="J129" s="66"/>
-      <c r="K129" s="66"/>
-      <c r="L129" s="66"/>
-      <c r="M129" s="66"/>
-      <c r="N129" s="66"/>
-      <c r="O129" s="66"/>
-      <c r="P129" s="66"/>
-      <c r="R129" s="66"/>
-      <c r="S129" s="66"/>
-      <c r="T129" s="66"/>
-      <c r="U129" s="66"/>
     </row>
     <row r="130" spans="1:21" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A130" s="65" t="s">
+      <c r="A130" s="57" t="s">
         <v>1069</v>
       </c>
-      <c r="B130" s="66"/>
-      <c r="C130" s="66"/>
-      <c r="D130" s="66"/>
-      <c r="E130" s="66"/>
-      <c r="F130" s="66"/>
-      <c r="G130" s="66"/>
-      <c r="H130" s="66"/>
-      <c r="I130" s="66"/>
-      <c r="J130" s="66"/>
-      <c r="K130" s="66"/>
-      <c r="L130" s="66"/>
-      <c r="M130" s="66"/>
-      <c r="N130" s="66"/>
-      <c r="O130" s="66"/>
-      <c r="P130" s="66"/>
-      <c r="R130" s="66"/>
-      <c r="S130" s="66"/>
-      <c r="T130" s="66"/>
-      <c r="U130" s="66"/>
     </row>
     <row r="131" spans="1:21" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A131" s="34">
@@ -15327,7 +14829,7 @@
       <c r="P131" s="36" t="s">
         <v>9</v>
       </c>
-      <c r="Q131" s="71"/>
+      <c r="Q131" s="62"/>
       <c r="R131" s="35" t="s">
         <v>1080</v>
       </c>
@@ -15384,7 +14886,7 @@
       <c r="P132" s="36" t="s">
         <v>9</v>
       </c>
-      <c r="Q132" s="71"/>
+      <c r="Q132" s="62"/>
       <c r="R132" s="35" t="s">
         <v>1080</v>
       </c>
@@ -15441,7 +14943,7 @@
       <c r="P133" s="36" t="s">
         <v>9</v>
       </c>
-      <c r="Q133" s="71"/>
+      <c r="Q133" s="62"/>
       <c r="R133" s="35" t="s">
         <v>1080</v>
       </c>
@@ -15498,7 +15000,7 @@
       <c r="P134" s="36" t="s">
         <v>9</v>
       </c>
-      <c r="Q134" s="71"/>
+      <c r="Q134" s="62"/>
       <c r="R134" s="35" t="s">
         <v>1080</v>
       </c>
@@ -15507,28 +15009,9 @@
       <c r="U134" s="35"/>
     </row>
     <row r="135" spans="1:21" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A135" s="65" t="s">
+      <c r="A135" s="57" t="s">
         <v>1103</v>
       </c>
-      <c r="B135" s="66"/>
-      <c r="C135" s="66"/>
-      <c r="D135" s="66"/>
-      <c r="E135" s="66"/>
-      <c r="F135" s="66"/>
-      <c r="G135" s="66"/>
-      <c r="H135" s="66"/>
-      <c r="I135" s="66"/>
-      <c r="J135" s="66"/>
-      <c r="K135" s="66"/>
-      <c r="L135" s="66"/>
-      <c r="M135" s="66"/>
-      <c r="N135" s="66"/>
-      <c r="O135" s="66"/>
-      <c r="P135" s="66"/>
-      <c r="R135" s="66"/>
-      <c r="S135" s="66"/>
-      <c r="T135" s="66"/>
-      <c r="U135" s="66"/>
     </row>
     <row r="136" spans="1:21" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A136" s="34">
@@ -15579,7 +15062,7 @@
       <c r="P136" s="36" t="s">
         <v>9</v>
       </c>
-      <c r="Q136" s="71"/>
+      <c r="Q136" s="62"/>
       <c r="R136" s="35" t="s">
         <v>1080</v>
       </c>
@@ -15636,7 +15119,7 @@
       <c r="P137" s="36" t="s">
         <v>9</v>
       </c>
-      <c r="Q137" s="71"/>
+      <c r="Q137" s="62"/>
       <c r="R137" s="35" t="s">
         <v>1080</v>
       </c>
@@ -15693,7 +15176,7 @@
       <c r="P138" s="36" t="s">
         <v>9</v>
       </c>
-      <c r="Q138" s="71"/>
+      <c r="Q138" s="62"/>
       <c r="R138" s="35" t="s">
         <v>1080</v>
       </c>
@@ -15750,7 +15233,7 @@
       <c r="P139" s="36" t="s">
         <v>9</v>
       </c>
-      <c r="Q139" s="71"/>
+      <c r="Q139" s="62"/>
       <c r="R139" s="35" t="s">
         <v>1080</v>
       </c>
@@ -15807,7 +15290,7 @@
       <c r="P140" s="36" t="s">
         <v>9</v>
       </c>
-      <c r="Q140" s="71"/>
+      <c r="Q140" s="62"/>
       <c r="R140" s="35" t="s">
         <v>1080</v>
       </c>
@@ -15864,7 +15347,7 @@
       <c r="P141" s="36" t="s">
         <v>9</v>
       </c>
-      <c r="Q141" s="71"/>
+      <c r="Q141" s="62"/>
       <c r="R141" s="35" t="s">
         <v>1080</v>
       </c>
@@ -15921,7 +15404,7 @@
       <c r="P142" s="36" t="s">
         <v>9</v>
       </c>
-      <c r="Q142" s="71"/>
+      <c r="Q142" s="62"/>
       <c r="R142" s="35" t="s">
         <v>1080</v>
       </c>
@@ -15978,7 +15461,7 @@
       <c r="P143" s="36" t="s">
         <v>9</v>
       </c>
-      <c r="Q143" s="71"/>
+      <c r="Q143" s="62"/>
       <c r="R143" s="35" t="s">
         <v>1080</v>
       </c>
@@ -16035,7 +15518,7 @@
       <c r="P144" s="36" t="s">
         <v>9</v>
       </c>
-      <c r="Q144" s="71"/>
+      <c r="Q144" s="62"/>
       <c r="R144" s="35" t="s">
         <v>1080</v>
       </c>
@@ -16092,7 +15575,7 @@
       <c r="P145" s="36" t="s">
         <v>9</v>
       </c>
-      <c r="Q145" s="71" t="s">
+      <c r="Q145" s="62" t="s">
         <v>1181</v>
       </c>
       <c r="R145" s="35" t="s">
@@ -16103,28 +15586,9 @@
       <c r="U145" s="35"/>
     </row>
     <row r="146" spans="1:21" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A146" s="65" t="s">
+      <c r="A146" s="57" t="s">
         <v>1182</v>
       </c>
-      <c r="B146" s="66"/>
-      <c r="C146" s="66"/>
-      <c r="D146" s="66"/>
-      <c r="E146" s="66"/>
-      <c r="F146" s="66"/>
-      <c r="G146" s="66"/>
-      <c r="H146" s="66"/>
-      <c r="I146" s="66"/>
-      <c r="J146" s="66"/>
-      <c r="K146" s="66"/>
-      <c r="L146" s="66"/>
-      <c r="M146" s="66"/>
-      <c r="N146" s="66"/>
-      <c r="O146" s="66"/>
-      <c r="P146" s="66"/>
-      <c r="R146" s="66"/>
-      <c r="S146" s="66"/>
-      <c r="T146" s="66"/>
-      <c r="U146" s="66"/>
     </row>
     <row r="147" spans="1:21" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A147" s="34">
@@ -16175,7 +15639,7 @@
       <c r="P147" s="36" t="s">
         <v>9</v>
       </c>
-      <c r="Q147" s="71"/>
+      <c r="Q147" s="62"/>
       <c r="R147" s="35" t="s">
         <v>1080</v>
       </c>
@@ -16232,7 +15696,7 @@
       <c r="P148" s="36" t="s">
         <v>9</v>
       </c>
-      <c r="Q148" s="71"/>
+      <c r="Q148" s="62"/>
       <c r="R148" s="35" t="s">
         <v>1080</v>
       </c>
@@ -16289,7 +15753,7 @@
       <c r="P149" s="36" t="s">
         <v>9</v>
       </c>
-      <c r="Q149" s="71"/>
+      <c r="Q149" s="62"/>
       <c r="R149" s="35" t="s">
         <v>1080</v>
       </c>
@@ -16346,7 +15810,7 @@
       <c r="P150" s="36" t="s">
         <v>9</v>
       </c>
-      <c r="Q150" s="71"/>
+      <c r="Q150" s="62"/>
       <c r="R150" s="35" t="s">
         <v>1080</v>
       </c>
@@ -16403,7 +15867,7 @@
       <c r="P151" s="36" t="s">
         <v>9</v>
       </c>
-      <c r="Q151" s="71"/>
+      <c r="Q151" s="62"/>
       <c r="R151" s="35" t="s">
         <v>1080</v>
       </c>
@@ -16460,7 +15924,7 @@
       <c r="P152" s="36" t="s">
         <v>9</v>
       </c>
-      <c r="Q152" s="71"/>
+      <c r="Q152" s="62"/>
       <c r="R152" s="35" t="s">
         <v>1080</v>
       </c>
@@ -16517,7 +15981,7 @@
       <c r="P153" s="36" t="s">
         <v>9</v>
       </c>
-      <c r="Q153" s="71"/>
+      <c r="Q153" s="62"/>
       <c r="R153" s="35" t="s">
         <v>1080</v>
       </c>
@@ -16574,7 +16038,7 @@
       <c r="P154" s="36" t="s">
         <v>9</v>
       </c>
-      <c r="Q154" s="71"/>
+      <c r="Q154" s="62"/>
       <c r="R154" s="35" t="s">
         <v>1080</v>
       </c>
@@ -16583,28 +16047,9 @@
       <c r="U154" s="35"/>
     </row>
     <row r="155" spans="1:21" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A155" s="65" t="s">
+      <c r="A155" s="57" t="s">
         <v>1243</v>
       </c>
-      <c r="B155" s="66"/>
-      <c r="C155" s="66"/>
-      <c r="D155" s="66"/>
-      <c r="E155" s="66"/>
-      <c r="F155" s="66"/>
-      <c r="G155" s="66"/>
-      <c r="H155" s="66"/>
-      <c r="I155" s="66"/>
-      <c r="J155" s="66"/>
-      <c r="K155" s="66"/>
-      <c r="L155" s="66"/>
-      <c r="M155" s="66"/>
-      <c r="N155" s="66"/>
-      <c r="O155" s="66"/>
-      <c r="P155" s="66"/>
-      <c r="R155" s="66"/>
-      <c r="S155" s="66"/>
-      <c r="T155" s="66"/>
-      <c r="U155" s="66"/>
     </row>
     <row r="156" spans="1:21" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A156" s="34">
@@ -16655,7 +16100,7 @@
       <c r="P156" s="36" t="s">
         <v>17</v>
       </c>
-      <c r="Q156" s="71"/>
+      <c r="Q156" s="62"/>
       <c r="R156" s="35" t="s">
         <v>1080</v>
       </c>
@@ -16712,7 +16157,7 @@
       <c r="P157" s="36" t="s">
         <v>17</v>
       </c>
-      <c r="Q157" s="71"/>
+      <c r="Q157" s="62"/>
       <c r="R157" s="35" t="s">
         <v>1080</v>
       </c>
@@ -16769,7 +16214,7 @@
       <c r="P158" s="36" t="s">
         <v>17</v>
       </c>
-      <c r="Q158" s="71"/>
+      <c r="Q158" s="62"/>
       <c r="R158" s="35" t="s">
         <v>1080</v>
       </c>
@@ -16778,28 +16223,9 @@
       <c r="U158" s="35"/>
     </row>
     <row r="159" spans="1:21" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A159" s="65" t="s">
+      <c r="A159" s="57" t="s">
         <v>1267</v>
       </c>
-      <c r="B159" s="66"/>
-      <c r="C159" s="66"/>
-      <c r="D159" s="66"/>
-      <c r="E159" s="66"/>
-      <c r="F159" s="66"/>
-      <c r="G159" s="66"/>
-      <c r="H159" s="66"/>
-      <c r="I159" s="66"/>
-      <c r="J159" s="66"/>
-      <c r="K159" s="66"/>
-      <c r="L159" s="66"/>
-      <c r="M159" s="66"/>
-      <c r="N159" s="66"/>
-      <c r="O159" s="66"/>
-      <c r="P159" s="66"/>
-      <c r="R159" s="66"/>
-      <c r="S159" s="66"/>
-      <c r="T159" s="66"/>
-      <c r="U159" s="66"/>
     </row>
     <row r="160" spans="1:21" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A160" s="34">
@@ -16850,7 +16276,7 @@
       <c r="P160" s="36" t="s">
         <v>17</v>
       </c>
-      <c r="Q160" s="71"/>
+      <c r="Q160" s="62"/>
       <c r="R160" s="35" t="s">
         <v>1080</v>
       </c>
@@ -16907,7 +16333,7 @@
       <c r="P161" s="36" t="s">
         <v>17</v>
       </c>
-      <c r="Q161" s="71"/>
+      <c r="Q161" s="62"/>
       <c r="R161" s="35" t="s">
         <v>1080</v>
       </c>
@@ -16916,28 +16342,9 @@
       <c r="U161" s="35"/>
     </row>
     <row r="162" spans="1:21" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A162" s="65" t="s">
+      <c r="A162" s="57" t="s">
         <v>1283</v>
       </c>
-      <c r="B162" s="66"/>
-      <c r="C162" s="66"/>
-      <c r="D162" s="66"/>
-      <c r="E162" s="66"/>
-      <c r="F162" s="66"/>
-      <c r="G162" s="66"/>
-      <c r="H162" s="66"/>
-      <c r="I162" s="66"/>
-      <c r="J162" s="66"/>
-      <c r="K162" s="66"/>
-      <c r="L162" s="66"/>
-      <c r="M162" s="66"/>
-      <c r="N162" s="66"/>
-      <c r="O162" s="66"/>
-      <c r="P162" s="66"/>
-      <c r="R162" s="66"/>
-      <c r="S162" s="66"/>
-      <c r="T162" s="66"/>
-      <c r="U162" s="66"/>
     </row>
     <row r="163" spans="1:21" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A163" s="34">
@@ -16988,7 +16395,7 @@
       <c r="P163" s="36" t="s">
         <v>17</v>
       </c>
-      <c r="Q163" s="71"/>
+      <c r="Q163" s="62"/>
       <c r="R163" s="35" t="s">
         <v>1080</v>
       </c>
@@ -17045,7 +16452,7 @@
       <c r="P164" s="36" t="s">
         <v>17</v>
       </c>
-      <c r="Q164" s="71"/>
+      <c r="Q164" s="62"/>
       <c r="R164" s="35" t="s">
         <v>1080</v>
       </c>
@@ -17102,7 +16509,7 @@
       <c r="P165" s="36" t="s">
         <v>17</v>
       </c>
-      <c r="Q165" s="71"/>
+      <c r="Q165" s="62"/>
       <c r="R165" s="35" t="s">
         <v>1080</v>
       </c>
@@ -17111,52 +16518,14 @@
       <c r="U165" s="35"/>
     </row>
     <row r="166" spans="1:21" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A166" s="67" t="s">
+      <c r="A166" s="58" t="s">
         <v>1309</v>
       </c>
-      <c r="B166" s="66"/>
-      <c r="C166" s="66"/>
-      <c r="D166" s="66"/>
-      <c r="E166" s="66"/>
-      <c r="F166" s="66"/>
-      <c r="G166" s="66"/>
-      <c r="H166" s="66"/>
-      <c r="I166" s="66"/>
-      <c r="J166" s="66"/>
-      <c r="K166" s="66"/>
-      <c r="L166" s="66"/>
-      <c r="M166" s="66"/>
-      <c r="N166" s="66"/>
-      <c r="O166" s="66"/>
-      <c r="P166" s="66"/>
-      <c r="R166" s="66"/>
-      <c r="S166" s="66"/>
-      <c r="T166" s="66"/>
-      <c r="U166" s="66"/>
     </row>
     <row r="167" spans="1:21" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A167" s="65" t="s">
+      <c r="A167" s="57" t="s">
         <v>1310</v>
       </c>
-      <c r="B167" s="66"/>
-      <c r="C167" s="66"/>
-      <c r="D167" s="66"/>
-      <c r="E167" s="66"/>
-      <c r="F167" s="66"/>
-      <c r="G167" s="66"/>
-      <c r="H167" s="66"/>
-      <c r="I167" s="66"/>
-      <c r="J167" s="66"/>
-      <c r="K167" s="66"/>
-      <c r="L167" s="66"/>
-      <c r="M167" s="66"/>
-      <c r="N167" s="66"/>
-      <c r="O167" s="66"/>
-      <c r="P167" s="66"/>
-      <c r="R167" s="66"/>
-      <c r="S167" s="66"/>
-      <c r="T167" s="66"/>
-      <c r="U167" s="66"/>
     </row>
     <row r="168" spans="1:21" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A168" s="34">
@@ -17207,7 +16576,7 @@
       <c r="P168" s="36" t="s">
         <v>17</v>
       </c>
-      <c r="Q168" s="71"/>
+      <c r="Q168" s="62"/>
       <c r="R168" s="35"/>
       <c r="S168" s="34"/>
       <c r="T168" s="35"/>
@@ -17262,7 +16631,7 @@
       <c r="P169" s="36" t="s">
         <v>17</v>
       </c>
-      <c r="Q169" s="71"/>
+      <c r="Q169" s="62"/>
       <c r="R169" s="35"/>
       <c r="S169" s="34"/>
       <c r="T169" s="35"/>
@@ -17317,35 +16686,16 @@
       <c r="P170" s="36" t="s">
         <v>17</v>
       </c>
-      <c r="Q170" s="71"/>
+      <c r="Q170" s="62"/>
       <c r="R170" s="35"/>
       <c r="S170" s="34"/>
       <c r="T170" s="35"/>
       <c r="U170" s="35"/>
     </row>
     <row r="171" spans="1:21" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A171" s="65" t="s">
+      <c r="A171" s="57" t="s">
         <v>1333</v>
       </c>
-      <c r="B171" s="66"/>
-      <c r="C171" s="66"/>
-      <c r="D171" s="66"/>
-      <c r="E171" s="66"/>
-      <c r="F171" s="66"/>
-      <c r="G171" s="66"/>
-      <c r="H171" s="66"/>
-      <c r="I171" s="66"/>
-      <c r="J171" s="66"/>
-      <c r="K171" s="66"/>
-      <c r="L171" s="66"/>
-      <c r="M171" s="66"/>
-      <c r="N171" s="66"/>
-      <c r="O171" s="66"/>
-      <c r="P171" s="66"/>
-      <c r="R171" s="66"/>
-      <c r="S171" s="66"/>
-      <c r="T171" s="66"/>
-      <c r="U171" s="66"/>
     </row>
     <row r="172" spans="1:21" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A172" s="34">
@@ -17396,7 +16746,7 @@
       <c r="P172" s="36" t="s">
         <v>17</v>
       </c>
-      <c r="Q172" s="71"/>
+      <c r="Q172" s="62"/>
       <c r="R172" s="35"/>
       <c r="S172" s="34" t="s">
         <v>1343</v>
@@ -17457,7 +16807,7 @@
       <c r="P173" s="36" t="s">
         <v>17</v>
       </c>
-      <c r="Q173" s="71"/>
+      <c r="Q173" s="62"/>
       <c r="R173" s="35"/>
       <c r="S173" s="34"/>
       <c r="T173" s="35"/>
@@ -17512,35 +16862,16 @@
       <c r="P174" s="36" t="s">
         <v>17</v>
       </c>
-      <c r="Q174" s="71"/>
+      <c r="Q174" s="62"/>
       <c r="R174" s="35"/>
       <c r="S174" s="34"/>
       <c r="T174" s="35"/>
       <c r="U174" s="35"/>
     </row>
     <row r="175" spans="1:21" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A175" s="65" t="s">
+      <c r="A175" s="57" t="s">
         <v>1362</v>
       </c>
-      <c r="B175" s="66"/>
-      <c r="C175" s="66"/>
-      <c r="D175" s="66"/>
-      <c r="E175" s="66"/>
-      <c r="F175" s="66"/>
-      <c r="G175" s="66"/>
-      <c r="H175" s="66"/>
-      <c r="I175" s="66"/>
-      <c r="J175" s="66"/>
-      <c r="K175" s="66"/>
-      <c r="L175" s="66"/>
-      <c r="M175" s="66"/>
-      <c r="N175" s="66"/>
-      <c r="O175" s="66"/>
-      <c r="P175" s="66"/>
-      <c r="R175" s="66"/>
-      <c r="S175" s="66"/>
-      <c r="T175" s="66"/>
-      <c r="U175" s="66"/>
     </row>
     <row r="176" spans="1:21" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A176" s="34">
@@ -17591,7 +16922,7 @@
       <c r="P176" s="36" t="s">
         <v>17</v>
       </c>
-      <c r="Q176" s="71"/>
+      <c r="Q176" s="62"/>
       <c r="R176" s="35"/>
       <c r="S176" s="34"/>
       <c r="T176" s="35"/>
@@ -17646,7 +16977,7 @@
       <c r="P177" s="36" t="s">
         <v>17</v>
       </c>
-      <c r="Q177" s="71"/>
+      <c r="Q177" s="62"/>
       <c r="R177" s="35"/>
       <c r="S177" s="34"/>
       <c r="T177" s="35"/>
@@ -17701,7 +17032,7 @@
       <c r="P178" s="36" t="s">
         <v>17</v>
       </c>
-      <c r="Q178" s="71"/>
+      <c r="Q178" s="62"/>
       <c r="R178" s="35"/>
       <c r="S178" s="34"/>
       <c r="T178" s="35"/>
@@ -17756,7 +17087,7 @@
       <c r="P179" s="36" t="s">
         <v>17</v>
       </c>
-      <c r="Q179" s="71"/>
+      <c r="Q179" s="62"/>
       <c r="R179" s="35"/>
       <c r="S179" s="34"/>
       <c r="T179" s="35"/>
@@ -17811,7 +17142,7 @@
       <c r="P180" s="36" t="s">
         <v>17</v>
       </c>
-      <c r="Q180" s="71"/>
+      <c r="Q180" s="62"/>
       <c r="R180" s="35"/>
       <c r="S180" s="34"/>
       <c r="T180" s="35"/>
@@ -17866,35 +17197,16 @@
       <c r="P181" s="36" t="s">
         <v>17</v>
       </c>
-      <c r="Q181" s="71"/>
+      <c r="Q181" s="62"/>
       <c r="R181" s="35"/>
       <c r="S181" s="34"/>
       <c r="T181" s="35"/>
       <c r="U181" s="35"/>
     </row>
     <row r="182" spans="1:21" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A182" s="65" t="s">
+      <c r="A182" s="57" t="s">
         <v>1404</v>
       </c>
-      <c r="B182" s="66"/>
-      <c r="C182" s="66"/>
-      <c r="D182" s="66"/>
-      <c r="E182" s="66"/>
-      <c r="F182" s="66"/>
-      <c r="G182" s="66"/>
-      <c r="H182" s="66"/>
-      <c r="I182" s="66"/>
-      <c r="J182" s="66"/>
-      <c r="K182" s="66"/>
-      <c r="L182" s="66"/>
-      <c r="M182" s="66"/>
-      <c r="N182" s="66"/>
-      <c r="O182" s="66"/>
-      <c r="P182" s="66"/>
-      <c r="R182" s="66"/>
-      <c r="S182" s="66"/>
-      <c r="T182" s="66"/>
-      <c r="U182" s="66"/>
     </row>
     <row r="183" spans="1:21" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A183" s="34">
@@ -17945,7 +17257,7 @@
       <c r="P183" s="36" t="s">
         <v>17</v>
       </c>
-      <c r="Q183" s="71"/>
+      <c r="Q183" s="62"/>
       <c r="R183" s="35"/>
       <c r="S183" s="34"/>
       <c r="T183" s="35"/>
@@ -18000,59 +17312,21 @@
       <c r="P184" s="36" t="s">
         <v>17</v>
       </c>
-      <c r="Q184" s="71"/>
+      <c r="Q184" s="62"/>
       <c r="R184" s="35"/>
       <c r="S184" s="34"/>
       <c r="T184" s="35"/>
       <c r="U184" s="35"/>
     </row>
     <row r="185" spans="1:21" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A185" s="67" t="s">
+      <c r="A185" s="58" t="s">
         <v>1422</v>
       </c>
-      <c r="B185" s="66"/>
-      <c r="C185" s="66"/>
-      <c r="D185" s="66"/>
-      <c r="E185" s="66"/>
-      <c r="F185" s="66"/>
-      <c r="G185" s="66"/>
-      <c r="H185" s="66"/>
-      <c r="I185" s="66"/>
-      <c r="J185" s="66"/>
-      <c r="K185" s="66"/>
-      <c r="L185" s="66"/>
-      <c r="M185" s="66"/>
-      <c r="N185" s="66"/>
-      <c r="O185" s="66"/>
-      <c r="P185" s="66"/>
-      <c r="R185" s="66"/>
-      <c r="S185" s="66"/>
-      <c r="T185" s="66"/>
-      <c r="U185" s="66"/>
     </row>
     <row r="186" spans="1:21" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A186" s="65" t="s">
+      <c r="A186" s="57" t="s">
         <v>1423</v>
       </c>
-      <c r="B186" s="66"/>
-      <c r="C186" s="66"/>
-      <c r="D186" s="66"/>
-      <c r="E186" s="66"/>
-      <c r="F186" s="66"/>
-      <c r="G186" s="66"/>
-      <c r="H186" s="66"/>
-      <c r="I186" s="66"/>
-      <c r="J186" s="66"/>
-      <c r="K186" s="66"/>
-      <c r="L186" s="66"/>
-      <c r="M186" s="66"/>
-      <c r="N186" s="66"/>
-      <c r="O186" s="66"/>
-      <c r="P186" s="66"/>
-      <c r="R186" s="66"/>
-      <c r="S186" s="66"/>
-      <c r="T186" s="66"/>
-      <c r="U186" s="66"/>
     </row>
     <row r="187" spans="1:21" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A187" s="34">
@@ -18103,7 +17377,7 @@
       <c r="P187" s="36" t="s">
         <v>17</v>
       </c>
-      <c r="Q187" s="71"/>
+      <c r="Q187" s="62"/>
       <c r="R187" s="35"/>
       <c r="S187" s="34"/>
       <c r="T187" s="35"/>
@@ -18158,7 +17432,7 @@
       <c r="P188" s="36" t="s">
         <v>17</v>
       </c>
-      <c r="Q188" s="71"/>
+      <c r="Q188" s="62"/>
       <c r="R188" s="35"/>
       <c r="S188" s="34"/>
       <c r="T188" s="35"/>
@@ -18213,7 +17487,7 @@
       <c r="P189" s="36" t="s">
         <v>17</v>
       </c>
-      <c r="Q189" s="71"/>
+      <c r="Q189" s="62"/>
       <c r="R189" s="35"/>
       <c r="S189" s="34"/>
       <c r="T189" s="35"/>
@@ -18268,35 +17542,16 @@
       <c r="P190" s="36" t="s">
         <v>17</v>
       </c>
-      <c r="Q190" s="71"/>
+      <c r="Q190" s="62"/>
       <c r="R190" s="35"/>
       <c r="S190" s="34"/>
       <c r="T190" s="35"/>
       <c r="U190" s="35"/>
     </row>
     <row r="191" spans="1:21" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A191" s="65" t="s">
+      <c r="A191" s="57" t="s">
         <v>1454</v>
       </c>
-      <c r="B191" s="66"/>
-      <c r="C191" s="66"/>
-      <c r="D191" s="66"/>
-      <c r="E191" s="66"/>
-      <c r="F191" s="66"/>
-      <c r="G191" s="66"/>
-      <c r="H191" s="66"/>
-      <c r="I191" s="66"/>
-      <c r="J191" s="66"/>
-      <c r="K191" s="66"/>
-      <c r="L191" s="66"/>
-      <c r="M191" s="66"/>
-      <c r="N191" s="66"/>
-      <c r="O191" s="66"/>
-      <c r="P191" s="66"/>
-      <c r="R191" s="66"/>
-      <c r="S191" s="66"/>
-      <c r="T191" s="66"/>
-      <c r="U191" s="66"/>
     </row>
     <row r="192" spans="1:21" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A192" s="34">
@@ -18347,7 +17602,7 @@
       <c r="P192" s="36" t="s">
         <v>17</v>
       </c>
-      <c r="Q192" s="71"/>
+      <c r="Q192" s="62"/>
       <c r="R192" s="35"/>
       <c r="S192" s="34" t="s">
         <v>1465</v>
@@ -18408,7 +17663,7 @@
       <c r="P193" s="36" t="s">
         <v>17</v>
       </c>
-      <c r="Q193" s="71"/>
+      <c r="Q193" s="62"/>
       <c r="R193" s="35"/>
       <c r="S193" s="34"/>
       <c r="T193" s="35"/>
@@ -18463,7 +17718,7 @@
       <c r="P194" s="36" t="s">
         <v>17</v>
       </c>
-      <c r="Q194" s="71"/>
+      <c r="Q194" s="62"/>
       <c r="R194" s="35"/>
       <c r="S194" s="34"/>
       <c r="T194" s="35"/>
@@ -18518,35 +17773,16 @@
       <c r="P195" s="36" t="s">
         <v>17</v>
       </c>
-      <c r="Q195" s="71"/>
+      <c r="Q195" s="62"/>
       <c r="R195" s="35"/>
       <c r="S195" s="34"/>
       <c r="T195" s="35"/>
       <c r="U195" s="35"/>
     </row>
     <row r="196" spans="1:21" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A196" s="65" t="s">
+      <c r="A196" s="57" t="s">
         <v>1491</v>
       </c>
-      <c r="B196" s="66"/>
-      <c r="C196" s="66"/>
-      <c r="D196" s="66"/>
-      <c r="E196" s="66"/>
-      <c r="F196" s="66"/>
-      <c r="G196" s="66"/>
-      <c r="H196" s="66"/>
-      <c r="I196" s="66"/>
-      <c r="J196" s="66"/>
-      <c r="K196" s="66"/>
-      <c r="L196" s="66"/>
-      <c r="M196" s="66"/>
-      <c r="N196" s="66"/>
-      <c r="O196" s="66"/>
-      <c r="P196" s="66"/>
-      <c r="R196" s="66"/>
-      <c r="S196" s="66"/>
-      <c r="T196" s="66"/>
-      <c r="U196" s="66"/>
     </row>
     <row r="197" spans="1:21" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A197" s="34">
@@ -18597,7 +17833,7 @@
       <c r="P197" s="36" t="s">
         <v>17</v>
       </c>
-      <c r="Q197" s="71"/>
+      <c r="Q197" s="62"/>
       <c r="R197" s="35"/>
       <c r="S197" s="34" t="s">
         <v>1501</v>
@@ -18658,35 +17894,16 @@
       <c r="P198" s="36" t="s">
         <v>17</v>
       </c>
-      <c r="Q198" s="71"/>
+      <c r="Q198" s="62"/>
       <c r="R198" s="35"/>
       <c r="S198" s="34"/>
       <c r="T198" s="35"/>
       <c r="U198" s="35"/>
     </row>
     <row r="199" spans="1:21" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A199" s="65" t="s">
+      <c r="A199" s="57" t="s">
         <v>1512</v>
       </c>
-      <c r="B199" s="66"/>
-      <c r="C199" s="66"/>
-      <c r="D199" s="66"/>
-      <c r="E199" s="66"/>
-      <c r="F199" s="66"/>
-      <c r="G199" s="66"/>
-      <c r="H199" s="66"/>
-      <c r="I199" s="66"/>
-      <c r="J199" s="66"/>
-      <c r="K199" s="66"/>
-      <c r="L199" s="66"/>
-      <c r="M199" s="66"/>
-      <c r="N199" s="66"/>
-      <c r="O199" s="66"/>
-      <c r="P199" s="66"/>
-      <c r="R199" s="66"/>
-      <c r="S199" s="66"/>
-      <c r="T199" s="66"/>
-      <c r="U199" s="66"/>
     </row>
     <row r="200" spans="1:21" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A200" s="34">
@@ -18737,7 +17954,7 @@
       <c r="P200" s="36" t="s">
         <v>17</v>
       </c>
-      <c r="Q200" s="71"/>
+      <c r="Q200" s="62"/>
       <c r="R200" s="35"/>
       <c r="S200" s="34"/>
       <c r="T200" s="35"/>
@@ -18792,7 +18009,7 @@
       <c r="P201" s="36" t="s">
         <v>17</v>
       </c>
-      <c r="Q201" s="71"/>
+      <c r="Q201" s="62"/>
       <c r="R201" s="35"/>
       <c r="S201" s="34"/>
       <c r="T201" s="35"/>
@@ -18847,7 +18064,7 @@
       <c r="P202" s="36" t="s">
         <v>17</v>
       </c>
-      <c r="Q202" s="71"/>
+      <c r="Q202" s="62"/>
       <c r="R202" s="35"/>
       <c r="S202" s="34"/>
       <c r="T202" s="35"/>
@@ -18902,35 +18119,16 @@
       <c r="P203" s="36" t="s">
         <v>17</v>
       </c>
-      <c r="Q203" s="71"/>
+      <c r="Q203" s="62"/>
       <c r="R203" s="35"/>
       <c r="S203" s="34"/>
       <c r="T203" s="35"/>
       <c r="U203" s="35"/>
     </row>
     <row r="204" spans="1:21" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A204" s="65" t="s">
+      <c r="A204" s="57" t="s">
         <v>1545</v>
       </c>
-      <c r="B204" s="66"/>
-      <c r="C204" s="66"/>
-      <c r="D204" s="66"/>
-      <c r="E204" s="66"/>
-      <c r="F204" s="66"/>
-      <c r="G204" s="66"/>
-      <c r="H204" s="66"/>
-      <c r="I204" s="66"/>
-      <c r="J204" s="66"/>
-      <c r="K204" s="66"/>
-      <c r="L204" s="66"/>
-      <c r="M204" s="66"/>
-      <c r="N204" s="66"/>
-      <c r="O204" s="66"/>
-      <c r="P204" s="66"/>
-      <c r="R204" s="66"/>
-      <c r="S204" s="66"/>
-      <c r="T204" s="66"/>
-      <c r="U204" s="66"/>
     </row>
     <row r="205" spans="1:21" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A205" s="34">
@@ -18981,7 +18179,7 @@
       <c r="P205" s="36" t="s">
         <v>17</v>
       </c>
-      <c r="Q205" s="71"/>
+      <c r="Q205" s="62"/>
       <c r="R205" s="35"/>
       <c r="S205" s="34"/>
       <c r="T205" s="35"/>
@@ -19036,7 +18234,7 @@
       <c r="P206" s="36" t="s">
         <v>17</v>
       </c>
-      <c r="Q206" s="71"/>
+      <c r="Q206" s="62"/>
       <c r="R206" s="35"/>
       <c r="S206" s="34"/>
       <c r="T206" s="35"/>
@@ -19091,7 +18289,7 @@
       <c r="P207" s="36" t="s">
         <v>17</v>
       </c>
-      <c r="Q207" s="71"/>
+      <c r="Q207" s="62"/>
       <c r="R207" s="35"/>
       <c r="S207" s="34"/>
       <c r="T207" s="35"/>
@@ -19146,7 +18344,7 @@
       <c r="P208" s="36" t="s">
         <v>17</v>
       </c>
-      <c r="Q208" s="71"/>
+      <c r="Q208" s="62"/>
       <c r="R208" s="35"/>
       <c r="S208" s="34"/>
       <c r="T208" s="35"/>

</xml_diff>